<commit_message>
working on error handling
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="24-09-2024" sheetId="1" r:id="rId1"/>
+    <sheet name="23-12-2024" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -451,140 +451,140 @@
         <v>GRT-1</v>
       </c>
       <c r="B2">
-        <v>132543.07852198277</v>
+        <v>138891.53255013344</v>
       </c>
       <c r="C2">
-        <v>229.33103942871094</v>
+        <v>233.59140014648438</v>
       </c>
       <c r="D2">
-        <v>224.56288146972656</v>
+        <v>234.11288452148438</v>
       </c>
       <c r="E2">
-        <v>226.25628662109375</v>
+        <v>236.14212036132812</v>
       </c>
       <c r="F2">
-        <v>180.7670135498047</v>
+        <v>32.17891311645508</v>
       </c>
       <c r="G2">
-        <v>178.73973083496094</v>
+        <v>34.63349914550781</v>
       </c>
       <c r="H2">
-        <v>169.6169891357422</v>
+        <v>36.207763671875</v>
       </c>
       <c r="I2">
-        <v>39982.6484375</v>
+        <v>7460.419921875</v>
       </c>
       <c r="J2">
-        <v>38902.109375</v>
+        <v>3562.072998046875</v>
       </c>
       <c r="K2">
-        <v>35460.4140625</v>
+        <v>6219.52783203125</v>
       </c>
       <c r="L2">
-        <v>0.9309607744216919</v>
+        <v>0.8150226473808289</v>
       </c>
       <c r="M2">
-        <v>0.9306735396385193</v>
+        <v>0.790442705154419</v>
       </c>
       <c r="N2">
-        <v>0.9149314165115356</v>
+        <v>0.9486470222473145</v>
       </c>
       <c r="O2">
-        <v>114345.171875</v>
+        <v>12619.7255859375</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Ampac-2</v>
+        <v>Ampak-2</v>
       </c>
       <c r="B3">
-        <v>28566.9455292934</v>
+        <v>41277.116609706674</v>
       </c>
       <c r="C3">
-        <v>229.42103576660156</v>
+        <v>233.29896545410156</v>
       </c>
       <c r="D3">
-        <v>224.8515167236328</v>
+        <v>233.5473175048828</v>
       </c>
       <c r="E3">
-        <v>226.67083740234375</v>
+        <v>236.05038452148438</v>
       </c>
       <c r="F3">
-        <v>33.914546966552734</v>
+        <v>32.63731384277344</v>
       </c>
       <c r="G3">
-        <v>28.47479248046875</v>
+        <v>31.923927307128906</v>
       </c>
       <c r="H3">
-        <v>22.22391128540039</v>
+        <v>25.443716049194336</v>
       </c>
       <c r="I3">
-        <v>7148.869140625</v>
+        <v>6615.59814453125</v>
       </c>
       <c r="J3">
-        <v>5909.40478515625</v>
+        <v>12773.4716796875</v>
       </c>
       <c r="K3">
-        <v>3904.443115234375</v>
+        <v>12164.94921875</v>
       </c>
       <c r="L3">
-        <v>0.916961669921875</v>
+        <v>0.9669831991195679</v>
       </c>
       <c r="M3">
-        <v>0.9229694604873657</v>
+        <v>0.9583166837692261</v>
       </c>
       <c r="N3">
-        <v>0.7750735878944397</v>
+        <v>0.9691182374954224</v>
       </c>
       <c r="O3">
-        <v>16962.716796875</v>
+        <v>38014.85546875</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Ledena voda-3</v>
+        <v>Ledena Voda-3</v>
       </c>
       <c r="B4">
-        <v>169290.75800421476</v>
+        <v>245426.2544324171</v>
       </c>
       <c r="C4">
-        <v>214.1186065673828</v>
+        <v>236.96189880371094</v>
       </c>
       <c r="D4">
-        <v>224.959716796875</v>
+        <v>236.66102600097656</v>
       </c>
       <c r="E4">
-        <v>222.288330078125</v>
+        <v>238.5266571044922</v>
       </c>
       <c r="F4">
-        <v>433.80767822265625</v>
+        <v>0.18555894494056702</v>
       </c>
       <c r="G4">
-        <v>452.18768310546875</v>
+        <v>0.24126143753528595</v>
       </c>
       <c r="H4">
-        <v>464.4580078125</v>
+        <v>0.4243241250514984</v>
       </c>
       <c r="I4">
-        <v>74681.984375</v>
+        <v>35.66485595703125</v>
       </c>
       <c r="J4">
-        <v>84475.09375</v>
+        <v>-10.9794282913208</v>
       </c>
       <c r="K4">
-        <v>79878.03125</v>
+        <v>50.80659484863281</v>
       </c>
       <c r="L4">
-        <v>0.8045222759246826</v>
+        <v>0.8111370205879211</v>
       </c>
       <c r="M4">
-        <v>0.830193281173706</v>
+        <v>0.19233039021492004</v>
       </c>
       <c r="N4">
-        <v>0.773685097694397</v>
+        <v>0.5024684071540833</v>
       </c>
       <c r="O4">
-        <v>239035.125</v>
+        <v>75.49201965332031</v>
       </c>
     </row>
     <row r="5">
@@ -592,46 +592,46 @@
         <v>Hladilnici-4</v>
       </c>
       <c r="B5">
-        <v>126548.69664732688</v>
+        <v>181073.94627291267</v>
       </c>
       <c r="C5">
-        <v>229.0010528564453</v>
+        <v>237.485595703125</v>
       </c>
       <c r="D5">
-        <v>228.0508270263672</v>
+        <v>236.2431182861328</v>
       </c>
       <c r="E5">
-        <v>228.25621032714844</v>
+        <v>236.02276611328125</v>
       </c>
       <c r="F5">
-        <v>143.90956115722656</v>
+        <v>4.2447381019592285</v>
       </c>
       <c r="G5">
-        <v>137.0200653076172</v>
+        <v>4.48966121673584</v>
       </c>
       <c r="H5">
-        <v>141.85440063476562</v>
+        <v>6.751872539520264</v>
       </c>
       <c r="I5">
-        <v>26278.375</v>
+        <v>973.0674438476562</v>
       </c>
       <c r="J5">
-        <v>24571.931640625</v>
+        <v>960.7402954101562</v>
       </c>
       <c r="K5">
-        <v>25736.556640625</v>
+        <v>1544.5211181640625</v>
       </c>
       <c r="L5">
-        <v>0.7992112636566162</v>
+        <v>0.9652832746505737</v>
       </c>
       <c r="M5">
-        <v>0.7866745591163635</v>
+        <v>0.9058019518852234</v>
       </c>
       <c r="N5">
-        <v>0.7953278422355652</v>
+        <v>0.9692052006721497</v>
       </c>
       <c r="O5">
-        <v>76586.8671875</v>
+        <v>3478.32861328125</v>
       </c>
     </row>
     <row r="6">
@@ -639,46 +639,46 @@
         <v>Kompresorno-5</v>
       </c>
       <c r="B6">
-        <v>27123.76328023742</v>
+        <v>49549.513013736614</v>
       </c>
       <c r="C6">
-        <v>227.05886840820312</v>
+        <v>236.26446533203125</v>
       </c>
       <c r="D6">
-        <v>229.96148681640625</v>
+        <v>233.4344482421875</v>
       </c>
       <c r="E6">
-        <v>224.58837890625</v>
+        <v>233.39625549316406</v>
       </c>
       <c r="F6">
-        <v>70.41529846191406</v>
+        <v>53.212242126464844</v>
       </c>
       <c r="G6">
-        <v>74.52837371826172</v>
+        <v>44.14026641845703</v>
       </c>
       <c r="H6">
-        <v>67.36648559570312</v>
+        <v>48.20628356933594</v>
       </c>
       <c r="I6">
-        <v>13735.98828125</v>
+        <v>10197.775390625</v>
       </c>
       <c r="J6">
-        <v>15235.8056640625</v>
+        <v>8387.74609375</v>
       </c>
       <c r="K6">
-        <v>13375.0498046875</v>
+        <v>8782.8017578125</v>
       </c>
       <c r="L6">
-        <v>0.8591211438179016</v>
+        <v>0.8385860323905945</v>
       </c>
       <c r="M6">
-        <v>0.8889731764793396</v>
+        <v>0.8119436502456665</v>
       </c>
       <c r="N6">
-        <v>0.8850979208946228</v>
+        <v>0.7790775299072266</v>
       </c>
       <c r="O6">
-        <v>42565.5625</v>
+        <v>27368.32421875</v>
       </c>
     </row>
     <row r="7">
@@ -686,98 +686,12 @@
         <v>Priemno-6</v>
       </c>
       <c r="B7">
-        <v>24872.04893086514</v>
-      </c>
-      <c r="C7">
-        <v>228.30458068847656</v>
-      </c>
-      <c r="D7">
-        <v>229.68382263183594</v>
-      </c>
-      <c r="E7">
-        <v>230.26058959960938</v>
-      </c>
-      <c r="F7">
-        <v>108.90827178955078</v>
-      </c>
-      <c r="G7">
-        <v>98.66710662841797</v>
-      </c>
-      <c r="H7">
-        <v>99.50196075439453</v>
-      </c>
-      <c r="I7">
-        <v>22575.791015625</v>
-      </c>
-      <c r="J7">
-        <v>20210.15234375</v>
-      </c>
-      <c r="K7">
-        <v>20241.068359375</v>
-      </c>
-      <c r="L7">
-        <v>0.9053029417991638</v>
-      </c>
-      <c r="M7">
-        <v>0.891526460647583</v>
-      </c>
-      <c r="N7">
-        <v>0.8836268782615662</v>
-      </c>
-      <c r="O7">
-        <v>63027.01171875</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Trafo#1-7</v>
-      </c>
-      <c r="B8">
-        <v>117906.93006688029</v>
-      </c>
-      <c r="C8">
-        <v>229.21128845214844</v>
-      </c>
-      <c r="D8">
-        <v>229.50796508789062</v>
-      </c>
-      <c r="E8">
-        <v>230.92616271972656</v>
-      </c>
-      <c r="F8">
-        <v>463.3951721191406</v>
-      </c>
-      <c r="G8">
-        <v>439.282470703125</v>
-      </c>
-      <c r="H8">
-        <v>442.8319091796875</v>
-      </c>
-      <c r="I8">
-        <v>92228.7265625</v>
-      </c>
-      <c r="J8">
-        <v>85754.6171875</v>
-      </c>
-      <c r="K8">
-        <v>86550.578125</v>
-      </c>
-      <c r="L8">
-        <v>0.8684120178222656</v>
-      </c>
-      <c r="M8">
-        <v>0.8505814671516418</v>
-      </c>
-      <c r="N8">
-        <v>0.8463655114173889</v>
-      </c>
-      <c r="O8">
-        <v>264533.9375</v>
+        <v>-1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
controller can rebot when internet is down
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:O2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -451,247 +451,12 @@
         <v>GRT-1</v>
       </c>
       <c r="B2">
-        <v>138891.53255013344</v>
-      </c>
-      <c r="C2">
-        <v>233.59140014648438</v>
-      </c>
-      <c r="D2">
-        <v>234.11288452148438</v>
-      </c>
-      <c r="E2">
-        <v>236.14212036132812</v>
-      </c>
-      <c r="F2">
-        <v>32.17891311645508</v>
-      </c>
-      <c r="G2">
-        <v>34.63349914550781</v>
-      </c>
-      <c r="H2">
-        <v>36.207763671875</v>
-      </c>
-      <c r="I2">
-        <v>7460.419921875</v>
-      </c>
-      <c r="J2">
-        <v>3562.072998046875</v>
-      </c>
-      <c r="K2">
-        <v>6219.52783203125</v>
-      </c>
-      <c r="L2">
-        <v>0.8150226473808289</v>
-      </c>
-      <c r="M2">
-        <v>0.790442705154419</v>
-      </c>
-      <c r="N2">
-        <v>0.9486470222473145</v>
-      </c>
-      <c r="O2">
-        <v>12619.7255859375</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Ampak-2</v>
-      </c>
-      <c r="B3">
-        <v>41277.116609706674</v>
-      </c>
-      <c r="C3">
-        <v>233.29896545410156</v>
-      </c>
-      <c r="D3">
-        <v>233.5473175048828</v>
-      </c>
-      <c r="E3">
-        <v>236.05038452148438</v>
-      </c>
-      <c r="F3">
-        <v>32.63731384277344</v>
-      </c>
-      <c r="G3">
-        <v>31.923927307128906</v>
-      </c>
-      <c r="H3">
-        <v>25.443716049194336</v>
-      </c>
-      <c r="I3">
-        <v>6615.59814453125</v>
-      </c>
-      <c r="J3">
-        <v>12773.4716796875</v>
-      </c>
-      <c r="K3">
-        <v>12164.94921875</v>
-      </c>
-      <c r="L3">
-        <v>0.9669831991195679</v>
-      </c>
-      <c r="M3">
-        <v>0.9583166837692261</v>
-      </c>
-      <c r="N3">
-        <v>0.9691182374954224</v>
-      </c>
-      <c r="O3">
-        <v>38014.85546875</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Ledena Voda-3</v>
-      </c>
-      <c r="B4">
-        <v>245426.2544324171</v>
-      </c>
-      <c r="C4">
-        <v>236.96189880371094</v>
-      </c>
-      <c r="D4">
-        <v>236.66102600097656</v>
-      </c>
-      <c r="E4">
-        <v>238.5266571044922</v>
-      </c>
-      <c r="F4">
-        <v>0.18555894494056702</v>
-      </c>
-      <c r="G4">
-        <v>0.24126143753528595</v>
-      </c>
-      <c r="H4">
-        <v>0.4243241250514984</v>
-      </c>
-      <c r="I4">
-        <v>35.66485595703125</v>
-      </c>
-      <c r="J4">
-        <v>-10.9794282913208</v>
-      </c>
-      <c r="K4">
-        <v>50.80659484863281</v>
-      </c>
-      <c r="L4">
-        <v>0.8111370205879211</v>
-      </c>
-      <c r="M4">
-        <v>0.19233039021492004</v>
-      </c>
-      <c r="N4">
-        <v>0.5024684071540833</v>
-      </c>
-      <c r="O4">
-        <v>75.49201965332031</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Hladilnici-4</v>
-      </c>
-      <c r="B5">
-        <v>181073.94627291267</v>
-      </c>
-      <c r="C5">
-        <v>237.485595703125</v>
-      </c>
-      <c r="D5">
-        <v>236.2431182861328</v>
-      </c>
-      <c r="E5">
-        <v>236.02276611328125</v>
-      </c>
-      <c r="F5">
-        <v>4.2447381019592285</v>
-      </c>
-      <c r="G5">
-        <v>4.48966121673584</v>
-      </c>
-      <c r="H5">
-        <v>6.751872539520264</v>
-      </c>
-      <c r="I5">
-        <v>973.0674438476562</v>
-      </c>
-      <c r="J5">
-        <v>960.7402954101562</v>
-      </c>
-      <c r="K5">
-        <v>1544.5211181640625</v>
-      </c>
-      <c r="L5">
-        <v>0.9652832746505737</v>
-      </c>
-      <c r="M5">
-        <v>0.9058019518852234</v>
-      </c>
-      <c r="N5">
-        <v>0.9692052006721497</v>
-      </c>
-      <c r="O5">
-        <v>3478.32861328125</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Kompresorno-5</v>
-      </c>
-      <c r="B6">
-        <v>49549.513013736614</v>
-      </c>
-      <c r="C6">
-        <v>236.26446533203125</v>
-      </c>
-      <c r="D6">
-        <v>233.4344482421875</v>
-      </c>
-      <c r="E6">
-        <v>233.39625549316406</v>
-      </c>
-      <c r="F6">
-        <v>53.212242126464844</v>
-      </c>
-      <c r="G6">
-        <v>44.14026641845703</v>
-      </c>
-      <c r="H6">
-        <v>48.20628356933594</v>
-      </c>
-      <c r="I6">
-        <v>10197.775390625</v>
-      </c>
-      <c r="J6">
-        <v>8387.74609375</v>
-      </c>
-      <c r="K6">
-        <v>8782.8017578125</v>
-      </c>
-      <c r="L6">
-        <v>0.8385860323905945</v>
-      </c>
-      <c r="M6">
-        <v>0.8119436502456665</v>
-      </c>
-      <c r="N6">
-        <v>0.7790775299072266</v>
-      </c>
-      <c r="O6">
-        <v>27368.32421875</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Priemno-6</v>
-      </c>
-      <c r="B7">
         <v>-1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
now it can read whit no internet
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -451,12 +451,333 @@
         <v>GRT-1</v>
       </c>
       <c r="B2">
-        <v>-1</v>
+        <v>138972.57177394602</v>
+      </c>
+      <c r="C2">
+        <v>233.02435302734375</v>
+      </c>
+      <c r="D2">
+        <v>228.67605590820312</v>
+      </c>
+      <c r="E2">
+        <v>230.71310424804688</v>
+      </c>
+      <c r="F2">
+        <v>78.19867706298828</v>
+      </c>
+      <c r="G2">
+        <v>53.66566467285156</v>
+      </c>
+      <c r="H2">
+        <v>53.12857437133789</v>
+      </c>
+      <c r="I2">
+        <v>17707.97265625</v>
+      </c>
+      <c r="J2">
+        <v>11653.673828125</v>
+      </c>
+      <c r="K2">
+        <v>11845</v>
+      </c>
+      <c r="L2">
+        <v>0.9771997332572937</v>
+      </c>
+      <c r="M2">
+        <v>0.9673282504081726</v>
+      </c>
+      <c r="N2">
+        <v>0.9568406343460083</v>
+      </c>
+      <c r="O2">
+        <v>43686.55078125</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Ampak-2</v>
+      </c>
+      <c r="B3">
+        <v>41337.72904483644</v>
+      </c>
+      <c r="C3">
+        <v>233.20648193359375</v>
+      </c>
+      <c r="D3">
+        <v>228.24420166015625</v>
+      </c>
+      <c r="E3">
+        <v>230.62147521972656</v>
+      </c>
+      <c r="F3">
+        <v>30.640697479248047</v>
+      </c>
+      <c r="G3">
+        <v>30.053237915039062</v>
+      </c>
+      <c r="H3">
+        <v>21.824016571044922</v>
+      </c>
+      <c r="I3">
+        <v>6432.7578125</v>
+      </c>
+      <c r="J3">
+        <v>6362.45361328125</v>
+      </c>
+      <c r="K3">
+        <v>4064.877685546875</v>
+      </c>
+      <c r="L3">
+        <v>0.9009012579917908</v>
+      </c>
+      <c r="M3">
+        <v>0.9267151355743408</v>
+      </c>
+      <c r="N3">
+        <v>0.8076311349868774</v>
+      </c>
+      <c r="O3">
+        <v>16860.08984375</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Ledena Voda-3</v>
+      </c>
+      <c r="B4">
+        <v>245671.4388525825</v>
+      </c>
+      <c r="C4">
+        <v>216.9678192138672</v>
+      </c>
+      <c r="D4">
+        <v>227.43545532226562</v>
+      </c>
+      <c r="E4">
+        <v>225.81552124023438</v>
+      </c>
+      <c r="F4">
+        <v>415.460205078125</v>
+      </c>
+      <c r="G4">
+        <v>431.6772155761719</v>
+      </c>
+      <c r="H4">
+        <v>452.146484375</v>
+      </c>
+      <c r="I4">
+        <v>71668.4453125</v>
+      </c>
+      <c r="J4">
+        <v>81577.2734375</v>
+      </c>
+      <c r="K4">
+        <v>78834.6484375</v>
+      </c>
+      <c r="L4">
+        <v>0.7950661182403564</v>
+      </c>
+      <c r="M4">
+        <v>0.8309059739112854</v>
+      </c>
+      <c r="N4">
+        <v>0.7726350426673889</v>
+      </c>
+      <c r="O4">
+        <v>232097.625</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Hladilnici-4</v>
+      </c>
+      <c r="B5">
+        <v>181133.76562073742</v>
+      </c>
+      <c r="C5">
+        <v>232.36517333984375</v>
+      </c>
+      <c r="D5">
+        <v>230.73361206054688</v>
+      </c>
+      <c r="E5">
+        <v>230.944580078125</v>
+      </c>
+      <c r="F5">
+        <v>135.97662353515625</v>
+      </c>
+      <c r="G5">
+        <v>130.81976318359375</v>
+      </c>
+      <c r="H5">
+        <v>133.08905029296875</v>
+      </c>
+      <c r="I5">
+        <v>23497.44921875</v>
+      </c>
+      <c r="J5">
+        <v>22390.810546875</v>
+      </c>
+      <c r="K5">
+        <v>23623.208984375</v>
+      </c>
+      <c r="L5">
+        <v>0.7435617446899414</v>
+      </c>
+      <c r="M5">
+        <v>0.7417832016944885</v>
+      </c>
+      <c r="N5">
+        <v>0.7685795426368713</v>
+      </c>
+      <c r="O5">
+        <v>69511.46875</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Kompresorno-5</v>
+      </c>
+      <c r="B6">
+        <v>49648.03699415744</v>
+      </c>
+      <c r="C6">
+        <v>230.18161010742188</v>
+      </c>
+      <c r="D6">
+        <v>231.96978759765625</v>
+      </c>
+      <c r="E6">
+        <v>227.5902099609375</v>
+      </c>
+      <c r="F6">
+        <v>59.44271469116211</v>
+      </c>
+      <c r="G6">
+        <v>62.66370391845703</v>
+      </c>
+      <c r="H6">
+        <v>55.28877258300781</v>
+      </c>
+      <c r="I6">
+        <v>11522.4814453125</v>
+      </c>
+      <c r="J6">
+        <v>12834.419921875</v>
+      </c>
+      <c r="K6">
+        <v>10947.328125</v>
+      </c>
+      <c r="L6">
+        <v>0.842125415802002</v>
+      </c>
+      <c r="M6">
+        <v>0.8829350471496582</v>
+      </c>
+      <c r="N6">
+        <v>0.8699966669082642</v>
+      </c>
+      <c r="O6">
+        <v>35304.2265625</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Priemno-6</v>
+      </c>
+      <c r="B7">
+        <v>59022.4688824011</v>
+      </c>
+      <c r="C7">
+        <v>230.23777770996094</v>
+      </c>
+      <c r="D7">
+        <v>231.36495971679688</v>
+      </c>
+      <c r="E7">
+        <v>232.64874267578125</v>
+      </c>
+      <c r="F7">
+        <v>178.28936767578125</v>
+      </c>
+      <c r="G7">
+        <v>161.32814025878906</v>
+      </c>
+      <c r="H7">
+        <v>169.42849731445312</v>
+      </c>
+      <c r="I7">
+        <v>36384.45703125</v>
+      </c>
+      <c r="J7">
+        <v>32877.23046875</v>
+      </c>
+      <c r="K7">
+        <v>34755.47265625</v>
+      </c>
+      <c r="L7">
+        <v>0.8871427774429321</v>
+      </c>
+      <c r="M7">
+        <v>0.8805782198905945</v>
+      </c>
+      <c r="N7">
+        <v>0.8813016414642334</v>
+      </c>
+      <c r="O7">
+        <v>104017.1640625</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="B8">
+        <v>237711.77615681977</v>
+      </c>
+      <c r="C8">
+        <v>231.53257751464844</v>
+      </c>
+      <c r="D8">
+        <v>231.9860076904297</v>
+      </c>
+      <c r="E8">
+        <v>234.1300811767578</v>
+      </c>
+      <c r="F8">
+        <v>459.37457275390625</v>
+      </c>
+      <c r="G8">
+        <v>446.49237060546875</v>
+      </c>
+      <c r="H8">
+        <v>454.9705505371094</v>
+      </c>
+      <c r="I8">
+        <v>93380.34375</v>
+      </c>
+      <c r="J8">
+        <v>88964.6015625</v>
+      </c>
+      <c r="K8">
+        <v>91752.921875</v>
+      </c>
+      <c r="L8">
+        <v>0.878089189529419</v>
+      </c>
+      <c r="M8">
+        <v>0.8590894341468811</v>
+      </c>
+      <c r="N8">
+        <v>0.8614829778671265</v>
+      </c>
+      <c r="O8">
+        <v>274097.875</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added new way of writing sheet data
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -397,387 +397,1177 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:Q22"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>Date</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Time</v>
+      </c>
+      <c r="C1" t="str">
         <v>Meter Name</v>
       </c>
-      <c r="B1" t="str">
+      <c r="D1" t="str">
         <v>Active Energy</v>
       </c>
-      <c r="C1" t="str">
+      <c r="E1" t="str">
         <v>Voltage L1</v>
       </c>
-      <c r="D1" t="str">
+      <c r="F1" t="str">
         <v>Voltage L2</v>
       </c>
-      <c r="E1" t="str">
+      <c r="G1" t="str">
         <v>Voltage L3</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>Current L1</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>Current L2</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>Current L3</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>Active power L1</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>Active power L2</v>
       </c>
-      <c r="K1" t="str">
+      <c r="M1" t="str">
         <v>Active power L3</v>
       </c>
-      <c r="L1" t="str">
+      <c r="N1" t="str">
         <v>Power factor L1</v>
       </c>
-      <c r="M1" t="str">
+      <c r="O1" t="str">
         <v>Power factor L2</v>
       </c>
-      <c r="N1" t="str">
+      <c r="P1" t="str">
         <v>Power factor L3</v>
       </c>
-      <c r="O1" t="str">
+      <c r="Q1" t="str">
         <v>Total active power</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>23.12.2024 г.</v>
+      </c>
+      <c r="B2" t="str">
+        <v>14:31:02 ч.</v>
+      </c>
+      <c r="C2" t="str">
         <v>GRT-1</v>
       </c>
-      <c r="B2">
-        <v>138972.57177394602</v>
-      </c>
-      <c r="C2">
-        <v>233.02435302734375</v>
-      </c>
       <c r="D2">
-        <v>228.67605590820312</v>
+        <v>138987.5756267055</v>
       </c>
       <c r="E2">
-        <v>230.71310424804688</v>
+        <v>233.97169494628906</v>
       </c>
       <c r="F2">
-        <v>78.19867706298828</v>
+        <v>229.11773681640625</v>
       </c>
       <c r="G2">
-        <v>53.66566467285156</v>
+        <v>230.0638427734375</v>
       </c>
       <c r="H2">
-        <v>53.12857437133789</v>
+        <v>44.31674575805664</v>
       </c>
       <c r="I2">
-        <v>17707.97265625</v>
+        <v>28.622055053710938</v>
       </c>
       <c r="J2">
-        <v>11653.673828125</v>
+        <v>43.06321716308594</v>
       </c>
       <c r="K2">
-        <v>11845</v>
+        <v>12476.7802734375</v>
       </c>
       <c r="L2">
-        <v>0.9771997332572937</v>
+        <v>8280.376953125</v>
       </c>
       <c r="M2">
-        <v>0.9673282504081726</v>
+        <v>9259.6689453125</v>
       </c>
       <c r="N2">
-        <v>0.9568406343460083</v>
+        <v>0.951461911201477</v>
       </c>
       <c r="O2">
-        <v>43686.55078125</v>
+        <v>0.8834019899368286</v>
+      </c>
+      <c r="P2">
+        <v>0.9341639876365662</v>
+      </c>
+      <c r="Q2">
+        <v>27938.751953125</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>23.12.2024 г.</v>
+      </c>
+      <c r="B3" t="str">
+        <v>14:31:02 ч.</v>
+      </c>
+      <c r="C3" t="str">
         <v>Ampak-2</v>
       </c>
-      <c r="B3">
-        <v>41337.72904483644</v>
-      </c>
-      <c r="C3">
-        <v>233.20648193359375</v>
-      </c>
       <c r="D3">
-        <v>228.24420166015625</v>
+        <v>41346.78481988183</v>
       </c>
       <c r="E3">
-        <v>230.62147521972656</v>
+        <v>233.9862823486328</v>
       </c>
       <c r="F3">
-        <v>30.640697479248047</v>
+        <v>228.604736328125</v>
       </c>
       <c r="G3">
-        <v>30.053237915039062</v>
+        <v>230.3919677734375</v>
       </c>
       <c r="H3">
-        <v>21.824016571044922</v>
+        <v>32.691932678222656</v>
       </c>
       <c r="I3">
-        <v>6432.7578125</v>
+        <v>24.041351318359375</v>
       </c>
       <c r="J3">
-        <v>6362.45361328125</v>
+        <v>22.397602081298828</v>
       </c>
       <c r="K3">
-        <v>4064.877685546875</v>
+        <v>6877.10546875</v>
       </c>
       <c r="L3">
-        <v>0.9009012579917908</v>
+        <v>4801.4931640625</v>
       </c>
       <c r="M3">
-        <v>0.9267151355743408</v>
+        <v>3991.1064453125</v>
       </c>
       <c r="N3">
-        <v>0.8076311349868774</v>
+        <v>0.8986256122589111</v>
       </c>
       <c r="O3">
-        <v>16860.08984375</v>
+        <v>0.8732107877731323</v>
+      </c>
+      <c r="P3">
+        <v>0.7734361290931702</v>
+      </c>
+      <c r="Q3">
+        <v>15669.705078125</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>23.12.2024 г.</v>
+      </c>
+      <c r="B4" t="str">
+        <v>14:31:02 ч.</v>
+      </c>
+      <c r="C4" t="str">
         <v>Ledena Voda-3</v>
       </c>
-      <c r="B4">
-        <v>245671.4388525825</v>
-      </c>
-      <c r="C4">
-        <v>216.9678192138672</v>
-      </c>
       <c r="D4">
-        <v>227.43545532226562</v>
+        <v>245779.0725968223</v>
       </c>
       <c r="E4">
-        <v>225.81552124023438</v>
+        <v>216.92747497558594</v>
       </c>
       <c r="F4">
-        <v>415.460205078125</v>
+        <v>227.7540283203125</v>
       </c>
       <c r="G4">
-        <v>431.6772155761719</v>
+        <v>225.33023071289062</v>
       </c>
       <c r="H4">
-        <v>452.146484375</v>
+        <v>416.38360595703125</v>
       </c>
       <c r="I4">
-        <v>71668.4453125</v>
+        <v>430.85931396484375</v>
       </c>
       <c r="J4">
-        <v>81577.2734375</v>
+        <v>451.3459777832031</v>
       </c>
       <c r="K4">
-        <v>78834.6484375</v>
+        <v>72526.265625</v>
       </c>
       <c r="L4">
-        <v>0.7950661182403564</v>
+        <v>82009.578125</v>
       </c>
       <c r="M4">
-        <v>0.8309059739112854</v>
+        <v>79285.1875</v>
       </c>
       <c r="N4">
-        <v>0.7726350426673889</v>
+        <v>0.8029475212097168</v>
       </c>
       <c r="O4">
-        <v>232097.625</v>
+        <v>0.8357243537902832</v>
+      </c>
+      <c r="P4">
+        <v>0.7795842289924622</v>
+      </c>
+      <c r="Q4">
+        <v>233821.03125</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>23.12.2024 г.</v>
+      </c>
+      <c r="B5" t="str">
+        <v>14:31:02 ч.</v>
+      </c>
+      <c r="C5" t="str">
         <v>Hladilnici-4</v>
       </c>
-      <c r="B5">
-        <v>181133.76562073742</v>
-      </c>
-      <c r="C5">
-        <v>232.36517333984375</v>
-      </c>
       <c r="D5">
-        <v>230.73361206054688</v>
+        <v>181155.92401194514</v>
       </c>
       <c r="E5">
-        <v>230.944580078125</v>
+        <v>232.39183044433594</v>
       </c>
       <c r="F5">
-        <v>135.97662353515625</v>
+        <v>230.99398803710938</v>
       </c>
       <c r="G5">
-        <v>130.81976318359375</v>
+        <v>231.28884887695312</v>
       </c>
       <c r="H5">
-        <v>133.08905029296875</v>
+        <v>118.58063507080078</v>
       </c>
       <c r="I5">
-        <v>23497.44921875</v>
+        <v>114.51309204101562</v>
       </c>
       <c r="J5">
-        <v>22390.810546875</v>
+        <v>118.57257843017578</v>
       </c>
       <c r="K5">
-        <v>23623.208984375</v>
+        <v>20499.34765625</v>
       </c>
       <c r="L5">
-        <v>0.7435617446899414</v>
+        <v>19805.08984375</v>
       </c>
       <c r="M5">
-        <v>0.7417832016944885</v>
+        <v>21250.53125</v>
       </c>
       <c r="N5">
-        <v>0.7685795426368713</v>
+        <v>0.7438843846321106</v>
       </c>
       <c r="O5">
-        <v>69511.46875</v>
+        <v>0.7487226128578186</v>
+      </c>
+      <c r="P5">
+        <v>0.7762773036956787</v>
+      </c>
+      <c r="Q5">
+        <v>61562.09375</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>23.12.2024 г.</v>
+      </c>
+      <c r="B6" t="str">
+        <v>14:31:02 ч.</v>
+      </c>
+      <c r="C6" t="str">
         <v>Kompresorno-5</v>
       </c>
-      <c r="B6">
-        <v>49648.03699415744</v>
-      </c>
-      <c r="C6">
-        <v>230.18161010742188</v>
-      </c>
       <c r="D6">
-        <v>231.96978759765625</v>
+        <v>49664.48563194836</v>
       </c>
       <c r="E6">
-        <v>227.5902099609375</v>
+        <v>230.3798370361328</v>
       </c>
       <c r="F6">
-        <v>59.44271469116211</v>
+        <v>233.77122497558594</v>
       </c>
       <c r="G6">
-        <v>62.66370391845703</v>
+        <v>228.1894989013672</v>
       </c>
       <c r="H6">
-        <v>55.28877258300781</v>
+        <v>61.7668342590332</v>
       </c>
       <c r="I6">
-        <v>11522.4814453125</v>
+        <v>63.97842788696289</v>
       </c>
       <c r="J6">
-        <v>12834.419921875</v>
+        <v>57.77893829345703</v>
       </c>
       <c r="K6">
-        <v>10947.328125</v>
+        <v>12084.7470703125</v>
       </c>
       <c r="L6">
-        <v>0.842125415802002</v>
+        <v>13183.4765625</v>
       </c>
       <c r="M6">
-        <v>0.8829350471496582</v>
+        <v>11505.01171875</v>
       </c>
       <c r="N6">
-        <v>0.8699966669082642</v>
+        <v>0.8501742482185364</v>
       </c>
       <c r="O6">
-        <v>35304.2265625</v>
+        <v>0.8847309350967407</v>
+      </c>
+      <c r="P6">
+        <v>0.8726133704185486</v>
+      </c>
+      <c r="Q6">
+        <v>36773.234375</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
+        <v>23.12.2024 г.</v>
+      </c>
+      <c r="B7" t="str">
+        <v>14:31:02 ч.</v>
+      </c>
+      <c r="C7" t="str">
         <v>Priemno-6</v>
       </c>
-      <c r="B7">
-        <v>59022.4688824011</v>
-      </c>
-      <c r="C7">
-        <v>230.23777770996094</v>
-      </c>
       <c r="D7">
-        <v>231.36495971679688</v>
+        <v>59068.367265375724</v>
       </c>
       <c r="E7">
-        <v>232.64874267578125</v>
+        <v>230.13314819335938</v>
       </c>
       <c r="F7">
-        <v>178.28936767578125</v>
+        <v>231.38917541503906</v>
       </c>
       <c r="G7">
-        <v>161.32814025878906</v>
+        <v>232.70306396484375</v>
       </c>
       <c r="H7">
-        <v>169.42849731445312</v>
+        <v>154.28164672851562</v>
       </c>
       <c r="I7">
-        <v>36384.45703125</v>
+        <v>138.1094970703125</v>
       </c>
       <c r="J7">
-        <v>32877.23046875</v>
+        <v>144.01779174804688</v>
       </c>
       <c r="K7">
-        <v>34755.47265625</v>
+        <v>31394.392578125</v>
       </c>
       <c r="L7">
-        <v>0.8871427774429321</v>
+        <v>27967.46484375</v>
       </c>
       <c r="M7">
-        <v>0.8805782198905945</v>
+        <v>29055.498046875</v>
       </c>
       <c r="N7">
-        <v>0.8813016414642334</v>
+        <v>0.8840821981430054</v>
       </c>
       <c r="O7">
-        <v>104017.1640625</v>
+        <v>0.8752752542495728</v>
+      </c>
+      <c r="P7">
+        <v>0.8710250854492188</v>
+      </c>
+      <c r="Q7">
+        <v>88187.1953125</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>23.12.2024 г.</v>
+      </c>
+      <c r="B8" t="str">
+        <v>14:31:02 ч.</v>
+      </c>
+      <c r="C8" t="str">
         <v>Trafo#1-7</v>
       </c>
-      <c r="B8">
-        <v>237711.77615681977</v>
-      </c>
-      <c r="C8">
-        <v>231.53257751464844</v>
-      </c>
       <c r="D8">
-        <v>231.9860076904297</v>
+        <v>237830.03480002732</v>
       </c>
       <c r="E8">
-        <v>234.1300811767578</v>
+        <v>231.3763427734375</v>
       </c>
       <c r="F8">
-        <v>459.37457275390625</v>
+        <v>231.7626190185547</v>
       </c>
       <c r="G8">
-        <v>446.49237060546875</v>
+        <v>233.90667724609375</v>
       </c>
       <c r="H8">
-        <v>454.9705505371094</v>
+        <v>433.1043701171875</v>
       </c>
       <c r="I8">
-        <v>93380.34375</v>
+        <v>420.84783935546875</v>
       </c>
       <c r="J8">
-        <v>88964.6015625</v>
+        <v>432.7939453125</v>
       </c>
       <c r="K8">
-        <v>91752.921875</v>
+        <v>88133.2421875</v>
       </c>
       <c r="L8">
-        <v>0.878089189529419</v>
+        <v>83746.7734375</v>
       </c>
       <c r="M8">
-        <v>0.8590894341468811</v>
+        <v>87312.7890625</v>
       </c>
       <c r="N8">
-        <v>0.8614829778671265</v>
+        <v>0.8794845342636108</v>
       </c>
       <c r="O8">
-        <v>274097.875</v>
+        <v>0.8586172461509705</v>
+      </c>
+      <c r="P8">
+        <v>0.8624899983406067</v>
+      </c>
+      <c r="Q8">
+        <v>259192.796875</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>23.12.2024 г.</v>
+      </c>
+      <c r="B9" t="str">
+        <v>14:33:02 ч.</v>
+      </c>
+      <c r="C9" t="str">
+        <v>GRT-1</v>
+      </c>
+      <c r="D9">
+        <v>138988.70168527492</v>
+      </c>
+      <c r="E9">
+        <v>232.78439331054688</v>
+      </c>
+      <c r="F9">
+        <v>227.9639892578125</v>
+      </c>
+      <c r="G9">
+        <v>230.39898681640625</v>
+      </c>
+      <c r="H9">
+        <v>86.29752349853516</v>
+      </c>
+      <c r="I9">
+        <v>62.01639938354492</v>
+      </c>
+      <c r="J9">
+        <v>51.766597747802734</v>
+      </c>
+      <c r="K9">
+        <v>17194.306640625</v>
+      </c>
+      <c r="L9">
+        <v>11238.873046875</v>
+      </c>
+      <c r="M9">
+        <v>11279.9921875</v>
+      </c>
+      <c r="N9">
+        <v>0.9761987328529358</v>
+      </c>
+      <c r="O9">
+        <v>0.9617502093315125</v>
+      </c>
+      <c r="P9">
+        <v>0.9448742866516113</v>
+      </c>
+      <c r="Q9">
+        <v>36221.08984375</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>23.12.2024 г.</v>
+      </c>
+      <c r="B10" t="str">
+        <v>14:33:02 ч.</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Ampak-2</v>
+      </c>
+      <c r="D10">
+        <v>41347.467485822955</v>
+      </c>
+      <c r="E10">
+        <v>233.6977081298828</v>
+      </c>
+      <c r="F10">
+        <v>228.23406982421875</v>
+      </c>
+      <c r="G10">
+        <v>230.61932373046875</v>
+      </c>
+      <c r="H10">
+        <v>31.952651977539062</v>
+      </c>
+      <c r="I10">
+        <v>29.127277374267578</v>
+      </c>
+      <c r="J10">
+        <v>21.742889404296875</v>
+      </c>
+      <c r="K10">
+        <v>6778.09375</v>
+      </c>
+      <c r="L10">
+        <v>6096.57177734375</v>
+      </c>
+      <c r="M10">
+        <v>3986.06103515625</v>
+      </c>
+      <c r="N10">
+        <v>0.909540057182312</v>
+      </c>
+      <c r="O10">
+        <v>0.9173862338066101</v>
+      </c>
+      <c r="P10">
+        <v>0.7949338555335999</v>
+      </c>
+      <c r="Q10">
+        <v>16860.7265625</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>23.12.2024 г.</v>
+      </c>
+      <c r="B11" t="str">
+        <v>14:33:02 ч.</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Ledena Voda-3</v>
+      </c>
+      <c r="D11">
+        <v>245786.8697305408</v>
+      </c>
+      <c r="E11">
+        <v>217.36993408203125</v>
+      </c>
+      <c r="F11">
+        <v>228.03318786621094</v>
+      </c>
+      <c r="G11">
+        <v>226.19741821289062</v>
+      </c>
+      <c r="H11">
+        <v>411.15802001953125</v>
+      </c>
+      <c r="I11">
+        <v>427.0341491699219</v>
+      </c>
+      <c r="J11">
+        <v>447.12213134765625</v>
+      </c>
+      <c r="K11">
+        <v>71339.890625</v>
+      </c>
+      <c r="L11">
+        <v>81146.6328125</v>
+      </c>
+      <c r="M11">
+        <v>78392.5</v>
+      </c>
+      <c r="N11">
+        <v>0.7982229590415955</v>
+      </c>
+      <c r="O11">
+        <v>0.8333162069320679</v>
+      </c>
+      <c r="P11">
+        <v>0.7751052975654602</v>
+      </c>
+      <c r="Q11">
+        <v>230879.03125</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>23.12.2024 г.</v>
+      </c>
+      <c r="B12" t="str">
+        <v>14:33:02 ч.</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Hladilnici-4</v>
+      </c>
+      <c r="D12">
+        <v>181157.74180387773</v>
+      </c>
+      <c r="E12">
+        <v>233.1964569091797</v>
+      </c>
+      <c r="F12">
+        <v>231.5274658203125</v>
+      </c>
+      <c r="G12">
+        <v>231.87860107421875</v>
+      </c>
+      <c r="H12">
+        <v>75.93072509765625</v>
+      </c>
+      <c r="I12">
+        <v>74.73974609375</v>
+      </c>
+      <c r="J12">
+        <v>78.40796661376953</v>
+      </c>
+      <c r="K12">
+        <v>12658.7197265625</v>
+      </c>
+      <c r="L12">
+        <v>12535.115234375</v>
+      </c>
+      <c r="M12">
+        <v>13804.1416015625</v>
+      </c>
+      <c r="N12">
+        <v>0.7146540880203247</v>
+      </c>
+      <c r="O12">
+        <v>0.7245587706565857</v>
+      </c>
+      <c r="P12">
+        <v>0.7591849565505981</v>
+      </c>
+      <c r="Q12">
+        <v>39008.01953125</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>23.12.2024 г.</v>
+      </c>
+      <c r="B13" t="str">
+        <v>14:33:02 ч.</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Kompresorno-5</v>
+      </c>
+      <c r="D13">
+        <v>49665.70160216702</v>
+      </c>
+      <c r="E13">
+        <v>230.8756866455078</v>
+      </c>
+      <c r="F13">
+        <v>233.74951171875</v>
+      </c>
+      <c r="G13">
+        <v>228.46600341796875</v>
+      </c>
+      <c r="H13">
+        <v>61.081966400146484</v>
+      </c>
+      <c r="I13">
+        <v>63.50481033325195</v>
+      </c>
+      <c r="J13">
+        <v>57.122154235839844</v>
+      </c>
+      <c r="K13">
+        <v>11962.6162109375</v>
+      </c>
+      <c r="L13">
+        <v>13116.236328125</v>
+      </c>
+      <c r="M13">
+        <v>11359.6240234375</v>
+      </c>
+      <c r="N13">
+        <v>0.8487828373908997</v>
+      </c>
+      <c r="O13">
+        <v>0.8835922479629517</v>
+      </c>
+      <c r="P13">
+        <v>0.8704379200935364</v>
+      </c>
+      <c r="Q13">
+        <v>36438.4765625</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>23.12.2024 г.</v>
+      </c>
+      <c r="B14" t="str">
+        <v>14:33:02 ч.</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Priemno-6</v>
+      </c>
+      <c r="D14">
+        <v>59071.33243934023</v>
+      </c>
+      <c r="E14">
+        <v>230.65895080566406</v>
+      </c>
+      <c r="F14">
+        <v>232.17489624023438</v>
+      </c>
+      <c r="G14">
+        <v>233.32534790039062</v>
+      </c>
+      <c r="H14">
+        <v>154.385498046875</v>
+      </c>
+      <c r="I14">
+        <v>139.25413513183594</v>
+      </c>
+      <c r="J14">
+        <v>144.87010192871094</v>
+      </c>
+      <c r="K14">
+        <v>31392.638671875</v>
+      </c>
+      <c r="L14">
+        <v>28212.337890625</v>
+      </c>
+      <c r="M14">
+        <v>29443.6171875</v>
+      </c>
+      <c r="N14">
+        <v>0.8821487426757812</v>
+      </c>
+      <c r="O14">
+        <v>0.8745988011360168</v>
+      </c>
+      <c r="P14">
+        <v>0.870652973651886</v>
+      </c>
+      <c r="Q14">
+        <v>89048.59375</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>23.12.2024 г.</v>
+      </c>
+      <c r="B15" t="str">
+        <v>14:33:02 ч.</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="D15">
+        <v>237838.59757922692</v>
+      </c>
+      <c r="E15">
+        <v>231.94664001464844</v>
+      </c>
+      <c r="F15">
+        <v>232.24468994140625</v>
+      </c>
+      <c r="G15">
+        <v>234.3175811767578</v>
+      </c>
+      <c r="H15">
+        <v>405.49859619140625</v>
+      </c>
+      <c r="I15">
+        <v>397.1994323730469</v>
+      </c>
+      <c r="J15">
+        <v>407.0566711425781</v>
+      </c>
+      <c r="K15">
+        <v>82369.453125</v>
+      </c>
+      <c r="L15">
+        <v>79267.9765625</v>
+      </c>
+      <c r="M15">
+        <v>82161.8671875</v>
+      </c>
+      <c r="N15">
+        <v>0.8757672905921936</v>
+      </c>
+      <c r="O15">
+        <v>0.8592970967292786</v>
+      </c>
+      <c r="P15">
+        <v>0.8582150340080261</v>
+      </c>
+      <c r="Q15">
+        <v>240302.125</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>23.12.2024 г.</v>
+      </c>
+      <c r="B16" t="str">
+        <v>14:35:02 ч.</v>
+      </c>
+      <c r="C16" t="str">
+        <v>GRT-1</v>
+      </c>
+      <c r="D16">
+        <v>138989.78438496383</v>
+      </c>
+      <c r="E16">
+        <v>232.69252014160156</v>
+      </c>
+      <c r="F16">
+        <v>228.14930725097656</v>
+      </c>
+      <c r="G16">
+        <v>230.12881469726562</v>
+      </c>
+      <c r="H16">
+        <v>69.36378479003906</v>
+      </c>
+      <c r="I16">
+        <v>67.13031768798828</v>
+      </c>
+      <c r="J16">
+        <v>68.61233520507812</v>
+      </c>
+      <c r="K16">
+        <v>20017.349609375</v>
+      </c>
+      <c r="L16">
+        <v>15002.18359375</v>
+      </c>
+      <c r="M16">
+        <v>15264.515625</v>
+      </c>
+      <c r="N16">
+        <v>0.9859331250190735</v>
+      </c>
+      <c r="O16">
+        <v>0.9812178611755371</v>
+      </c>
+      <c r="P16">
+        <v>0.9661869406700134</v>
+      </c>
+      <c r="Q16">
+        <v>34670.4921875</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>23.12.2024 г.</v>
+      </c>
+      <c r="B17" t="str">
+        <v>14:35:02 ч.</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Ampak-2</v>
+      </c>
+      <c r="D17">
+        <v>41348.15785646919</v>
+      </c>
+      <c r="E17">
+        <v>233.21351623535156</v>
+      </c>
+      <c r="F17">
+        <v>227.87913513183594</v>
+      </c>
+      <c r="G17">
+        <v>230.38169860839844</v>
+      </c>
+      <c r="H17">
+        <v>31.613910675048828</v>
+      </c>
+      <c r="I17">
+        <v>27.994688034057617</v>
+      </c>
+      <c r="J17">
+        <v>22.61420440673828</v>
+      </c>
+      <c r="K17">
+        <v>6533.1689453125</v>
+      </c>
+      <c r="L17">
+        <v>5594.0126953125</v>
+      </c>
+      <c r="M17">
+        <v>4153.4892578125</v>
+      </c>
+      <c r="N17">
+        <v>0.8869346976280212</v>
+      </c>
+      <c r="O17">
+        <v>0.8768863081932068</v>
+      </c>
+      <c r="P17">
+        <v>0.7972303628921509</v>
+      </c>
+      <c r="Q17">
+        <v>16280.669921875</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>23.12.2024 г.</v>
+      </c>
+      <c r="B18" t="str">
+        <v>14:35:02 ч.</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Ledena Voda-3</v>
+      </c>
+      <c r="D18">
+        <v>245794.42821694905</v>
+      </c>
+      <c r="E18">
+        <v>217.15158081054688</v>
+      </c>
+      <c r="F18">
+        <v>227.47239685058594</v>
+      </c>
+      <c r="G18">
+        <v>225.67738342285156</v>
+      </c>
+      <c r="H18">
+        <v>409.4804382324219</v>
+      </c>
+      <c r="I18">
+        <v>422.5149230957031</v>
+      </c>
+      <c r="J18">
+        <v>445.4045104980469</v>
+      </c>
+      <c r="K18">
+        <v>70492.203125</v>
+      </c>
+      <c r="L18">
+        <v>79812.28125</v>
+      </c>
+      <c r="M18">
+        <v>77746.6484375</v>
+      </c>
+      <c r="N18">
+        <v>0.7927657961845398</v>
+      </c>
+      <c r="O18">
+        <v>0.8304222822189331</v>
+      </c>
+      <c r="P18">
+        <v>0.7734620571136475</v>
+      </c>
+      <c r="Q18">
+        <v>228051.125</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>23.12.2024 г.</v>
+      </c>
+      <c r="B19" t="str">
+        <v>14:35:02 ч.</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Hladilnici-4</v>
+      </c>
+      <c r="D19">
+        <v>181159.45246995293</v>
+      </c>
+      <c r="E19">
+        <v>232.59686279296875</v>
+      </c>
+      <c r="F19">
+        <v>231.04505920410156</v>
+      </c>
+      <c r="G19">
+        <v>231.04832458496094</v>
+      </c>
+      <c r="H19">
+        <v>106.71151733398438</v>
+      </c>
+      <c r="I19">
+        <v>102.04054260253906</v>
+      </c>
+      <c r="J19">
+        <v>105.11617279052734</v>
+      </c>
+      <c r="K19">
+        <v>18832.953125</v>
+      </c>
+      <c r="L19">
+        <v>17696.3828125</v>
+      </c>
+      <c r="M19">
+        <v>18937.544921875</v>
+      </c>
+      <c r="N19">
+        <v>0.7587579488754272</v>
+      </c>
+      <c r="O19">
+        <v>0.7506112456321716</v>
+      </c>
+      <c r="P19">
+        <v>0.7804346084594727</v>
+      </c>
+      <c r="Q19">
+        <v>55354.73828125</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>23.12.2024 г.</v>
+      </c>
+      <c r="B20" t="str">
+        <v>14:35:02 ч.</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Kompresorno-5</v>
+      </c>
+      <c r="D20">
+        <v>49666.9169553479</v>
+      </c>
+      <c r="E20">
+        <v>230.7620849609375</v>
+      </c>
+      <c r="F20">
+        <v>233.38270568847656</v>
+      </c>
+      <c r="G20">
+        <v>228.1303253173828</v>
+      </c>
+      <c r="H20">
+        <v>61.18912124633789</v>
+      </c>
+      <c r="I20">
+        <v>63.53916931152344</v>
+      </c>
+      <c r="J20">
+        <v>57.5395622253418</v>
+      </c>
+      <c r="K20">
+        <v>11945.3701171875</v>
+      </c>
+      <c r="L20">
+        <v>13075.8310546875</v>
+      </c>
+      <c r="M20">
+        <v>11395.3662109375</v>
+      </c>
+      <c r="N20">
+        <v>0.8468726873397827</v>
+      </c>
+      <c r="O20">
+        <v>0.8817775845527649</v>
+      </c>
+      <c r="P20">
+        <v>0.8681178689002991</v>
+      </c>
+      <c r="Q20">
+        <v>36416.56640625</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>23.12.2024 г.</v>
+      </c>
+      <c r="B21" t="str">
+        <v>14:35:02 ч.</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Priemno-6</v>
+      </c>
+      <c r="D21">
+        <v>59074.34145974504</v>
+      </c>
+      <c r="E21">
+        <v>230.57603454589844</v>
+      </c>
+      <c r="F21">
+        <v>231.75135803222656</v>
+      </c>
+      <c r="G21">
+        <v>233.10556030273438</v>
+      </c>
+      <c r="H21">
+        <v>155.58944702148438</v>
+      </c>
+      <c r="I21">
+        <v>138.60610961914062</v>
+      </c>
+      <c r="J21">
+        <v>143.5069580078125</v>
+      </c>
+      <c r="K21">
+        <v>31804.373046875</v>
+      </c>
+      <c r="L21">
+        <v>27910.1171875</v>
+      </c>
+      <c r="M21">
+        <v>29100.109375</v>
+      </c>
+      <c r="N21">
+        <v>0.8846926689147949</v>
+      </c>
+      <c r="O21">
+        <v>0.870451033115387</v>
+      </c>
+      <c r="P21">
+        <v>0.8709163665771484</v>
+      </c>
+      <c r="Q21">
+        <v>88814.59375</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>23.12.2024 г.</v>
+      </c>
+      <c r="B22" t="str">
+        <v>14:35:02 ч.</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="D22">
+        <v>237846.99347524397</v>
+      </c>
+      <c r="E22">
+        <v>231.53598022460938</v>
+      </c>
+      <c r="F22">
+        <v>232.08328247070312</v>
+      </c>
+      <c r="G22">
+        <v>234.13307189941406</v>
+      </c>
+      <c r="H22">
+        <v>430.6531982421875</v>
+      </c>
+      <c r="I22">
+        <v>422.250732421875</v>
+      </c>
+      <c r="J22">
+        <v>423.9256896972656</v>
+      </c>
+      <c r="K22">
+        <v>87790.5234375</v>
+      </c>
+      <c r="L22">
+        <v>84725.65625</v>
+      </c>
+      <c r="M22">
+        <v>85751.21875</v>
+      </c>
+      <c r="N22">
+        <v>0.8804435133934021</v>
+      </c>
+      <c r="O22">
+        <v>0.8645710349082947</v>
+      </c>
+      <c r="P22">
+        <v>0.863948404788971</v>
+      </c>
+      <c r="Q22">
+        <v>248752.265625</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Now the system reads if there is no internet and sends data when internet arives to the system
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -992,7 +992,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q131"/>
+  <dimension ref="A1:Q204"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7937,9 +7937,3878 @@
         <v>258.9279479980469</v>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B132" t="str">
+        <v>10:05:52 ч.</v>
+      </c>
+      <c r="C132" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D132">
+        <v>139038.82966594945</v>
+      </c>
+      <c r="E132">
+        <v>234.3379364013672</v>
+      </c>
+      <c r="F132">
+        <v>234.25074768066406</v>
+      </c>
+      <c r="G132">
+        <v>236.3994598388672</v>
+      </c>
+      <c r="H132">
+        <v>1.596269965171814</v>
+      </c>
+      <c r="I132">
+        <v>1.6259244680404663</v>
+      </c>
+      <c r="J132">
+        <v>1.4595266580581665</v>
+      </c>
+      <c r="K132">
+        <v>267.5269775390625</v>
+      </c>
+      <c r="L132">
+        <v>199.90513610839844</v>
+      </c>
+      <c r="M132">
+        <v>212.3627166748047</v>
+      </c>
+      <c r="N132">
+        <v>0.7163926959037781</v>
+      </c>
+      <c r="O132">
+        <v>0.5262004733085632</v>
+      </c>
+      <c r="P132">
+        <v>0.6177560687065125</v>
+      </c>
+      <c r="Q132">
+        <v>682.6998901367188</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B133" t="str">
+        <v>10:05:52 ч.</v>
+      </c>
+      <c r="C133" t="str">
+        <v>Ampak</v>
+      </c>
+      <c r="D133">
+        <v>41468.11233721404</v>
+      </c>
+      <c r="E133">
+        <v>234.22459411621094</v>
+      </c>
+      <c r="F133">
+        <v>233.80526733398438</v>
+      </c>
+      <c r="G133">
+        <v>236.34405517578125</v>
+      </c>
+      <c r="H133">
+        <v>28.35898208618164</v>
+      </c>
+      <c r="I133">
+        <v>26.11907196044922</v>
+      </c>
+      <c r="J133">
+        <v>23.58832359313965</v>
+      </c>
+      <c r="K133">
+        <v>5681.552734375</v>
+      </c>
+      <c r="L133">
+        <v>4940.8427734375</v>
+      </c>
+      <c r="M133">
+        <v>4686.970703125</v>
+      </c>
+      <c r="N133">
+        <v>0.8550119400024414</v>
+      </c>
+      <c r="O133">
+        <v>0.8085864186286926</v>
+      </c>
+      <c r="P133">
+        <v>0.8408719301223755</v>
+      </c>
+      <c r="Q133">
+        <v>15309.365234375</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B134" t="str">
+        <v>10:05:52 ч.</v>
+      </c>
+      <c r="C134" t="str">
+        <v>Ledena Voda</v>
+      </c>
+      <c r="D134">
+        <v>246437.48456314032</v>
+      </c>
+      <c r="E134">
+        <v>236.73129272460938</v>
+      </c>
+      <c r="F134">
+        <v>236.8014373779297</v>
+      </c>
+      <c r="G134">
+        <v>238.53994750976562</v>
+      </c>
+      <c r="H134">
+        <v>0.17195656895637512</v>
+      </c>
+      <c r="I134">
+        <v>0.25974810123443604</v>
+      </c>
+      <c r="J134">
+        <v>0.4380113184452057</v>
+      </c>
+      <c r="K134">
+        <v>32.49019241333008</v>
+      </c>
+      <c r="L134">
+        <v>-15.475045204162598</v>
+      </c>
+      <c r="M134">
+        <v>54.018035888671875</v>
+      </c>
+      <c r="N134">
+        <v>0.7981376647949219</v>
+      </c>
+      <c r="O134">
+        <v>0.2515910863876343</v>
+      </c>
+      <c r="P134">
+        <v>0.5170021653175354</v>
+      </c>
+      <c r="Q134">
+        <v>71.0331802368164</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B135" t="str">
+        <v>10:05:52 ч.</v>
+      </c>
+      <c r="C135" t="str">
+        <v>Hladilnici</v>
+      </c>
+      <c r="D135">
+        <v>181733.25036826535</v>
+      </c>
+      <c r="E135">
+        <v>237.9813995361328</v>
+      </c>
+      <c r="F135">
+        <v>236.27490234375</v>
+      </c>
+      <c r="G135">
+        <v>236.24462890625</v>
+      </c>
+      <c r="H135">
+        <v>9.764253616333008</v>
+      </c>
+      <c r="I135">
+        <v>8.86584186553955</v>
+      </c>
+      <c r="J135">
+        <v>11.950848579406738</v>
+      </c>
+      <c r="K135">
+        <v>1934.1417236328125</v>
+      </c>
+      <c r="L135">
+        <v>1747.9234619140625</v>
+      </c>
+      <c r="M135">
+        <v>2604.105712890625</v>
+      </c>
+      <c r="N135">
+        <v>0.832350492477417</v>
+      </c>
+      <c r="O135">
+        <v>0.8344202637672424</v>
+      </c>
+      <c r="P135">
+        <v>0.9228771924972534</v>
+      </c>
+      <c r="Q135">
+        <v>6278.93017578125</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B136" t="str">
+        <v>10:05:52 ч.</v>
+      </c>
+      <c r="C136" t="str">
+        <v>Kompresorno</v>
+      </c>
+      <c r="D136">
+        <v>49908.94625115918</v>
+      </c>
+      <c r="E136">
+        <v>236.18849182128906</v>
+      </c>
+      <c r="F136">
+        <v>233.78163146972656</v>
+      </c>
+      <c r="G136">
+        <v>233.20616149902344</v>
+      </c>
+      <c r="H136">
+        <v>48.48004913330078</v>
+      </c>
+      <c r="I136">
+        <v>38.980777740478516</v>
+      </c>
+      <c r="J136">
+        <v>42.89822006225586</v>
+      </c>
+      <c r="K136">
+        <v>9493.46484375</v>
+      </c>
+      <c r="L136">
+        <v>7359.7451171875</v>
+      </c>
+      <c r="M136">
+        <v>7474.52392578125</v>
+      </c>
+      <c r="N136">
+        <v>0.8306685090065002</v>
+      </c>
+      <c r="O136">
+        <v>0.8090044856071472</v>
+      </c>
+      <c r="P136">
+        <v>0.7398101687431335</v>
+      </c>
+      <c r="Q136">
+        <v>24577.802734375</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B137" t="str">
+        <v>10:05:52 ч.</v>
+      </c>
+      <c r="C137" t="str">
+        <v>Priemno</v>
+      </c>
+      <c r="D137">
+        <v>59430.81839353656</v>
+      </c>
+      <c r="E137">
+        <v>235.5655059814453</v>
+      </c>
+      <c r="F137">
+        <v>236.27061462402344</v>
+      </c>
+      <c r="G137">
+        <v>237.86557006835938</v>
+      </c>
+      <c r="H137">
+        <v>46.149818420410156</v>
+      </c>
+      <c r="I137">
+        <v>38.80215835571289</v>
+      </c>
+      <c r="J137">
+        <v>41.217498779296875</v>
+      </c>
+      <c r="K137">
+        <v>6248.7626953125</v>
+      </c>
+      <c r="L137">
+        <v>4457.24755859375</v>
+      </c>
+      <c r="M137">
+        <v>4367.04296875</v>
+      </c>
+      <c r="N137">
+        <v>0.574813961982727</v>
+      </c>
+      <c r="O137">
+        <v>0.48618456721305847</v>
+      </c>
+      <c r="P137">
+        <v>0.4454246461391449</v>
+      </c>
+      <c r="Q137">
+        <v>15073.0537109375</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B138" t="str">
+        <v>10:05:52 ч.</v>
+      </c>
+      <c r="C138" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="D138">
+        <v>239016.2596277693</v>
+      </c>
+      <c r="E138">
+        <v>236.04750061035156</v>
+      </c>
+      <c r="F138">
+        <v>236.0789031982422</v>
+      </c>
+      <c r="G138">
+        <v>238.68898010253906</v>
+      </c>
+      <c r="H138">
+        <v>61.46122741699219</v>
+      </c>
+      <c r="I138">
+        <v>84.59583282470703</v>
+      </c>
+      <c r="J138">
+        <v>78.5202407836914</v>
+      </c>
+      <c r="K138">
+        <v>12686.583984375</v>
+      </c>
+      <c r="L138">
+        <v>16673.93359375</v>
+      </c>
+      <c r="M138">
+        <v>16951.71875</v>
+      </c>
+      <c r="N138">
+        <v>0.8744682669639587</v>
+      </c>
+      <c r="O138">
+        <v>0.8348950743675232</v>
+      </c>
+      <c r="P138">
+        <v>0.8978033661842346</v>
+      </c>
+      <c r="Q138">
+        <v>46014.75</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B139" t="str">
+        <v>10:05:52 ч.</v>
+      </c>
+      <c r="C139" t="str">
+        <v>HOMO UHT</v>
+      </c>
+      <c r="D139">
+        <v>1828.0669753117434</v>
+      </c>
+      <c r="E139">
+        <v>235.48020935058594</v>
+      </c>
+      <c r="F139">
+        <v>236.49623107910156</v>
+      </c>
+      <c r="G139">
+        <v>237.80047607421875</v>
+      </c>
+      <c r="H139">
+        <v>0.24702957272529602</v>
+      </c>
+      <c r="I139">
+        <v>0.11187910288572311</v>
+      </c>
+      <c r="J139">
+        <v>0.21930746734142303</v>
+      </c>
+      <c r="K139">
+        <v>36.2958984375</v>
+      </c>
+      <c r="L139">
+        <v>14.646340370178223</v>
+      </c>
+      <c r="M139">
+        <v>14.819193840026855</v>
+      </c>
+      <c r="N139">
+        <v>0.6239563226699829</v>
+      </c>
+      <c r="O139">
+        <v>0.5535488128662109</v>
+      </c>
+      <c r="P139">
+        <v>0.28415703773498535</v>
+      </c>
+      <c r="Q139">
+        <v>65.76142883300781</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B140" t="str">
+        <v>10:05:52 ч.</v>
+      </c>
+      <c r="C140" t="str">
+        <v>Priem KM</v>
+      </c>
+      <c r="D140">
+        <v>5574.673881582665</v>
+      </c>
+      <c r="E140">
+        <v>235.56222534179688</v>
+      </c>
+      <c r="F140">
+        <v>236.5330352783203</v>
+      </c>
+      <c r="G140">
+        <v>238.04075622558594</v>
+      </c>
+      <c r="H140">
+        <v>40.05534744262695</v>
+      </c>
+      <c r="I140">
+        <v>38.19553756713867</v>
+      </c>
+      <c r="J140">
+        <v>41.98490524291992</v>
+      </c>
+      <c r="K140">
+        <v>3727.2548828125</v>
+      </c>
+      <c r="L140">
+        <v>4078.33544921875</v>
+      </c>
+      <c r="M140">
+        <v>3865.7626953125</v>
+      </c>
+      <c r="N140">
+        <v>0.39502352476119995</v>
+      </c>
+      <c r="O140">
+        <v>0.4770459234714508</v>
+      </c>
+      <c r="P140">
+        <v>0.41199299693107605</v>
+      </c>
+      <c r="Q140">
+        <v>12604.201171875</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B141" t="str">
+        <v>10:05:52 ч.</v>
+      </c>
+      <c r="C141" t="str">
+        <v>Priem UHT</v>
+      </c>
+      <c r="D141">
+        <v>866.4177837402655</v>
+      </c>
+      <c r="E141">
+        <v>235.59054565429688</v>
+      </c>
+      <c r="F141">
+        <v>236.34896850585938</v>
+      </c>
+      <c r="G141">
+        <v>237.9160919189453</v>
+      </c>
+      <c r="H141">
+        <v>0.9161816835403442</v>
+      </c>
+      <c r="I141">
+        <v>0.5081156492233276</v>
+      </c>
+      <c r="J141">
+        <v>0.824709415435791</v>
+      </c>
+      <c r="K141">
+        <v>114.8641586303711</v>
+      </c>
+      <c r="L141">
+        <v>84.51676940917969</v>
+      </c>
+      <c r="M141">
+        <v>59.6165657043457</v>
+      </c>
+      <c r="N141">
+        <v>0.5334383845329285</v>
+      </c>
+      <c r="O141">
+        <v>0.7038540244102478</v>
+      </c>
+      <c r="P141">
+        <v>0.3038809895515442</v>
+      </c>
+      <c r="Q141">
+        <v>258.99749755859375</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B142" t="str">
+        <v>10:07:46 ч.</v>
+      </c>
+      <c r="C142" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D142">
+        <v>139038.85193970645</v>
+      </c>
+      <c r="E142">
+        <v>234.4202423095703</v>
+      </c>
+      <c r="F142">
+        <v>234.07421875</v>
+      </c>
+      <c r="G142">
+        <v>236.30401611328125</v>
+      </c>
+      <c r="H142">
+        <v>1.6000113487243652</v>
+      </c>
+      <c r="I142">
+        <v>1.6304835081100464</v>
+      </c>
+      <c r="J142">
+        <v>1.4644216299057007</v>
+      </c>
+      <c r="K142">
+        <v>268.4554443359375</v>
+      </c>
+      <c r="L142">
+        <v>200.66139221191406</v>
+      </c>
+      <c r="M142">
+        <v>213.86036682128906</v>
+      </c>
+      <c r="N142">
+        <v>0.7181345224380493</v>
+      </c>
+      <c r="O142">
+        <v>0.5237480401992798</v>
+      </c>
+      <c r="P142">
+        <v>0.6184430718421936</v>
+      </c>
+      <c r="Q142">
+        <v>682.406494140625</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B143" t="str">
+        <v>10:07:46 ч.</v>
+      </c>
+      <c r="C143" t="str">
+        <v>Ampak</v>
+      </c>
+      <c r="D143">
+        <v>41468.77509226041</v>
+      </c>
+      <c r="E143">
+        <v>234.240966796875</v>
+      </c>
+      <c r="F143">
+        <v>233.7522735595703</v>
+      </c>
+      <c r="G143">
+        <v>236.0378875732422</v>
+      </c>
+      <c r="H143">
+        <v>32.59639358520508</v>
+      </c>
+      <c r="I143">
+        <v>31.129425048828125</v>
+      </c>
+      <c r="J143">
+        <v>27.009258270263672</v>
+      </c>
+      <c r="K143">
+        <v>6664.2763671875</v>
+      </c>
+      <c r="L143">
+        <v>5656.4033203125</v>
+      </c>
+      <c r="M143">
+        <v>5021.212890625</v>
+      </c>
+      <c r="N143">
+        <v>0.8555071949958801</v>
+      </c>
+      <c r="O143">
+        <v>0.8399644494056702</v>
+      </c>
+      <c r="P143">
+        <v>0.8522481918334961</v>
+      </c>
+      <c r="Q143">
+        <v>16511.4921875</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B144" t="str">
+        <v>10:07:46 ч.</v>
+      </c>
+      <c r="C144" t="str">
+        <v>Ledena Voda</v>
+      </c>
+      <c r="D144">
+        <v>246437.48687132457</v>
+      </c>
+      <c r="E144">
+        <v>236.63165283203125</v>
+      </c>
+      <c r="F144">
+        <v>236.8091583251953</v>
+      </c>
+      <c r="G144">
+        <v>238.39784240722656</v>
+      </c>
+      <c r="H144">
+        <v>0.18328116834163666</v>
+      </c>
+      <c r="I144">
+        <v>0.2521653473377228</v>
+      </c>
+      <c r="J144">
+        <v>0.43402397632598877</v>
+      </c>
+      <c r="K144">
+        <v>33.69425582885742</v>
+      </c>
+      <c r="L144">
+        <v>-14.907113075256348</v>
+      </c>
+      <c r="M144">
+        <v>51.84940719604492</v>
+      </c>
+      <c r="N144">
+        <v>0.7868720293045044</v>
+      </c>
+      <c r="O144">
+        <v>0.24964788556098938</v>
+      </c>
+      <c r="P144">
+        <v>0.5012145638465881</v>
+      </c>
+      <c r="Q144">
+        <v>70.63655090332031</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B145" t="str">
+        <v>10:07:46 ч.</v>
+      </c>
+      <c r="C145" t="str">
+        <v>Hladilnici</v>
+      </c>
+      <c r="D145">
+        <v>181733.44334208718</v>
+      </c>
+      <c r="E145">
+        <v>237.87799072265625</v>
+      </c>
+      <c r="F145">
+        <v>236.2108612060547</v>
+      </c>
+      <c r="G145">
+        <v>236.2318572998047</v>
+      </c>
+      <c r="H145">
+        <v>8.760384559631348</v>
+      </c>
+      <c r="I145">
+        <v>8.866854667663574</v>
+      </c>
+      <c r="J145">
+        <v>12.108942031860352</v>
+      </c>
+      <c r="K145">
+        <v>1766.250244140625</v>
+      </c>
+      <c r="L145">
+        <v>1748.7772216796875</v>
+      </c>
+      <c r="M145">
+        <v>2641.2021484375</v>
+      </c>
+      <c r="N145">
+        <v>0.8474342226982117</v>
+      </c>
+      <c r="O145">
+        <v>0.8349378108978271</v>
+      </c>
+      <c r="P145">
+        <v>0.9231994152069092</v>
+      </c>
+      <c r="Q145">
+        <v>6156.2294921875</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B146" t="str">
+        <v>10:07:46 ч.</v>
+      </c>
+      <c r="C146" t="str">
+        <v>Kompresorno</v>
+      </c>
+      <c r="D146">
+        <v>49909.73538388203</v>
+      </c>
+      <c r="E146">
+        <v>236.27798461914062</v>
+      </c>
+      <c r="F146">
+        <v>234.4562530517578</v>
+      </c>
+      <c r="G146">
+        <v>233.79757690429688</v>
+      </c>
+      <c r="H146">
+        <v>47.07633972167969</v>
+      </c>
+      <c r="I146">
+        <v>40.98766326904297</v>
+      </c>
+      <c r="J146">
+        <v>43.52935791015625</v>
+      </c>
+      <c r="K146">
+        <v>9595.525390625</v>
+      </c>
+      <c r="L146">
+        <v>7772.333984375</v>
+      </c>
+      <c r="M146">
+        <v>7591.5</v>
+      </c>
+      <c r="N146">
+        <v>0.8261484503746033</v>
+      </c>
+      <c r="O146">
+        <v>0.8090413808822632</v>
+      </c>
+      <c r="P146">
+        <v>0.7458528876304626</v>
+      </c>
+      <c r="Q146">
+        <v>24959.359375</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B147" t="str">
+        <v>10:07:46 ч.</v>
+      </c>
+      <c r="C147" t="str">
+        <v>Priemno</v>
+      </c>
+      <c r="D147">
+        <v>59431.26673482882</v>
+      </c>
+      <c r="E147">
+        <v>235.53033447265625</v>
+      </c>
+      <c r="F147">
+        <v>236.14801025390625</v>
+      </c>
+      <c r="G147">
+        <v>237.72854614257812</v>
+      </c>
+      <c r="H147">
+        <v>41.51793670654297</v>
+      </c>
+      <c r="I147">
+        <v>36.309532165527344</v>
+      </c>
+      <c r="J147">
+        <v>38.4262809753418</v>
+      </c>
+      <c r="K147">
+        <v>5313.9541015625</v>
+      </c>
+      <c r="L147">
+        <v>3863.73974609375</v>
+      </c>
+      <c r="M147">
+        <v>3728.0751953125</v>
+      </c>
+      <c r="N147">
+        <v>0.5434194803237915</v>
+      </c>
+      <c r="O147">
+        <v>0.4506121575832367</v>
+      </c>
+      <c r="P147">
+        <v>0.4081079065799713</v>
+      </c>
+      <c r="Q147">
+        <v>12964.5185546875</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B148" t="str">
+        <v>10:07:46 ч.</v>
+      </c>
+      <c r="C148" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="D148">
+        <v>239017.7367868474</v>
+      </c>
+      <c r="E148">
+        <v>235.9672393798828</v>
+      </c>
+      <c r="F148">
+        <v>236.05841064453125</v>
+      </c>
+      <c r="G148">
+        <v>238.51885986328125</v>
+      </c>
+      <c r="H148">
+        <v>72.84121704101562</v>
+      </c>
+      <c r="I148">
+        <v>96.97046661376953</v>
+      </c>
+      <c r="J148">
+        <v>88.14380645751953</v>
+      </c>
+      <c r="K148">
+        <v>15778.60546875</v>
+      </c>
+      <c r="L148">
+        <v>20133.685546875</v>
+      </c>
+      <c r="M148">
+        <v>19606.6953125</v>
+      </c>
+      <c r="N148">
+        <v>0.9179937243461609</v>
+      </c>
+      <c r="O148">
+        <v>0.8562889695167542</v>
+      </c>
+      <c r="P148">
+        <v>0.9077420830726624</v>
+      </c>
+      <c r="Q148">
+        <v>48222.39453125</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B149" t="str">
+        <v>10:07:46 ч.</v>
+      </c>
+      <c r="C149" t="str">
+        <v>HOMO UHT</v>
+      </c>
+      <c r="D149">
+        <v>1828.0690574332384</v>
+      </c>
+      <c r="E149">
+        <v>235.42430114746094</v>
+      </c>
+      <c r="F149">
+        <v>236.3950958251953</v>
+      </c>
+      <c r="G149">
+        <v>237.57473754882812</v>
+      </c>
+      <c r="H149">
+        <v>0.25658783316612244</v>
+      </c>
+      <c r="I149">
+        <v>0.10946732014417648</v>
+      </c>
+      <c r="J149">
+        <v>0.22869843244552612</v>
+      </c>
+      <c r="K149">
+        <v>36.784523010253906</v>
+      </c>
+      <c r="L149">
+        <v>14.105795860290527</v>
+      </c>
+      <c r="M149">
+        <v>14.942697525024414</v>
+      </c>
+      <c r="N149">
+        <v>0.608784556388855</v>
+      </c>
+      <c r="O149">
+        <v>0.545098066329956</v>
+      </c>
+      <c r="P149">
+        <v>0.2750208079814911</v>
+      </c>
+      <c r="Q149">
+        <v>65.83302307128906</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B150" t="str">
+        <v>10:07:46 ч.</v>
+      </c>
+      <c r="C150" t="str">
+        <v>Priem KM</v>
+      </c>
+      <c r="D150">
+        <v>5575.002560837673</v>
+      </c>
+      <c r="E150">
+        <v>235.5012969970703</v>
+      </c>
+      <c r="F150">
+        <v>236.3583984375</v>
+      </c>
+      <c r="G150">
+        <v>237.7665557861328</v>
+      </c>
+      <c r="H150">
+        <v>35.71556854248047</v>
+      </c>
+      <c r="I150">
+        <v>35.24736022949219</v>
+      </c>
+      <c r="J150">
+        <v>38.78123474121094</v>
+      </c>
+      <c r="K150">
+        <v>2565.2099609375</v>
+      </c>
+      <c r="L150">
+        <v>3190.16943359375</v>
+      </c>
+      <c r="M150">
+        <v>2971.54345703125</v>
+      </c>
+      <c r="N150">
+        <v>0.30498048663139343</v>
+      </c>
+      <c r="O150">
+        <v>0.3829270899295807</v>
+      </c>
+      <c r="P150">
+        <v>0.3222624659538269</v>
+      </c>
+      <c r="Q150">
+        <v>8726.9228515625</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B151" t="str">
+        <v>10:07:46 ч.</v>
+      </c>
+      <c r="C151" t="str">
+        <v>Priem UHT</v>
+      </c>
+      <c r="D151">
+        <v>866.4260400147607</v>
+      </c>
+      <c r="E151">
+        <v>235.5994873046875</v>
+      </c>
+      <c r="F151">
+        <v>236.18235778808594</v>
+      </c>
+      <c r="G151">
+        <v>237.7251434326172</v>
+      </c>
+      <c r="H151">
+        <v>0.9274381399154663</v>
+      </c>
+      <c r="I151">
+        <v>0.48298996686935425</v>
+      </c>
+      <c r="J151">
+        <v>0.8515982627868652</v>
+      </c>
+      <c r="K151">
+        <v>118.79798889160156</v>
+      </c>
+      <c r="L151">
+        <v>79.66654205322266</v>
+      </c>
+      <c r="M151">
+        <v>59.603248596191406</v>
+      </c>
+      <c r="N151">
+        <v>0.5436880588531494</v>
+      </c>
+      <c r="O151">
+        <v>0.698377788066864</v>
+      </c>
+      <c r="P151">
+        <v>0.29531827569007874</v>
+      </c>
+      <c r="Q151">
+        <v>258.8445739746094</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B152" t="str">
+        <v>10:09:46 ч.</v>
+      </c>
+      <c r="C152" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D152">
+        <v>139038.87465770615</v>
+      </c>
+      <c r="E152">
+        <v>234.33596801757812</v>
+      </c>
+      <c r="F152">
+        <v>234.11766052246094</v>
+      </c>
+      <c r="G152">
+        <v>236.28158569335938</v>
+      </c>
+      <c r="H152">
+        <v>1.5814902782440186</v>
+      </c>
+      <c r="I152">
+        <v>1.6229403018951416</v>
+      </c>
+      <c r="J152">
+        <v>1.4708837270736694</v>
+      </c>
+      <c r="K152">
+        <v>265.0804138183594</v>
+      </c>
+      <c r="L152">
+        <v>202.046142578125</v>
+      </c>
+      <c r="M152">
+        <v>214.6230010986328</v>
+      </c>
+      <c r="N152">
+        <v>0.7144915461540222</v>
+      </c>
+      <c r="O152">
+        <v>0.5321532487869263</v>
+      </c>
+      <c r="P152">
+        <v>0.6154894828796387</v>
+      </c>
+      <c r="Q152">
+        <v>681.5570068359375</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B153" t="str">
+        <v>10:09:46 ч.</v>
+      </c>
+      <c r="C153" t="str">
+        <v>Ampak</v>
+      </c>
+      <c r="D153">
+        <v>41469.44904075628</v>
+      </c>
+      <c r="E153">
+        <v>234.354248046875</v>
+      </c>
+      <c r="F153">
+        <v>233.98309326171875</v>
+      </c>
+      <c r="G153">
+        <v>236.22413635253906</v>
+      </c>
+      <c r="H153">
+        <v>26.22492027282715</v>
+      </c>
+      <c r="I153">
+        <v>25.168630599975586</v>
+      </c>
+      <c r="J153">
+        <v>18.51403045654297</v>
+      </c>
+      <c r="K153">
+        <v>5561.69140625</v>
+      </c>
+      <c r="L153">
+        <v>5178.9052734375</v>
+      </c>
+      <c r="M153">
+        <v>3544.65869140625</v>
+      </c>
+      <c r="N153">
+        <v>0.8946020603179932</v>
+      </c>
+      <c r="O153">
+        <v>0.8652332425117493</v>
+      </c>
+      <c r="P153">
+        <v>0.8693605661392212</v>
+      </c>
+      <c r="Q153">
+        <v>13580.166015625</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B154" t="str">
+        <v>10:09:46 ч.</v>
+      </c>
+      <c r="C154" t="str">
+        <v>Ledena Voda</v>
+      </c>
+      <c r="D154">
+        <v>246437.4892180964</v>
+      </c>
+      <c r="E154">
+        <v>236.6395721435547</v>
+      </c>
+      <c r="F154">
+        <v>236.68344116210938</v>
+      </c>
+      <c r="G154">
+        <v>238.3091278076172</v>
+      </c>
+      <c r="H154">
+        <v>0.17987188696861267</v>
+      </c>
+      <c r="I154">
+        <v>0.2516337037086487</v>
+      </c>
+      <c r="J154">
+        <v>0.4365887939929962</v>
+      </c>
+      <c r="K154">
+        <v>33.74800109863281</v>
+      </c>
+      <c r="L154">
+        <v>-15.809187889099121</v>
+      </c>
+      <c r="M154">
+        <v>52.3038330078125</v>
+      </c>
+      <c r="N154">
+        <v>0.790748119354248</v>
+      </c>
+      <c r="O154">
+        <v>0.265376478433609</v>
+      </c>
+      <c r="P154">
+        <v>0.5026472210884094</v>
+      </c>
+      <c r="Q154">
+        <v>70.24264526367188</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B155" t="str">
+        <v>10:09:46 ч.</v>
+      </c>
+      <c r="C155" t="str">
+        <v>Hladilnici</v>
+      </c>
+      <c r="D155">
+        <v>181733.66179211845</v>
+      </c>
+      <c r="E155">
+        <v>237.9149169921875</v>
+      </c>
+      <c r="F155">
+        <v>236.2926025390625</v>
+      </c>
+      <c r="G155">
+        <v>236.29171752929688</v>
+      </c>
+      <c r="H155">
+        <v>10.361954689025879</v>
+      </c>
+      <c r="I155">
+        <v>8.860551834106445</v>
+      </c>
+      <c r="J155">
+        <v>10.481780052185059</v>
+      </c>
+      <c r="K155">
+        <v>2114.6611328125</v>
+      </c>
+      <c r="L155">
+        <v>1746.1680908203125</v>
+      </c>
+      <c r="M155">
+        <v>2305.8671875</v>
+      </c>
+      <c r="N155">
+        <v>0.857825517654419</v>
+      </c>
+      <c r="O155">
+        <v>0.8340619206428528</v>
+      </c>
+      <c r="P155">
+        <v>0.931113600730896</v>
+      </c>
+      <c r="Q155">
+        <v>6166.6962890625</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B156" t="str">
+        <v>10:09:46 ч.</v>
+      </c>
+      <c r="C156" t="str">
+        <v>Kompresorno</v>
+      </c>
+      <c r="D156">
+        <v>49910.525377403486</v>
+      </c>
+      <c r="E156">
+        <v>236.4041748046875</v>
+      </c>
+      <c r="F156">
+        <v>234.44497680664062</v>
+      </c>
+      <c r="G156">
+        <v>233.98765563964844</v>
+      </c>
+      <c r="H156">
+        <v>43.40854263305664</v>
+      </c>
+      <c r="I156">
+        <v>38.09847640991211</v>
+      </c>
+      <c r="J156">
+        <v>42.02516555786133</v>
+      </c>
+      <c r="K156">
+        <v>8522.77734375</v>
+      </c>
+      <c r="L156">
+        <v>7077.5615234375</v>
+      </c>
+      <c r="M156">
+        <v>7416.9306640625</v>
+      </c>
+      <c r="N156">
+        <v>0.8046689629554749</v>
+      </c>
+      <c r="O156">
+        <v>0.7924172878265381</v>
+      </c>
+      <c r="P156">
+        <v>0.7545533180236816</v>
+      </c>
+      <c r="Q156">
+        <v>23017.26953125</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B157" t="str">
+        <v>10:09:46 ч.</v>
+      </c>
+      <c r="C157" t="str">
+        <v>Priemno</v>
+      </c>
+      <c r="D157">
+        <v>59431.71146617841</v>
+      </c>
+      <c r="E157">
+        <v>235.4910888671875</v>
+      </c>
+      <c r="F157">
+        <v>236.04736328125</v>
+      </c>
+      <c r="G157">
+        <v>237.72645568847656</v>
+      </c>
+      <c r="H157">
+        <v>41.98965072631836</v>
+      </c>
+      <c r="I157">
+        <v>37.042423248291016</v>
+      </c>
+      <c r="J157">
+        <v>39.568809509277344</v>
+      </c>
+      <c r="K157">
+        <v>5171.74755859375</v>
+      </c>
+      <c r="L157">
+        <v>3844.668701171875</v>
+      </c>
+      <c r="M157">
+        <v>3673.114013671875</v>
+      </c>
+      <c r="N157">
+        <v>0.522693932056427</v>
+      </c>
+      <c r="O157">
+        <v>0.4404057562351227</v>
+      </c>
+      <c r="P157">
+        <v>0.3899399936199188</v>
+      </c>
+      <c r="Q157">
+        <v>12693.3125</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B158" t="str">
+        <v>10:09:46 ч.</v>
+      </c>
+      <c r="C158" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="D158">
+        <v>239019.2689921339</v>
+      </c>
+      <c r="E158">
+        <v>235.8297119140625</v>
+      </c>
+      <c r="F158">
+        <v>235.98764038085938</v>
+      </c>
+      <c r="G158">
+        <v>238.5072021484375</v>
+      </c>
+      <c r="H158">
+        <v>68.87393188476562</v>
+      </c>
+      <c r="I158">
+        <v>92.2104263305664</v>
+      </c>
+      <c r="J158">
+        <v>84.86144256591797</v>
+      </c>
+      <c r="K158">
+        <v>11508.4404296875</v>
+      </c>
+      <c r="L158">
+        <v>16262.248046875</v>
+      </c>
+      <c r="M158">
+        <v>15389.162109375</v>
+      </c>
+      <c r="N158">
+        <v>0.8589008450508118</v>
+      </c>
+      <c r="O158">
+        <v>0.8425077795982361</v>
+      </c>
+      <c r="P158">
+        <v>0.8996776342391968</v>
+      </c>
+      <c r="Q158">
+        <v>43159.8515625</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B159" t="str">
+        <v>10:09:46 ч.</v>
+      </c>
+      <c r="C159" t="str">
+        <v>HOMO UHT</v>
+      </c>
+      <c r="D159">
+        <v>1828.0712517134036</v>
+      </c>
+      <c r="E159">
+        <v>235.4991455078125</v>
+      </c>
+      <c r="F159">
+        <v>236.2744903564453</v>
+      </c>
+      <c r="G159">
+        <v>237.64549255371094</v>
+      </c>
+      <c r="H159">
+        <v>0.2539060413837433</v>
+      </c>
+      <c r="I159">
+        <v>0.1100335419178009</v>
+      </c>
+      <c r="J159">
+        <v>0.22672219574451447</v>
+      </c>
+      <c r="K159">
+        <v>36.73411178588867</v>
+      </c>
+      <c r="L159">
+        <v>14.218984603881836</v>
+      </c>
+      <c r="M159">
+        <v>14.881683349609375</v>
+      </c>
+      <c r="N159">
+        <v>0.6143377423286438</v>
+      </c>
+      <c r="O159">
+        <v>0.5469235777854919</v>
+      </c>
+      <c r="P159">
+        <v>0.2762030363082886</v>
+      </c>
+      <c r="Q159">
+        <v>65.68411254882812</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B160" t="str">
+        <v>10:09:46 ч.</v>
+      </c>
+      <c r="C160" t="str">
+        <v>Priem KM</v>
+      </c>
+      <c r="D160">
+        <v>5575.334192722248</v>
+      </c>
+      <c r="E160">
+        <v>235.47010803222656</v>
+      </c>
+      <c r="F160">
+        <v>236.1797332763672</v>
+      </c>
+      <c r="G160">
+        <v>237.81637573242188</v>
+      </c>
+      <c r="H160">
+        <v>37.84632873535156</v>
+      </c>
+      <c r="I160">
+        <v>36.95769119262695</v>
+      </c>
+      <c r="J160">
+        <v>41.12369155883789</v>
+      </c>
+      <c r="K160">
+        <v>2875.138916015625</v>
+      </c>
+      <c r="L160">
+        <v>3564.572998046875</v>
+      </c>
+      <c r="M160">
+        <v>3447.0439453125</v>
+      </c>
+      <c r="N160">
+        <v>0.3226259648799896</v>
+      </c>
+      <c r="O160">
+        <v>0.40874022245407104</v>
+      </c>
+      <c r="P160">
+        <v>0.35107529163360596</v>
+      </c>
+      <c r="Q160">
+        <v>9885.7724609375</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B161" t="str">
+        <v>10:09:46 ч.</v>
+      </c>
+      <c r="C161" t="str">
+        <v>Priem UHT</v>
+      </c>
+      <c r="D161">
+        <v>866.4346700782572</v>
+      </c>
+      <c r="E161">
+        <v>235.5757293701172</v>
+      </c>
+      <c r="F161">
+        <v>236.0371856689453</v>
+      </c>
+      <c r="G161">
+        <v>237.83978271484375</v>
+      </c>
+      <c r="H161">
+        <v>0.9270001649856567</v>
+      </c>
+      <c r="I161">
+        <v>0.48280489444732666</v>
+      </c>
+      <c r="J161">
+        <v>0.8536068201065063</v>
+      </c>
+      <c r="K161">
+        <v>119.40567779541016</v>
+      </c>
+      <c r="L161">
+        <v>79.3748550415039</v>
+      </c>
+      <c r="M161">
+        <v>60.00950241088867</v>
+      </c>
+      <c r="N161">
+        <v>0.5466350317001343</v>
+      </c>
+      <c r="O161">
+        <v>0.6978422999382019</v>
+      </c>
+      <c r="P161">
+        <v>0.2954161763191223</v>
+      </c>
+      <c r="Q161">
+        <v>258.7900390625</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B162" t="str">
+        <v>10:12:24 ч.</v>
+      </c>
+      <c r="C162" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D162">
+        <v>139038.9063620763</v>
+      </c>
+      <c r="E162">
+        <v>233.9184112548828</v>
+      </c>
+      <c r="F162">
+        <v>234.0709991455078</v>
+      </c>
+      <c r="G162">
+        <v>235.79954528808594</v>
+      </c>
+      <c r="H162">
+        <v>1.5935478210449219</v>
+      </c>
+      <c r="I162">
+        <v>1.6359525918960571</v>
+      </c>
+      <c r="J162">
+        <v>1.4711313247680664</v>
+      </c>
+      <c r="K162">
+        <v>266.3359375</v>
+      </c>
+      <c r="L162">
+        <v>200.6943359375</v>
+      </c>
+      <c r="M162">
+        <v>214.740234375</v>
+      </c>
+      <c r="N162">
+        <v>0.7158357501029968</v>
+      </c>
+      <c r="O162">
+        <v>0.5280730724334717</v>
+      </c>
+      <c r="P162">
+        <v>0.618415892124176</v>
+      </c>
+      <c r="Q162">
+        <v>680.575439453125</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B163" t="str">
+        <v>10:13:07 ч.</v>
+      </c>
+      <c r="C163" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D163">
+        <v>139038.91452775756</v>
+      </c>
+      <c r="E163">
+        <v>233.2443084716797</v>
+      </c>
+      <c r="F163">
+        <v>233.31358337402344</v>
+      </c>
+      <c r="G163">
+        <v>235.51087951660156</v>
+      </c>
+      <c r="H163">
+        <v>1.5912911891937256</v>
+      </c>
+      <c r="I163">
+        <v>1.6258680820465088</v>
+      </c>
+      <c r="J163">
+        <v>1.4644173383712769</v>
+      </c>
+      <c r="K163">
+        <v>266.283203125</v>
+      </c>
+      <c r="L163">
+        <v>200.31027221679688</v>
+      </c>
+      <c r="M163">
+        <v>213.51031494140625</v>
+      </c>
+      <c r="N163">
+        <v>0.7184930443763733</v>
+      </c>
+      <c r="O163">
+        <v>0.5284240245819092</v>
+      </c>
+      <c r="P163">
+        <v>0.618896484375</v>
+      </c>
+      <c r="Q163">
+        <v>680.103759765625</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B164" t="str">
+        <v>10:15:28 ч.</v>
+      </c>
+      <c r="C164" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D164">
+        <v>139038.94110983695</v>
+      </c>
+      <c r="E164">
+        <v>233.40924072265625</v>
+      </c>
+      <c r="F164">
+        <v>233.77662658691406</v>
+      </c>
+      <c r="G164">
+        <v>235.8629150390625</v>
+      </c>
+      <c r="H164">
+        <v>1.592231273651123</v>
+      </c>
+      <c r="I164">
+        <v>1.6274354457855225</v>
+      </c>
+      <c r="J164">
+        <v>1.4654366970062256</v>
+      </c>
+      <c r="K164">
+        <v>266.2231140136719</v>
+      </c>
+      <c r="L164">
+        <v>201.3376007080078</v>
+      </c>
+      <c r="M164">
+        <v>212.95350646972656</v>
+      </c>
+      <c r="N164">
+        <v>0.7170530557632446</v>
+      </c>
+      <c r="O164">
+        <v>0.5287478566169739</v>
+      </c>
+      <c r="P164">
+        <v>0.6159896850585938</v>
+      </c>
+      <c r="Q164">
+        <v>680.5142211914062</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B165" t="str">
+        <v>10:16:18 ч.</v>
+      </c>
+      <c r="C165" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D165">
+        <v>139038.94873200206</v>
+      </c>
+      <c r="E165">
+        <v>233.57957458496094</v>
+      </c>
+      <c r="F165">
+        <v>233.86566162109375</v>
+      </c>
+      <c r="G165">
+        <v>235.97010803222656</v>
+      </c>
+      <c r="H165">
+        <v>1.597031593322754</v>
+      </c>
+      <c r="I165">
+        <v>1.626981496810913</v>
+      </c>
+      <c r="J165">
+        <v>1.4634515047073364</v>
+      </c>
+      <c r="K165">
+        <v>267.8522033691406</v>
+      </c>
+      <c r="L165">
+        <v>200.3492431640625</v>
+      </c>
+      <c r="M165">
+        <v>211.87673950195312</v>
+      </c>
+      <c r="N165">
+        <v>0.7180991172790527</v>
+      </c>
+      <c r="O165">
+        <v>0.5264173746109009</v>
+      </c>
+      <c r="P165">
+        <v>0.6158956289291382</v>
+      </c>
+      <c r="Q165">
+        <v>680.33544921875</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B166" t="str">
+        <v>10:16:18 ч.</v>
+      </c>
+      <c r="C166" t="str">
+        <v>Ampak</v>
+      </c>
+      <c r="D166">
+        <v>41471.6432372685</v>
+      </c>
+      <c r="E166">
+        <v>233.4939727783203</v>
+      </c>
+      <c r="F166">
+        <v>233.57516479492188</v>
+      </c>
+      <c r="G166">
+        <v>235.9759063720703</v>
+      </c>
+      <c r="H166">
+        <v>29.422210693359375</v>
+      </c>
+      <c r="I166">
+        <v>29.369155883789062</v>
+      </c>
+      <c r="J166">
+        <v>22.8621768951416</v>
+      </c>
+      <c r="K166">
+        <v>5973.927734375</v>
+      </c>
+      <c r="L166">
+        <v>5842.45361328125</v>
+      </c>
+      <c r="M166">
+        <v>4507.55810546875</v>
+      </c>
+      <c r="N166">
+        <v>0.8919548988342285</v>
+      </c>
+      <c r="O166">
+        <v>0.837527334690094</v>
+      </c>
+      <c r="P166">
+        <v>0.8618908524513245</v>
+      </c>
+      <c r="Q166">
+        <v>16107.57421875</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B167" t="str">
+        <v>10:16:18 ч.</v>
+      </c>
+      <c r="C167" t="str">
+        <v>Ledena Voda</v>
+      </c>
+      <c r="D167">
+        <v>246437.75887710074</v>
+      </c>
+      <c r="E167">
+        <v>236.15293884277344</v>
+      </c>
+      <c r="F167">
+        <v>236.32449340820312</v>
+      </c>
+      <c r="G167">
+        <v>237.91795349121094</v>
+      </c>
+      <c r="H167">
+        <v>6.954192161560059</v>
+      </c>
+      <c r="I167">
+        <v>8.027462005615234</v>
+      </c>
+      <c r="J167">
+        <v>6.862682819366455</v>
+      </c>
+      <c r="K167">
+        <v>1138.18310546875</v>
+      </c>
+      <c r="L167">
+        <v>1437.2991943359375</v>
+      </c>
+      <c r="M167">
+        <v>1165.8040771484375</v>
+      </c>
+      <c r="N167">
+        <v>0.6926103830337524</v>
+      </c>
+      <c r="O167">
+        <v>0.7579642534255981</v>
+      </c>
+      <c r="P167">
+        <v>0.7138960957527161</v>
+      </c>
+      <c r="Q167">
+        <v>3741.286376953125</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B168" t="str">
+        <v>10:16:18 ч.</v>
+      </c>
+      <c r="C168" t="str">
+        <v>Hladilnici</v>
+      </c>
+      <c r="D168">
+        <v>181736.34021316012</v>
+      </c>
+      <c r="E168">
+        <v>236.9237823486328</v>
+      </c>
+      <c r="F168">
+        <v>235.42295837402344</v>
+      </c>
+      <c r="G168">
+        <v>235.43060302734375</v>
+      </c>
+      <c r="H168">
+        <v>72.1514663696289</v>
+      </c>
+      <c r="I168">
+        <v>65.73540496826172</v>
+      </c>
+      <c r="J168">
+        <v>68.43484497070312</v>
+      </c>
+      <c r="K168">
+        <v>13603.205078125</v>
+      </c>
+      <c r="L168">
+        <v>11931.603515625</v>
+      </c>
+      <c r="M168">
+        <v>13162.4375</v>
+      </c>
+      <c r="N168">
+        <v>0.7958451509475708</v>
+      </c>
+      <c r="O168">
+        <v>0.7709059119224548</v>
+      </c>
+      <c r="P168">
+        <v>0.8165121674537659</v>
+      </c>
+      <c r="Q168">
+        <v>38697.24609375</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B169" t="str">
+        <v>10:16:18 ч.</v>
+      </c>
+      <c r="C169" t="str">
+        <v>Kompresorno</v>
+      </c>
+      <c r="D169">
+        <v>49913.11635633038</v>
+      </c>
+      <c r="E169">
+        <v>236.036865234375</v>
+      </c>
+      <c r="F169">
+        <v>233.62484741210938</v>
+      </c>
+      <c r="G169">
+        <v>233.40478515625</v>
+      </c>
+      <c r="H169">
+        <v>47.42576599121094</v>
+      </c>
+      <c r="I169">
+        <v>38.610233306884766</v>
+      </c>
+      <c r="J169">
+        <v>41.94444274902344</v>
+      </c>
+      <c r="K169">
+        <v>9242.611328125</v>
+      </c>
+      <c r="L169">
+        <v>7254.80419921875</v>
+      </c>
+      <c r="M169">
+        <v>7217.8876953125</v>
+      </c>
+      <c r="N169">
+        <v>0.8266968727111816</v>
+      </c>
+      <c r="O169">
+        <v>0.8068402409553528</v>
+      </c>
+      <c r="P169">
+        <v>0.7374032139778137</v>
+      </c>
+      <c r="Q169">
+        <v>23725.685546875</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B170" t="str">
+        <v>10:16:18 ч.</v>
+      </c>
+      <c r="C170" t="str">
+        <v>Priemno</v>
+      </c>
+      <c r="D170">
+        <v>59433.24272701978</v>
+      </c>
+      <c r="E170">
+        <v>235.06935119628906</v>
+      </c>
+      <c r="F170">
+        <v>235.82254028320312</v>
+      </c>
+      <c r="G170">
+        <v>237.39805603027344</v>
+      </c>
+      <c r="H170">
+        <v>44.30183792114258</v>
+      </c>
+      <c r="I170">
+        <v>37.56626510620117</v>
+      </c>
+      <c r="J170">
+        <v>39.81857681274414</v>
+      </c>
+      <c r="K170">
+        <v>5732.3798828125</v>
+      </c>
+      <c r="L170">
+        <v>4048.6943359375</v>
+      </c>
+      <c r="M170">
+        <v>3798.21435546875</v>
+      </c>
+      <c r="N170">
+        <v>0.5504491329193115</v>
+      </c>
+      <c r="O170">
+        <v>0.4570162296295166</v>
+      </c>
+      <c r="P170">
+        <v>0.40180614590644836</v>
+      </c>
+      <c r="Q170">
+        <v>13579.2890625</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B171" t="str">
+        <v>10:16:18 ч.</v>
+      </c>
+      <c r="C171" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="D171">
+        <v>239025.5916478937</v>
+      </c>
+      <c r="E171">
+        <v>235.50486755371094</v>
+      </c>
+      <c r="F171">
+        <v>235.61520385742188</v>
+      </c>
+      <c r="G171">
+        <v>238.13792419433594</v>
+      </c>
+      <c r="H171">
+        <v>108.91168975830078</v>
+      </c>
+      <c r="I171">
+        <v>127.32691955566406</v>
+      </c>
+      <c r="J171">
+        <v>123.61947631835938</v>
+      </c>
+      <c r="K171">
+        <v>22608.681640625</v>
+      </c>
+      <c r="L171">
+        <v>25526.5390625</v>
+      </c>
+      <c r="M171">
+        <v>26446.234375</v>
+      </c>
+      <c r="N171">
+        <v>0.8814563751220703</v>
+      </c>
+      <c r="O171">
+        <v>0.8522439002990723</v>
+      </c>
+      <c r="P171">
+        <v>0.9021543860435486</v>
+      </c>
+      <c r="Q171">
+        <v>75372.7734375</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B172" t="str">
+        <v>10:16:18 ч.</v>
+      </c>
+      <c r="C172" t="str">
+        <v>HOMO UHT</v>
+      </c>
+      <c r="D172">
+        <v>1828.0783656193123</v>
+      </c>
+      <c r="E172">
+        <v>234.9899139404297</v>
+      </c>
+      <c r="F172">
+        <v>235.89285278320312</v>
+      </c>
+      <c r="G172">
+        <v>237.1737060546875</v>
+      </c>
+      <c r="H172">
+        <v>0.25214165449142456</v>
+      </c>
+      <c r="I172">
+        <v>0.12093327939510345</v>
+      </c>
+      <c r="J172">
+        <v>0.22853901982307434</v>
+      </c>
+      <c r="K172">
+        <v>35.21328353881836</v>
+      </c>
+      <c r="L172">
+        <v>15.61124324798584</v>
+      </c>
+      <c r="M172">
+        <v>15.393515586853027</v>
+      </c>
+      <c r="N172">
+        <v>0.5943095088005066</v>
+      </c>
+      <c r="O172">
+        <v>0.547238826751709</v>
+      </c>
+      <c r="P172">
+        <v>0.2839951515197754</v>
+      </c>
+      <c r="Q172">
+        <v>66.2180404663086</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B173" t="str">
+        <v>10:16:18 ч.</v>
+      </c>
+      <c r="C173" t="str">
+        <v>Priem KM</v>
+      </c>
+      <c r="D173">
+        <v>5576.478226097153</v>
+      </c>
+      <c r="E173">
+        <v>234.98863220214844</v>
+      </c>
+      <c r="F173">
+        <v>235.8878173828125</v>
+      </c>
+      <c r="G173">
+        <v>237.3472442626953</v>
+      </c>
+      <c r="H173">
+        <v>39.772850036621094</v>
+      </c>
+      <c r="I173">
+        <v>37.39226531982422</v>
+      </c>
+      <c r="J173">
+        <v>41.21622085571289</v>
+      </c>
+      <c r="K173">
+        <v>3438.820556640625</v>
+      </c>
+      <c r="L173">
+        <v>3743.72509765625</v>
+      </c>
+      <c r="M173">
+        <v>3567.16162109375</v>
+      </c>
+      <c r="N173">
+        <v>0.3679390847682953</v>
+      </c>
+      <c r="O173">
+        <v>0.4244403541088104</v>
+      </c>
+      <c r="P173">
+        <v>0.3646451234817505</v>
+      </c>
+      <c r="Q173">
+        <v>10749.70703125</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B174" t="str">
+        <v>10:16:18 ч.</v>
+      </c>
+      <c r="C174" t="str">
+        <v>Priem UHT</v>
+      </c>
+      <c r="D174">
+        <v>866.4628253136856</v>
+      </c>
+      <c r="E174">
+        <v>235.1066436767578</v>
+      </c>
+      <c r="F174">
+        <v>235.78005981445312</v>
+      </c>
+      <c r="G174">
+        <v>237.32534790039062</v>
+      </c>
+      <c r="H174">
+        <v>0.9132435321807861</v>
+      </c>
+      <c r="I174">
+        <v>0.5132526755332947</v>
+      </c>
+      <c r="J174">
+        <v>0.8215022087097168</v>
+      </c>
+      <c r="K174">
+        <v>113.85385131835938</v>
+      </c>
+      <c r="L174">
+        <v>85.0272216796875</v>
+      </c>
+      <c r="M174">
+        <v>59.353668212890625</v>
+      </c>
+      <c r="N174">
+        <v>0.5302689671516418</v>
+      </c>
+      <c r="O174">
+        <v>0.7026186585426331</v>
+      </c>
+      <c r="P174">
+        <v>0.3046988546848297</v>
+      </c>
+      <c r="Q174">
+        <v>258.3858947753906</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B175" t="str">
+        <v>10:22:54 ч.</v>
+      </c>
+      <c r="C175" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D175">
+        <v>139039.0242592375</v>
+      </c>
+      <c r="E175">
+        <v>234.25209045410156</v>
+      </c>
+      <c r="F175">
+        <v>234.22598266601562</v>
+      </c>
+      <c r="G175">
+        <v>236.50875854492188</v>
+      </c>
+      <c r="H175">
+        <v>1.5967365503311157</v>
+      </c>
+      <c r="I175">
+        <v>1.630573034286499</v>
+      </c>
+      <c r="J175">
+        <v>1.4553890228271484</v>
+      </c>
+      <c r="K175">
+        <v>269.30755615234375</v>
+      </c>
+      <c r="L175">
+        <v>201.08444213867188</v>
+      </c>
+      <c r="M175">
+        <v>211.6575469970703</v>
+      </c>
+      <c r="N175">
+        <v>0.7200155854225159</v>
+      </c>
+      <c r="O175">
+        <v>0.5267025232315063</v>
+      </c>
+      <c r="P175">
+        <v>0.6159418225288391</v>
+      </c>
+      <c r="Q175">
+        <v>681.951416015625</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B176" t="str">
+        <v>10:22:54 ч.</v>
+      </c>
+      <c r="C176" t="str">
+        <v>Ampak</v>
+      </c>
+      <c r="D176">
+        <v>41473.92432848292</v>
+      </c>
+      <c r="E176">
+        <v>234.19619750976562</v>
+      </c>
+      <c r="F176">
+        <v>233.9932098388672</v>
+      </c>
+      <c r="G176">
+        <v>236.48936462402344</v>
+      </c>
+      <c r="H176">
+        <v>30.81443977355957</v>
+      </c>
+      <c r="I176">
+        <v>30.318397521972656</v>
+      </c>
+      <c r="J176">
+        <v>22.33641815185547</v>
+      </c>
+      <c r="K176">
+        <v>6472.74169921875</v>
+      </c>
+      <c r="L176">
+        <v>6268.96484375</v>
+      </c>
+      <c r="M176">
+        <v>4136.37109375</v>
+      </c>
+      <c r="N176">
+        <v>0.8694884181022644</v>
+      </c>
+      <c r="O176">
+        <v>0.8904913067817688</v>
+      </c>
+      <c r="P176">
+        <v>0.8426569700241089</v>
+      </c>
+      <c r="Q176">
+        <v>16260.7109375</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B177" t="str">
+        <v>10:22:54 ч.</v>
+      </c>
+      <c r="C177" t="str">
+        <v>Ledena Voda</v>
+      </c>
+      <c r="D177">
+        <v>246438.08419086115</v>
+      </c>
+      <c r="E177">
+        <v>236.5606231689453</v>
+      </c>
+      <c r="F177">
+        <v>236.81832885742188</v>
+      </c>
+      <c r="G177">
+        <v>238.47384643554688</v>
+      </c>
+      <c r="H177">
+        <v>5.456319332122803</v>
+      </c>
+      <c r="I177">
+        <v>6.202317237854004</v>
+      </c>
+      <c r="J177">
+        <v>4.018193244934082</v>
+      </c>
+      <c r="K177">
+        <v>1237.8038330078125</v>
+      </c>
+      <c r="L177">
+        <v>1462.928466796875</v>
+      </c>
+      <c r="M177">
+        <v>956.259033203125</v>
+      </c>
+      <c r="N177">
+        <v>0.9588804244995117</v>
+      </c>
+      <c r="O177">
+        <v>0.9960519671440125</v>
+      </c>
+      <c r="P177">
+        <v>0.9979410171508789</v>
+      </c>
+      <c r="Q177">
+        <v>3653.870849609375</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B178" t="str">
+        <v>10:22:54 ч.</v>
+      </c>
+      <c r="C178" t="str">
+        <v>Hladilnici</v>
+      </c>
+      <c r="D178">
+        <v>181738.78724336156</v>
+      </c>
+      <c r="E178">
+        <v>237.72567749023438</v>
+      </c>
+      <c r="F178">
+        <v>235.93853759765625</v>
+      </c>
+      <c r="G178">
+        <v>236.0908660888672</v>
+      </c>
+      <c r="H178">
+        <v>28.571727752685547</v>
+      </c>
+      <c r="I178">
+        <v>27.92185401916504</v>
+      </c>
+      <c r="J178">
+        <v>30.270366668701172</v>
+      </c>
+      <c r="K178">
+        <v>5401.146484375</v>
+      </c>
+      <c r="L178">
+        <v>5203.60107421875</v>
+      </c>
+      <c r="M178">
+        <v>6043.24072265625</v>
+      </c>
+      <c r="N178">
+        <v>0.7953523397445679</v>
+      </c>
+      <c r="O178">
+        <v>0.790048360824585</v>
+      </c>
+      <c r="P178">
+        <v>0.8457584977149963</v>
+      </c>
+      <c r="Q178">
+        <v>16647.98828125</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B179" t="str">
+        <v>10:22:54 ч.</v>
+      </c>
+      <c r="C179" t="str">
+        <v>Kompresorno</v>
+      </c>
+      <c r="D179">
+        <v>49915.80441297029</v>
+      </c>
+      <c r="E179">
+        <v>236.51133728027344</v>
+      </c>
+      <c r="F179">
+        <v>233.9619598388672</v>
+      </c>
+      <c r="G179">
+        <v>233.60641479492188</v>
+      </c>
+      <c r="H179">
+        <v>45.81780242919922</v>
+      </c>
+      <c r="I179">
+        <v>39.274452209472656</v>
+      </c>
+      <c r="J179">
+        <v>42.629600524902344</v>
+      </c>
+      <c r="K179">
+        <v>8793.291015625</v>
+      </c>
+      <c r="L179">
+        <v>7335.4990234375</v>
+      </c>
+      <c r="M179">
+        <v>7538.2021484375</v>
+      </c>
+      <c r="N179">
+        <v>0.8110056519508362</v>
+      </c>
+      <c r="O179">
+        <v>0.7983149886131287</v>
+      </c>
+      <c r="P179">
+        <v>0.7569579482078552</v>
+      </c>
+      <c r="Q179">
+        <v>23666.9921875</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B180" t="str">
+        <v>10:22:54 ч.</v>
+      </c>
+      <c r="C180" t="str">
+        <v>Priemno</v>
+      </c>
+      <c r="D180">
+        <v>59434.85980461466</v>
+      </c>
+      <c r="E180">
+        <v>235.42201232910156</v>
+      </c>
+      <c r="F180">
+        <v>236.17431640625</v>
+      </c>
+      <c r="G180">
+        <v>237.7490997314453</v>
+      </c>
+      <c r="H180">
+        <v>46.46643829345703</v>
+      </c>
+      <c r="I180">
+        <v>39.07941818237305</v>
+      </c>
+      <c r="J180">
+        <v>42.82606887817383</v>
+      </c>
+      <c r="K180">
+        <v>6347.78759765625</v>
+      </c>
+      <c r="L180">
+        <v>4555.3525390625</v>
+      </c>
+      <c r="M180">
+        <v>4777.19384765625</v>
+      </c>
+      <c r="N180">
+        <v>0.5802875757217407</v>
+      </c>
+      <c r="O180">
+        <v>0.49358057975769043</v>
+      </c>
+      <c r="P180">
+        <v>0.46920308470726013</v>
+      </c>
+      <c r="Q180">
+        <v>15680.333984375</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B181" t="str">
+        <v>10:22:54 ч.</v>
+      </c>
+      <c r="C181" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="D181">
+        <v>239031.95911920388</v>
+      </c>
+      <c r="E181">
+        <v>235.87879943847656</v>
+      </c>
+      <c r="F181">
+        <v>235.88465881347656</v>
+      </c>
+      <c r="G181">
+        <v>238.4943389892578</v>
+      </c>
+      <c r="H181">
+        <v>86.54972076416016</v>
+      </c>
+      <c r="I181">
+        <v>104.48892974853516</v>
+      </c>
+      <c r="J181">
+        <v>102.38387298583984</v>
+      </c>
+      <c r="K181">
+        <v>18730.20703125</v>
+      </c>
+      <c r="L181">
+        <v>21343.765625</v>
+      </c>
+      <c r="M181">
+        <v>22383.658203125</v>
+      </c>
+      <c r="N181">
+        <v>0.9174618124961853</v>
+      </c>
+      <c r="O181">
+        <v>0.8704409003257751</v>
+      </c>
+      <c r="P181">
+        <v>0.9185888767242432</v>
+      </c>
+      <c r="Q181">
+        <v>63752.94140625</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B182" t="str">
+        <v>10:22:54 ч.</v>
+      </c>
+      <c r="C182" t="str">
+        <v>HOMO UHT</v>
+      </c>
+      <c r="D182">
+        <v>1828.0855897450683</v>
+      </c>
+      <c r="E182">
+        <v>235.35513305664062</v>
+      </c>
+      <c r="F182">
+        <v>236.28167724609375</v>
+      </c>
+      <c r="G182">
+        <v>237.5709686279297</v>
+      </c>
+      <c r="H182">
+        <v>0.2566913962364197</v>
+      </c>
+      <c r="I182">
+        <v>0.11107921600341797</v>
+      </c>
+      <c r="J182">
+        <v>0.23181721568107605</v>
+      </c>
+      <c r="K182">
+        <v>36.724430084228516</v>
+      </c>
+      <c r="L182">
+        <v>14.486054420471191</v>
+      </c>
+      <c r="M182">
+        <v>15.097098350524902</v>
+      </c>
+      <c r="N182">
+        <v>0.6078830361366272</v>
+      </c>
+      <c r="O182">
+        <v>0.5523841977119446</v>
+      </c>
+      <c r="P182">
+        <v>0.2727678120136261</v>
+      </c>
+      <c r="Q182">
+        <v>65.653564453125</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B183" t="str">
+        <v>10:22:54 ч.</v>
+      </c>
+      <c r="C183" t="str">
+        <v>Priem KM</v>
+      </c>
+      <c r="D183">
+        <v>5577.676081404852</v>
+      </c>
+      <c r="E183">
+        <v>235.38633728027344</v>
+      </c>
+      <c r="F183">
+        <v>236.3342742919922</v>
+      </c>
+      <c r="G183">
+        <v>237.76255798339844</v>
+      </c>
+      <c r="H183">
+        <v>39.85047912597656</v>
+      </c>
+      <c r="I183">
+        <v>37.594444274902344</v>
+      </c>
+      <c r="J183">
+        <v>41.190494537353516</v>
+      </c>
+      <c r="K183">
+        <v>3510.474853515625</v>
+      </c>
+      <c r="L183">
+        <v>3783.44677734375</v>
+      </c>
+      <c r="M183">
+        <v>3586.8681640625</v>
+      </c>
+      <c r="N183">
+        <v>0.37418708205223083</v>
+      </c>
+      <c r="O183">
+        <v>0.4257546067237854</v>
+      </c>
+      <c r="P183">
+        <v>0.3662477135658264</v>
+      </c>
+      <c r="Q183">
+        <v>10880.7900390625</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B184" t="str">
+        <v>10:22:54 ч.</v>
+      </c>
+      <c r="C184" t="str">
+        <v>Priem UHT</v>
+      </c>
+      <c r="D184">
+        <v>866.5099585890044</v>
+      </c>
+      <c r="E184">
+        <v>235.43679809570312</v>
+      </c>
+      <c r="F184">
+        <v>236.15199279785156</v>
+      </c>
+      <c r="G184">
+        <v>237.64144897460938</v>
+      </c>
+      <c r="H184">
+        <v>0.9098092317581177</v>
+      </c>
+      <c r="I184">
+        <v>0.49625125527381897</v>
+      </c>
+      <c r="J184">
+        <v>1.9394457340240479</v>
+      </c>
+      <c r="K184">
+        <v>115.78582763671875</v>
+      </c>
+      <c r="L184">
+        <v>86.02084350585938</v>
+      </c>
+      <c r="M184">
+        <v>425.4066467285156</v>
+      </c>
+      <c r="N184">
+        <v>0.5397743582725525</v>
+      </c>
+      <c r="O184">
+        <v>0.7341309189796448</v>
+      </c>
+      <c r="P184">
+        <v>0.9219455122947693</v>
+      </c>
+      <c r="Q184">
+        <v>627.3309936523438</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B185" t="str">
+        <v>10:24:54 ч.</v>
+      </c>
+      <c r="C185" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D185">
+        <v>139039.04695992946</v>
+      </c>
+      <c r="E185">
+        <v>234.14816284179688</v>
+      </c>
+      <c r="F185">
+        <v>234.24647521972656</v>
+      </c>
+      <c r="G185">
+        <v>236.22409057617188</v>
+      </c>
+      <c r="H185">
+        <v>1.6003913879394531</v>
+      </c>
+      <c r="I185">
+        <v>1.6339069604873657</v>
+      </c>
+      <c r="J185">
+        <v>1.4529505968093872</v>
+      </c>
+      <c r="K185">
+        <v>270.4565734863281</v>
+      </c>
+      <c r="L185">
+        <v>200.79225158691406</v>
+      </c>
+      <c r="M185">
+        <v>211.59132385253906</v>
+      </c>
+      <c r="N185">
+        <v>0.7223880887031555</v>
+      </c>
+      <c r="O185">
+        <v>0.5238502025604248</v>
+      </c>
+      <c r="P185">
+        <v>0.6159518957138062</v>
+      </c>
+      <c r="Q185">
+        <v>681.333740234375</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B186" t="str">
+        <v>10:24:54 ч.</v>
+      </c>
+      <c r="C186" t="str">
+        <v>Ampak</v>
+      </c>
+      <c r="D186">
+        <v>41474.604911879236</v>
+      </c>
+      <c r="E186">
+        <v>234.13595581054688</v>
+      </c>
+      <c r="F186">
+        <v>233.95632934570312</v>
+      </c>
+      <c r="G186">
+        <v>236.2974853515625</v>
+      </c>
+      <c r="H186">
+        <v>31.603759765625</v>
+      </c>
+      <c r="I186">
+        <v>28.717723846435547</v>
+      </c>
+      <c r="J186">
+        <v>21.248838424682617</v>
+      </c>
+      <c r="K186">
+        <v>6547.4794921875</v>
+      </c>
+      <c r="L186">
+        <v>5413.75439453125</v>
+      </c>
+      <c r="M186">
+        <v>4585.767578125</v>
+      </c>
+      <c r="N186">
+        <v>0.8501692414283752</v>
+      </c>
+      <c r="O186">
+        <v>0.8373067378997803</v>
+      </c>
+      <c r="P186">
+        <v>0.8399859070777893</v>
+      </c>
+      <c r="Q186">
+        <v>15578.5302734375</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B187" t="str">
+        <v>10:24:54 ч.</v>
+      </c>
+      <c r="C187" t="str">
+        <v>Ledena Voda</v>
+      </c>
+      <c r="D187">
+        <v>246438.20556742913</v>
+      </c>
+      <c r="E187">
+        <v>236.54782104492188</v>
+      </c>
+      <c r="F187">
+        <v>236.87875366210938</v>
+      </c>
+      <c r="G187">
+        <v>238.24339294433594</v>
+      </c>
+      <c r="H187">
+        <v>5.414567470550537</v>
+      </c>
+      <c r="I187">
+        <v>6.180356979370117</v>
+      </c>
+      <c r="J187">
+        <v>4.002279281616211</v>
+      </c>
+      <c r="K187">
+        <v>1227.626953125</v>
+      </c>
+      <c r="L187">
+        <v>1458.37255859375</v>
+      </c>
+      <c r="M187">
+        <v>951.0567626953125</v>
+      </c>
+      <c r="N187">
+        <v>0.9585199952125549</v>
+      </c>
+      <c r="O187">
+        <v>0.9962196946144104</v>
+      </c>
+      <c r="P187">
+        <v>0.9978104829788208</v>
+      </c>
+      <c r="Q187">
+        <v>3637.7412109375</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B188" t="str">
+        <v>10:24:54 ч.</v>
+      </c>
+      <c r="C188" t="str">
+        <v>Hladilnici</v>
+      </c>
+      <c r="D188">
+        <v>181739.33449061928</v>
+      </c>
+      <c r="E188">
+        <v>237.645751953125</v>
+      </c>
+      <c r="F188">
+        <v>236.0122833251953</v>
+      </c>
+      <c r="G188">
+        <v>236.1856689453125</v>
+      </c>
+      <c r="H188">
+        <v>26.477998733520508</v>
+      </c>
+      <c r="I188">
+        <v>23.32110023498535</v>
+      </c>
+      <c r="J188">
+        <v>26.217117309570312</v>
+      </c>
+      <c r="K188">
+        <v>4668.013671875</v>
+      </c>
+      <c r="L188">
+        <v>3812.627197265625</v>
+      </c>
+      <c r="M188">
+        <v>4952.11865234375</v>
+      </c>
+      <c r="N188">
+        <v>0.7369813323020935</v>
+      </c>
+      <c r="O188">
+        <v>0.7028473615646362</v>
+      </c>
+      <c r="P188">
+        <v>0.7998161911964417</v>
+      </c>
+      <c r="Q188">
+        <v>13432.759765625</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B189" t="str">
+        <v>10:24:54 ч.</v>
+      </c>
+      <c r="C189" t="str">
+        <v>Kompresorno</v>
+      </c>
+      <c r="D189">
+        <v>49916.6142408564</v>
+      </c>
+      <c r="E189">
+        <v>235.96127319335938</v>
+      </c>
+      <c r="F189">
+        <v>233.71998596191406</v>
+      </c>
+      <c r="G189">
+        <v>233.4184112548828</v>
+      </c>
+      <c r="H189">
+        <v>48.03102111816406</v>
+      </c>
+      <c r="I189">
+        <v>40.3111457824707</v>
+      </c>
+      <c r="J189">
+        <v>42.72304916381836</v>
+      </c>
+      <c r="K189">
+        <v>9353.671875</v>
+      </c>
+      <c r="L189">
+        <v>7636.068359375</v>
+      </c>
+      <c r="M189">
+        <v>7491.3974609375</v>
+      </c>
+      <c r="N189">
+        <v>0.8252677917480469</v>
+      </c>
+      <c r="O189">
+        <v>0.8104921579360962</v>
+      </c>
+      <c r="P189">
+        <v>0.7512171864509583</v>
+      </c>
+      <c r="Q189">
+        <v>24481.13671875</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B190" t="str">
+        <v>10:24:54 ч.</v>
+      </c>
+      <c r="C190" t="str">
+        <v>Priemno</v>
+      </c>
+      <c r="D190">
+        <v>59435.396559048764</v>
+      </c>
+      <c r="E190">
+        <v>235.53794860839844</v>
+      </c>
+      <c r="F190">
+        <v>236.34664916992188</v>
+      </c>
+      <c r="G190">
+        <v>237.76499938964844</v>
+      </c>
+      <c r="H190">
+        <v>48.50844955444336</v>
+      </c>
+      <c r="I190">
+        <v>42.37403106689453</v>
+      </c>
+      <c r="J190">
+        <v>44.750980377197266</v>
+      </c>
+      <c r="K190">
+        <v>7057.72412109375</v>
+      </c>
+      <c r="L190">
+        <v>5545.740234375</v>
+      </c>
+      <c r="M190">
+        <v>5538.12841796875</v>
+      </c>
+      <c r="N190">
+        <v>0.6177124977111816</v>
+      </c>
+      <c r="O190">
+        <v>0.5537456274032593</v>
+      </c>
+      <c r="P190">
+        <v>0.5204901695251465</v>
+      </c>
+      <c r="Q190">
+        <v>18141.591796875</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B191" t="str">
+        <v>10:24:54 ч.</v>
+      </c>
+      <c r="C191" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="D191">
+        <v>239033.7550774277</v>
+      </c>
+      <c r="E191">
+        <v>236.22735595703125</v>
+      </c>
+      <c r="F191">
+        <v>236.19070434570312</v>
+      </c>
+      <c r="G191">
+        <v>238.65664672851562</v>
+      </c>
+      <c r="H191">
+        <v>67.81549072265625</v>
+      </c>
+      <c r="I191">
+        <v>82.87037658691406</v>
+      </c>
+      <c r="J191">
+        <v>83.5685043334961</v>
+      </c>
+      <c r="K191">
+        <v>14158.919921875</v>
+      </c>
+      <c r="L191">
+        <v>16205.4306640625</v>
+      </c>
+      <c r="M191">
+        <v>17391.31640625</v>
+      </c>
+      <c r="N191">
+        <v>0.8850753903388977</v>
+      </c>
+      <c r="O191">
+        <v>0.8322169780731201</v>
+      </c>
+      <c r="P191">
+        <v>0.8905043005943298</v>
+      </c>
+      <c r="Q191">
+        <v>47741.88671875</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B192" t="str">
+        <v>10:24:54 ч.</v>
+      </c>
+      <c r="C192" t="str">
+        <v>HOMO UHT</v>
+      </c>
+      <c r="D192">
+        <v>1828.087768013257</v>
+      </c>
+      <c r="E192">
+        <v>235.60092163085938</v>
+      </c>
+      <c r="F192">
+        <v>236.55612182617188</v>
+      </c>
+      <c r="G192">
+        <v>237.73052978515625</v>
+      </c>
+      <c r="H192">
+        <v>0.22254806756973267</v>
+      </c>
+      <c r="I192">
+        <v>0.12238364666700363</v>
+      </c>
+      <c r="J192">
+        <v>0.19532816112041473</v>
+      </c>
+      <c r="K192">
+        <v>34.01036834716797</v>
+      </c>
+      <c r="L192">
+        <v>16.668807983398438</v>
+      </c>
+      <c r="M192">
+        <v>14.934586524963379</v>
+      </c>
+      <c r="N192">
+        <v>0.6602665185928345</v>
+      </c>
+      <c r="O192">
+        <v>0.5573752522468567</v>
+      </c>
+      <c r="P192">
+        <v>0.3303113877773285</v>
+      </c>
+      <c r="Q192">
+        <v>65.20209503173828</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B193" t="str">
+        <v>10:24:54 ч.</v>
+      </c>
+      <c r="C193" t="str">
+        <v>Priem KM</v>
+      </c>
+      <c r="D193">
+        <v>5578.032217809962</v>
+      </c>
+      <c r="E193">
+        <v>235.46128845214844</v>
+      </c>
+      <c r="F193">
+        <v>236.4347686767578</v>
+      </c>
+      <c r="G193">
+        <v>237.74017333984375</v>
+      </c>
+      <c r="H193">
+        <v>37.82333755493164</v>
+      </c>
+      <c r="I193">
+        <v>37.774627685546875</v>
+      </c>
+      <c r="J193">
+        <v>41.236595153808594</v>
+      </c>
+      <c r="K193">
+        <v>3125.078125</v>
+      </c>
+      <c r="L193">
+        <v>3820.767822265625</v>
+      </c>
+      <c r="M193">
+        <v>3552.668212890625</v>
+      </c>
+      <c r="N193">
+        <v>0.35089850425720215</v>
+      </c>
+      <c r="O193">
+        <v>0.4277983009815216</v>
+      </c>
+      <c r="P193">
+        <v>0.36238420009613037</v>
+      </c>
+      <c r="Q193">
+        <v>10498.5146484375</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B194" t="str">
+        <v>10:24:54 ч.</v>
+      </c>
+      <c r="C194" t="str">
+        <v>Priem UHT</v>
+      </c>
+      <c r="D194">
+        <v>866.5192368139122</v>
+      </c>
+      <c r="E194">
+        <v>235.5312957763672</v>
+      </c>
+      <c r="F194">
+        <v>236.24705505371094</v>
+      </c>
+      <c r="G194">
+        <v>237.73773193359375</v>
+      </c>
+      <c r="H194">
+        <v>0.9072798490524292</v>
+      </c>
+      <c r="I194">
+        <v>0.5247218608856201</v>
+      </c>
+      <c r="J194">
+        <v>0.816804051399231</v>
+      </c>
+      <c r="K194">
+        <v>112.47900390625</v>
+      </c>
+      <c r="L194">
+        <v>87.29956817626953</v>
+      </c>
+      <c r="M194">
+        <v>59.78335952758789</v>
+      </c>
+      <c r="N194">
+        <v>0.5260201096534729</v>
+      </c>
+      <c r="O194">
+        <v>0.7025721669197083</v>
+      </c>
+      <c r="P194">
+        <v>0.3077700138092041</v>
+      </c>
+      <c r="Q194">
+        <v>259.5619201660156</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B195" t="str">
+        <v>10:26:19 ч.</v>
+      </c>
+      <c r="C195" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D195">
+        <v>139039.06149236744</v>
+      </c>
+      <c r="E195">
+        <v>233.9817352294922</v>
+      </c>
+      <c r="F195">
+        <v>234.54605102539062</v>
+      </c>
+      <c r="G195">
+        <v>236.5984344482422</v>
+      </c>
+      <c r="H195">
+        <v>1.588517665863037</v>
+      </c>
+      <c r="I195">
+        <v>1.6263749599456787</v>
+      </c>
+      <c r="J195">
+        <v>1.464691400527954</v>
+      </c>
+      <c r="K195">
+        <v>267.912841796875</v>
+      </c>
+      <c r="L195">
+        <v>201.06646728515625</v>
+      </c>
+      <c r="M195">
+        <v>210.91571044921875</v>
+      </c>
+      <c r="N195">
+        <v>0.7223267555236816</v>
+      </c>
+      <c r="O195">
+        <v>0.5271904468536377</v>
+      </c>
+      <c r="P195">
+        <v>0.6125448942184448</v>
+      </c>
+      <c r="Q195">
+        <v>680.999267578125</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B196" t="str">
+        <v>10:26:19 ч.</v>
+      </c>
+      <c r="C196" t="str">
+        <v>Ampak</v>
+      </c>
+      <c r="D196">
+        <v>41475.0658776434</v>
+      </c>
+      <c r="E196">
+        <v>234.3819580078125</v>
+      </c>
+      <c r="F196">
+        <v>234.43161010742188</v>
+      </c>
+      <c r="G196">
+        <v>236.171630859375</v>
+      </c>
+      <c r="H196">
+        <v>26.72048568725586</v>
+      </c>
+      <c r="I196">
+        <v>26.465396881103516</v>
+      </c>
+      <c r="J196">
+        <v>19.741539001464844</v>
+      </c>
+      <c r="K196">
+        <v>5624.80859375</v>
+      </c>
+      <c r="L196">
+        <v>5214.068359375</v>
+      </c>
+      <c r="M196">
+        <v>3769.8193359375</v>
+      </c>
+      <c r="N196">
+        <v>0.8562756180763245</v>
+      </c>
+      <c r="O196">
+        <v>0.8407061100006104</v>
+      </c>
+      <c r="P196">
+        <v>0.8085592985153198</v>
+      </c>
+      <c r="Q196">
+        <v>14608.6962890625</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B197" t="str">
+        <v>10:26:19 ч.</v>
+      </c>
+      <c r="C197" t="str">
+        <v>Ledena Voda</v>
+      </c>
+      <c r="D197">
+        <v>246438.28892003876</v>
+      </c>
+      <c r="E197">
+        <v>236.84962463378906</v>
+      </c>
+      <c r="F197">
+        <v>236.80368041992188</v>
+      </c>
+      <c r="G197">
+        <v>238.17996215820312</v>
+      </c>
+      <c r="H197">
+        <v>5.4135637283325195</v>
+      </c>
+      <c r="I197">
+        <v>6.169074058532715</v>
+      </c>
+      <c r="J197">
+        <v>3.991792678833008</v>
+      </c>
+      <c r="K197">
+        <v>1228.9888916015625</v>
+      </c>
+      <c r="L197">
+        <v>1455.3514404296875</v>
+      </c>
+      <c r="M197">
+        <v>948.8785400390625</v>
+      </c>
+      <c r="N197">
+        <v>0.958381175994873</v>
+      </c>
+      <c r="O197">
+        <v>0.9962363243103027</v>
+      </c>
+      <c r="P197">
+        <v>0.9978419542312622</v>
+      </c>
+      <c r="Q197">
+        <v>3637.488037109375</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B198" t="str">
+        <v>10:26:19 ч.</v>
+      </c>
+      <c r="C198" t="str">
+        <v>Hladilnici</v>
+      </c>
+      <c r="D198">
+        <v>181739.4920827224</v>
+      </c>
+      <c r="E198">
+        <v>237.78192138671875</v>
+      </c>
+      <c r="F198">
+        <v>236.338623046875</v>
+      </c>
+      <c r="G198">
+        <v>236.24496459960938</v>
+      </c>
+      <c r="H198">
+        <v>10.105545043945312</v>
+      </c>
+      <c r="I198">
+        <v>8.881404876708984</v>
+      </c>
+      <c r="J198">
+        <v>11.943553924560547</v>
+      </c>
+      <c r="K198">
+        <v>2075.62255859375</v>
+      </c>
+      <c r="L198">
+        <v>1758.6192626953125</v>
+      </c>
+      <c r="M198">
+        <v>2608.964111328125</v>
+      </c>
+      <c r="N198">
+        <v>0.8637931942939758</v>
+      </c>
+      <c r="O198">
+        <v>0.8378291130065918</v>
+      </c>
+      <c r="P198">
+        <v>0.9246385097503662</v>
+      </c>
+      <c r="Q198">
+        <v>6443.2060546875</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B199" t="str">
+        <v>10:26:19 ч.</v>
+      </c>
+      <c r="C199" t="str">
+        <v>Kompresorno</v>
+      </c>
+      <c r="D199">
+        <v>49917.17290264915</v>
+      </c>
+      <c r="E199">
+        <v>235.72439575195312</v>
+      </c>
+      <c r="F199">
+        <v>233.53538513183594</v>
+      </c>
+      <c r="G199">
+        <v>233.56036376953125</v>
+      </c>
+      <c r="H199">
+        <v>45.7634162902832</v>
+      </c>
+      <c r="I199">
+        <v>39.079410552978516</v>
+      </c>
+      <c r="J199">
+        <v>41.619972229003906</v>
+      </c>
+      <c r="K199">
+        <v>8802.302734375</v>
+      </c>
+      <c r="L199">
+        <v>7326.533203125</v>
+      </c>
+      <c r="M199">
+        <v>7354.80908203125</v>
+      </c>
+      <c r="N199">
+        <v>0.81596839427948</v>
+      </c>
+      <c r="O199">
+        <v>0.802782416343689</v>
+      </c>
+      <c r="P199">
+        <v>0.756607174873352</v>
+      </c>
+      <c r="Q199">
+        <v>23483.64453125</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B200" t="str">
+        <v>10:26:19 ч.</v>
+      </c>
+      <c r="C200" t="str">
+        <v>Priemno</v>
+      </c>
+      <c r="D200">
+        <v>59435.82547662627</v>
+      </c>
+      <c r="E200">
+        <v>235.53916931152344</v>
+      </c>
+      <c r="F200">
+        <v>235.93492126464844</v>
+      </c>
+      <c r="G200">
+        <v>237.4164581298828</v>
+      </c>
+      <c r="H200">
+        <v>49.825130462646484</v>
+      </c>
+      <c r="I200">
+        <v>44.66664123535156</v>
+      </c>
+      <c r="J200">
+        <v>46.875404357910156</v>
+      </c>
+      <c r="K200">
+        <v>7427.59033203125</v>
+      </c>
+      <c r="L200">
+        <v>6184.44677734375</v>
+      </c>
+      <c r="M200">
+        <v>6354.88720703125</v>
+      </c>
+      <c r="N200">
+        <v>0.6350899338722229</v>
+      </c>
+      <c r="O200">
+        <v>0.5832528471946716</v>
+      </c>
+      <c r="P200">
+        <v>0.5672142505645752</v>
+      </c>
+      <c r="Q200">
+        <v>20057.6015625</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B201" t="str">
+        <v>10:26:19 ч.</v>
+      </c>
+      <c r="C201" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="D201">
+        <v>239034.91349416476</v>
+      </c>
+      <c r="E201">
+        <v>235.86256408691406</v>
+      </c>
+      <c r="F201">
+        <v>236.1346893310547</v>
+      </c>
+      <c r="G201">
+        <v>238.28086853027344</v>
+      </c>
+      <c r="H201">
+        <v>73.76100158691406</v>
+      </c>
+      <c r="I201">
+        <v>87.97610473632812</v>
+      </c>
+      <c r="J201">
+        <v>86.67045593261719</v>
+      </c>
+      <c r="K201">
+        <v>15064.767578125</v>
+      </c>
+      <c r="L201">
+        <v>17214.36328125</v>
+      </c>
+      <c r="M201">
+        <v>18036.59765625</v>
+      </c>
+      <c r="N201">
+        <v>0.8615300059318542</v>
+      </c>
+      <c r="O201">
+        <v>0.8159970045089722</v>
+      </c>
+      <c r="P201">
+        <v>0.8732785582542419</v>
+      </c>
+      <c r="Q201">
+        <v>50315.73046875</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B202" t="str">
+        <v>10:26:19 ч.</v>
+      </c>
+      <c r="C202" t="str">
+        <v>HOMO UHT</v>
+      </c>
+      <c r="D202">
+        <v>1828.0892908756512</v>
+      </c>
+      <c r="E202">
+        <v>235.57801818847656</v>
+      </c>
+      <c r="F202">
+        <v>236.20631408691406</v>
+      </c>
+      <c r="G202">
+        <v>237.21746826171875</v>
+      </c>
+      <c r="H202">
+        <v>0.22426998615264893</v>
+      </c>
+      <c r="I202">
+        <v>0.12240338325500488</v>
+      </c>
+      <c r="J202">
+        <v>0.1989315152168274</v>
+      </c>
+      <c r="K202">
+        <v>34.575828552246094</v>
+      </c>
+      <c r="L202">
+        <v>16.149890899658203</v>
+      </c>
+      <c r="M202">
+        <v>15.004110336303711</v>
+      </c>
+      <c r="N202">
+        <v>0.6544352173805237</v>
+      </c>
+      <c r="O202">
+        <v>0.5561305284500122</v>
+      </c>
+      <c r="P202">
+        <v>0.3228110671043396</v>
+      </c>
+      <c r="Q202">
+        <v>65.43677520751953</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B203" t="str">
+        <v>10:26:19 ч.</v>
+      </c>
+      <c r="C203" t="str">
+        <v>Priem KM</v>
+      </c>
+      <c r="D203">
+        <v>5578.279630816387</v>
+      </c>
+      <c r="E203">
+        <v>235.47682189941406</v>
+      </c>
+      <c r="F203">
+        <v>236.05856323242188</v>
+      </c>
+      <c r="G203">
+        <v>237.31724548339844</v>
+      </c>
+      <c r="H203">
+        <v>38.03615188598633</v>
+      </c>
+      <c r="I203">
+        <v>37.458065032958984</v>
+      </c>
+      <c r="J203">
+        <v>40.730743408203125</v>
+      </c>
+      <c r="K203">
+        <v>3167.77880859375</v>
+      </c>
+      <c r="L203">
+        <v>3707.9951171875</v>
+      </c>
+      <c r="M203">
+        <v>3554.32568359375</v>
+      </c>
+      <c r="N203">
+        <v>0.3522748649120331</v>
+      </c>
+      <c r="O203">
+        <v>0.4188157021999359</v>
+      </c>
+      <c r="P203">
+        <v>0.3672614097595215</v>
+      </c>
+      <c r="Q203">
+        <v>10415.2685546875</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B204" t="str">
+        <v>10:26:19 ч.</v>
+      </c>
+      <c r="C204" t="str">
+        <v>Priem UHT</v>
+      </c>
+      <c r="D204">
+        <v>866.5253112748732</v>
+      </c>
+      <c r="E204">
+        <v>235.56854248046875</v>
+      </c>
+      <c r="F204">
+        <v>235.95156860351562</v>
+      </c>
+      <c r="G204">
+        <v>237.3306121826172</v>
+      </c>
+      <c r="H204">
+        <v>0.9047417640686035</v>
+      </c>
+      <c r="I204">
+        <v>0.5343359112739563</v>
+      </c>
+      <c r="J204">
+        <v>0.8071332573890686</v>
+      </c>
+      <c r="K204">
+        <v>109.97601318359375</v>
+      </c>
+      <c r="L204">
+        <v>89.62322235107422</v>
+      </c>
+      <c r="M204">
+        <v>59.0061149597168</v>
+      </c>
+      <c r="N204">
+        <v>0.5176076889038086</v>
+      </c>
+      <c r="O204">
+        <v>0.7036102414131165</v>
+      </c>
+      <c r="P204">
+        <v>0.31126201152801514</v>
+      </c>
+      <c r="Q204">
+        <v>258.6053466796875</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q131"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q204"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed bug whit reconecting to the network
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -992,7 +992,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q204"/>
+  <dimension ref="A1:Q265"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -11806,9 +11806,3203 @@
         <v>258.6053466796875</v>
       </c>
     </row>
+    <row r="205">
+      <c r="A205" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B205" t="str">
+        <v>10:30:39 ч.</v>
+      </c>
+      <c r="C205" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D205">
+        <v>139039.1122722022</v>
+      </c>
+      <c r="E205">
+        <v>233.6160125732422</v>
+      </c>
+      <c r="F205">
+        <v>233.54428100585938</v>
+      </c>
+      <c r="G205">
+        <v>235.7630615234375</v>
+      </c>
+      <c r="H205">
+        <v>1.6086549758911133</v>
+      </c>
+      <c r="I205">
+        <v>1.6447025537490845</v>
+      </c>
+      <c r="J205">
+        <v>1.4721304178237915</v>
+      </c>
+      <c r="K205">
+        <v>268.0513000488281</v>
+      </c>
+      <c r="L205">
+        <v>202.4491424560547</v>
+      </c>
+      <c r="M205">
+        <v>213.2518310546875</v>
+      </c>
+      <c r="N205">
+        <v>0.709141731262207</v>
+      </c>
+      <c r="O205">
+        <v>0.5265881419181824</v>
+      </c>
+      <c r="P205">
+        <v>0.6139410138130188</v>
+      </c>
+      <c r="Q205">
+        <v>682.2791748046875</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B206" t="str">
+        <v>10:30:39 ч.</v>
+      </c>
+      <c r="C206" t="str">
+        <v>Ampak</v>
+      </c>
+      <c r="D206">
+        <v>41476.484440702014</v>
+      </c>
+      <c r="E206">
+        <v>234.2912139892578</v>
+      </c>
+      <c r="F206">
+        <v>233.83457946777344</v>
+      </c>
+      <c r="G206">
+        <v>236.02679443359375</v>
+      </c>
+      <c r="H206">
+        <v>25.738685607910156</v>
+      </c>
+      <c r="I206">
+        <v>29.367277145385742</v>
+      </c>
+      <c r="J206">
+        <v>19.458566665649414</v>
+      </c>
+      <c r="K206">
+        <v>5445.453125</v>
+      </c>
+      <c r="L206">
+        <v>6302.1533203125</v>
+      </c>
+      <c r="M206">
+        <v>4123.04443359375</v>
+      </c>
+      <c r="N206">
+        <v>0.9030081629753113</v>
+      </c>
+      <c r="O206">
+        <v>0.9177334308624268</v>
+      </c>
+      <c r="P206">
+        <v>0.8977302312850952</v>
+      </c>
+      <c r="Q206">
+        <v>15870.650390625</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B207" t="str">
+        <v>10:30:39 ч.</v>
+      </c>
+      <c r="C207" t="str">
+        <v>Ledena Voda</v>
+      </c>
+      <c r="D207">
+        <v>246438.53615790344</v>
+      </c>
+      <c r="E207">
+        <v>236.33975219726562</v>
+      </c>
+      <c r="F207">
+        <v>236.63217163085938</v>
+      </c>
+      <c r="G207">
+        <v>238.17384338378906</v>
+      </c>
+      <c r="H207">
+        <v>0.16986265778541565</v>
+      </c>
+      <c r="I207">
+        <v>0.2728463411331177</v>
+      </c>
+      <c r="J207">
+        <v>0.43916982412338257</v>
+      </c>
+      <c r="K207">
+        <v>31.068817138671875</v>
+      </c>
+      <c r="L207">
+        <v>-12.970857620239258</v>
+      </c>
+      <c r="M207">
+        <v>54.0776481628418</v>
+      </c>
+      <c r="N207">
+        <v>0.7739092707633972</v>
+      </c>
+      <c r="O207">
+        <v>0.20089855790138245</v>
+      </c>
+      <c r="P207">
+        <v>0.5170008540153503</v>
+      </c>
+      <c r="Q207">
+        <v>72.17560577392578</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B208" t="str">
+        <v>10:30:39 ч.</v>
+      </c>
+      <c r="C208" t="str">
+        <v>Hladilnici</v>
+      </c>
+      <c r="D208">
+        <v>181739.93605299832</v>
+      </c>
+      <c r="E208">
+        <v>237.74041748046875</v>
+      </c>
+      <c r="F208">
+        <v>236.07667541503906</v>
+      </c>
+      <c r="G208">
+        <v>236.09884643554688</v>
+      </c>
+      <c r="H208">
+        <v>8.623700141906738</v>
+      </c>
+      <c r="I208">
+        <v>8.869159698486328</v>
+      </c>
+      <c r="J208">
+        <v>11.890107154846191</v>
+      </c>
+      <c r="K208">
+        <v>1734.28173828125</v>
+      </c>
+      <c r="L208">
+        <v>1761.8232421875</v>
+      </c>
+      <c r="M208">
+        <v>2592.2294921875</v>
+      </c>
+      <c r="N208">
+        <v>0.8459078073501587</v>
+      </c>
+      <c r="O208">
+        <v>0.8414469957351685</v>
+      </c>
+      <c r="P208">
+        <v>0.9233986735343933</v>
+      </c>
+      <c r="Q208">
+        <v>6083.79931640625</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B209" t="str">
+        <v>10:30:39 ч.</v>
+      </c>
+      <c r="C209" t="str">
+        <v>Kompresorno</v>
+      </c>
+      <c r="D209">
+        <v>49918.83628921078</v>
+      </c>
+      <c r="E209">
+        <v>236.279052734375</v>
+      </c>
+      <c r="F209">
+        <v>234.46717834472656</v>
+      </c>
+      <c r="G209">
+        <v>233.760498046875</v>
+      </c>
+      <c r="H209">
+        <v>45.05590057373047</v>
+      </c>
+      <c r="I209">
+        <v>37.54328155517578</v>
+      </c>
+      <c r="J209">
+        <v>41.62570571899414</v>
+      </c>
+      <c r="K209">
+        <v>8703.2763671875</v>
+      </c>
+      <c r="L209">
+        <v>6996.837890625</v>
+      </c>
+      <c r="M209">
+        <v>7049.28173828125</v>
+      </c>
+      <c r="N209">
+        <v>0.8262863159179688</v>
+      </c>
+      <c r="O209">
+        <v>0.8067534565925598</v>
+      </c>
+      <c r="P209">
+        <v>0.7409927248954773</v>
+      </c>
+      <c r="Q209">
+        <v>22947.87109375</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B210" t="str">
+        <v>10:30:39 ч.</v>
+      </c>
+      <c r="C210" t="str">
+        <v>Priemno</v>
+      </c>
+      <c r="D210">
+        <v>59437.620707842936</v>
+      </c>
+      <c r="E210">
+        <v>235.22927856445312</v>
+      </c>
+      <c r="F210">
+        <v>235.90391540527344</v>
+      </c>
+      <c r="G210">
+        <v>237.39932250976562</v>
+      </c>
+      <c r="H210">
+        <v>66.88658905029297</v>
+      </c>
+      <c r="I210">
+        <v>58.20016098022461</v>
+      </c>
+      <c r="J210">
+        <v>60.69542694091797</v>
+      </c>
+      <c r="K210">
+        <v>11850.87109375</v>
+      </c>
+      <c r="L210">
+        <v>9884.421875</v>
+      </c>
+      <c r="M210">
+        <v>10391.3681640625</v>
+      </c>
+      <c r="N210">
+        <v>0.7520896196365356</v>
+      </c>
+      <c r="O210">
+        <v>0.7205538749694824</v>
+      </c>
+      <c r="P210">
+        <v>0.7219008207321167</v>
+      </c>
+      <c r="Q210">
+        <v>32126.66015625</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B211" t="str">
+        <v>10:30:39 ч.</v>
+      </c>
+      <c r="C211" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="D211">
+        <v>239038.65312811072</v>
+      </c>
+      <c r="E211">
+        <v>235.86624145507812</v>
+      </c>
+      <c r="F211">
+        <v>236.01702880859375</v>
+      </c>
+      <c r="G211">
+        <v>238.38624572753906</v>
+      </c>
+      <c r="H211">
+        <v>70.71864318847656</v>
+      </c>
+      <c r="I211">
+        <v>92.12740325927734</v>
+      </c>
+      <c r="J211">
+        <v>85.55168914794922</v>
+      </c>
+      <c r="K211">
+        <v>14713.2724609375</v>
+      </c>
+      <c r="L211">
+        <v>18501.125</v>
+      </c>
+      <c r="M211">
+        <v>18457.4140625</v>
+      </c>
+      <c r="N211">
+        <v>0.8820832371711731</v>
+      </c>
+      <c r="O211">
+        <v>0.8508753776550293</v>
+      </c>
+      <c r="P211">
+        <v>0.9050260186195374</v>
+      </c>
+      <c r="Q211">
+        <v>51671.8125</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B212" t="str">
+        <v>10:30:39 ч.</v>
+      </c>
+      <c r="C212" t="str">
+        <v>HOMO UHT</v>
+      </c>
+      <c r="D212">
+        <v>1828.0940176454292</v>
+      </c>
+      <c r="E212">
+        <v>235.14193725585938</v>
+      </c>
+      <c r="F212">
+        <v>235.995361328125</v>
+      </c>
+      <c r="G212">
+        <v>237.28378295898438</v>
+      </c>
+      <c r="H212">
+        <v>0.19846567511558533</v>
+      </c>
+      <c r="I212">
+        <v>0.143899604678154</v>
+      </c>
+      <c r="J212">
+        <v>0.17889045178890228</v>
+      </c>
+      <c r="K212">
+        <v>31.971660614013672</v>
+      </c>
+      <c r="L212">
+        <v>17.931798934936523</v>
+      </c>
+      <c r="M212">
+        <v>14.815681457519531</v>
+      </c>
+      <c r="N212">
+        <v>0.6850932836532593</v>
+      </c>
+      <c r="O212">
+        <v>0.528032660484314</v>
+      </c>
+      <c r="P212">
+        <v>0.3490329086780548</v>
+      </c>
+      <c r="Q212">
+        <v>64.71914672851562</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B213" t="str">
+        <v>10:30:39 ч.</v>
+      </c>
+      <c r="C213" t="str">
+        <v>Priem KM</v>
+      </c>
+      <c r="D213">
+        <v>5579.027915057825</v>
+      </c>
+      <c r="E213">
+        <v>235.07032775878906</v>
+      </c>
+      <c r="F213">
+        <v>235.76937866210938</v>
+      </c>
+      <c r="G213">
+        <v>237.34814453125</v>
+      </c>
+      <c r="H213">
+        <v>37.91604995727539</v>
+      </c>
+      <c r="I213">
+        <v>37.23908233642578</v>
+      </c>
+      <c r="J213">
+        <v>41.04484176635742</v>
+      </c>
+      <c r="K213">
+        <v>3079.670654296875</v>
+      </c>
+      <c r="L213">
+        <v>3718.757080078125</v>
+      </c>
+      <c r="M213">
+        <v>3586.460205078125</v>
+      </c>
+      <c r="N213">
+        <v>0.34508371353149414</v>
+      </c>
+      <c r="O213">
+        <v>0.4230785071849823</v>
+      </c>
+      <c r="P213">
+        <v>0.3681081235408783</v>
+      </c>
+      <c r="Q213">
+        <v>10384.8876953125</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B214" t="str">
+        <v>10:30:39 ч.</v>
+      </c>
+      <c r="C214" t="str">
+        <v>Priem UHT</v>
+      </c>
+      <c r="D214">
+        <v>866.5440731710104</v>
+      </c>
+      <c r="E214">
+        <v>235.2001495361328</v>
+      </c>
+      <c r="F214">
+        <v>235.67623901367188</v>
+      </c>
+      <c r="G214">
+        <v>237.3136749267578</v>
+      </c>
+      <c r="H214">
+        <v>0.9099137783050537</v>
+      </c>
+      <c r="I214">
+        <v>0.5376279354095459</v>
+      </c>
+      <c r="J214">
+        <v>0.812707781791687</v>
+      </c>
+      <c r="K214">
+        <v>112.09457397460938</v>
+      </c>
+      <c r="L214">
+        <v>88.24072265625</v>
+      </c>
+      <c r="M214">
+        <v>59.24945068359375</v>
+      </c>
+      <c r="N214">
+        <v>0.523777425289154</v>
+      </c>
+      <c r="O214">
+        <v>0.6964203119277954</v>
+      </c>
+      <c r="P214">
+        <v>0.3072041869163513</v>
+      </c>
+      <c r="Q214">
+        <v>258.99090576171875</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B215" t="str">
+        <v>10:32:39 ч.</v>
+      </c>
+      <c r="C215" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D215">
+        <v>139039.13498547123</v>
+      </c>
+      <c r="E215">
+        <v>233.88623046875</v>
+      </c>
+      <c r="F215">
+        <v>234.00674438476562</v>
+      </c>
+      <c r="G215">
+        <v>236.14801025390625</v>
+      </c>
+      <c r="H215">
+        <v>1.61445152759552</v>
+      </c>
+      <c r="I215">
+        <v>1.642197847366333</v>
+      </c>
+      <c r="J215">
+        <v>1.4843205213546753</v>
+      </c>
+      <c r="K215">
+        <v>265.220947265625</v>
+      </c>
+      <c r="L215">
+        <v>202.17654418945312</v>
+      </c>
+      <c r="M215">
+        <v>214.05519104003906</v>
+      </c>
+      <c r="N215">
+        <v>0.7041139006614685</v>
+      </c>
+      <c r="O215">
+        <v>0.5271958112716675</v>
+      </c>
+      <c r="P215">
+        <v>0.6105344295501709</v>
+      </c>
+      <c r="Q215">
+        <v>682.39013671875</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B216" t="str">
+        <v>10:32:39 ч.</v>
+      </c>
+      <c r="C216" t="str">
+        <v>Ampak</v>
+      </c>
+      <c r="D216">
+        <v>41477.134750001605</v>
+      </c>
+      <c r="E216">
+        <v>233.75035095214844</v>
+      </c>
+      <c r="F216">
+        <v>233.5705108642578</v>
+      </c>
+      <c r="G216">
+        <v>236.1805877685547</v>
+      </c>
+      <c r="H216">
+        <v>27.430696487426758</v>
+      </c>
+      <c r="I216">
+        <v>28.998308181762695</v>
+      </c>
+      <c r="J216">
+        <v>17.949710845947266</v>
+      </c>
+      <c r="K216">
+        <v>5865.123046875</v>
+      </c>
+      <c r="L216">
+        <v>6178.791015625</v>
+      </c>
+      <c r="M216">
+        <v>3694.89013671875</v>
+      </c>
+      <c r="N216">
+        <v>0.9147477746009827</v>
+      </c>
+      <c r="O216">
+        <v>0.9122478365898132</v>
+      </c>
+      <c r="P216">
+        <v>0.8715652227401733</v>
+      </c>
+      <c r="Q216">
+        <v>15738.8037109375</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B217" t="str">
+        <v>10:32:39 ч.</v>
+      </c>
+      <c r="C217" t="str">
+        <v>Ledena Voda</v>
+      </c>
+      <c r="D217">
+        <v>246438.53855392736</v>
+      </c>
+      <c r="E217">
+        <v>236.0473175048828</v>
+      </c>
+      <c r="F217">
+        <v>236.4557647705078</v>
+      </c>
+      <c r="G217">
+        <v>238.04168701171875</v>
+      </c>
+      <c r="H217">
+        <v>0.167975515127182</v>
+      </c>
+      <c r="I217">
+        <v>0.27461597323417664</v>
+      </c>
+      <c r="J217">
+        <v>0.44494813680648804</v>
+      </c>
+      <c r="K217">
+        <v>31.15643310546875</v>
+      </c>
+      <c r="L217">
+        <v>-14.00464916229248</v>
+      </c>
+      <c r="M217">
+        <v>54.705299377441406</v>
+      </c>
+      <c r="N217">
+        <v>0.7857831120491028</v>
+      </c>
+      <c r="O217">
+        <v>0.21567337214946747</v>
+      </c>
+      <c r="P217">
+        <v>0.5164960026741028</v>
+      </c>
+      <c r="Q217">
+        <v>71.85708618164062</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B218" t="str">
+        <v>10:32:39 ч.</v>
+      </c>
+      <c r="C218" t="str">
+        <v>Hladilnici</v>
+      </c>
+      <c r="D218">
+        <v>181740.4140239059</v>
+      </c>
+      <c r="E218">
+        <v>237.18768310546875</v>
+      </c>
+      <c r="F218">
+        <v>235.52586364746094</v>
+      </c>
+      <c r="G218">
+        <v>235.61709594726562</v>
+      </c>
+      <c r="H218">
+        <v>42.49772644042969</v>
+      </c>
+      <c r="I218">
+        <v>39.93517303466797</v>
+      </c>
+      <c r="J218">
+        <v>43.093536376953125</v>
+      </c>
+      <c r="K218">
+        <v>7897.12109375</v>
+      </c>
+      <c r="L218">
+        <v>7477.5</v>
+      </c>
+      <c r="M218">
+        <v>8538.255859375</v>
+      </c>
+      <c r="N218">
+        <v>0.7834494113922119</v>
+      </c>
+      <c r="O218">
+        <v>0.7949910163879395</v>
+      </c>
+      <c r="P218">
+        <v>0.842609167098999</v>
+      </c>
+      <c r="Q218">
+        <v>23932.439453125</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B219" t="str">
+        <v>10:32:39 ч.</v>
+      </c>
+      <c r="C219" t="str">
+        <v>Kompresorno</v>
+      </c>
+      <c r="D219">
+        <v>49919.596167447075</v>
+      </c>
+      <c r="E219">
+        <v>236.26593017578125</v>
+      </c>
+      <c r="F219">
+        <v>234.01156616210938</v>
+      </c>
+      <c r="G219">
+        <v>233.60243225097656</v>
+      </c>
+      <c r="H219">
+        <v>44.099456787109375</v>
+      </c>
+      <c r="I219">
+        <v>37.67361831665039</v>
+      </c>
+      <c r="J219">
+        <v>41.17554473876953</v>
+      </c>
+      <c r="K219">
+        <v>8414.7939453125</v>
+      </c>
+      <c r="L219">
+        <v>7025.513671875</v>
+      </c>
+      <c r="M219">
+        <v>7282.091796875</v>
+      </c>
+      <c r="N219">
+        <v>0.8075350522994995</v>
+      </c>
+      <c r="O219">
+        <v>0.7964720726013184</v>
+      </c>
+      <c r="P219">
+        <v>0.7602303624153137</v>
+      </c>
+      <c r="Q219">
+        <v>22919.80078125</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B220" t="str">
+        <v>10:32:39 ч.</v>
+      </c>
+      <c r="C220" t="str">
+        <v>Priemno</v>
+      </c>
+      <c r="D220">
+        <v>59438.78821455108</v>
+      </c>
+      <c r="E220">
+        <v>235.01107788085938</v>
+      </c>
+      <c r="F220">
+        <v>235.6643829345703</v>
+      </c>
+      <c r="G220">
+        <v>237.2516326904297</v>
+      </c>
+      <c r="H220">
+        <v>74.2812728881836</v>
+      </c>
+      <c r="I220">
+        <v>65.00670623779297</v>
+      </c>
+      <c r="J220">
+        <v>68.21916961669922</v>
+      </c>
+      <c r="K220">
+        <v>13786.19140625</v>
+      </c>
+      <c r="L220">
+        <v>11871.15234375</v>
+      </c>
+      <c r="M220">
+        <v>12518.7177734375</v>
+      </c>
+      <c r="N220">
+        <v>0.7910997271537781</v>
+      </c>
+      <c r="O220">
+        <v>0.7748034596443176</v>
+      </c>
+      <c r="P220">
+        <v>0.7734577655792236</v>
+      </c>
+      <c r="Q220">
+        <v>38235.09375</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B221" t="str">
+        <v>10:32:39 ч.</v>
+      </c>
+      <c r="C221" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="D221">
+        <v>239040.6225024932</v>
+      </c>
+      <c r="E221">
+        <v>235.7112579345703</v>
+      </c>
+      <c r="F221">
+        <v>235.72276306152344</v>
+      </c>
+      <c r="G221">
+        <v>238.17835998535156</v>
+      </c>
+      <c r="H221">
+        <v>105.88667297363281</v>
+      </c>
+      <c r="I221">
+        <v>123.51707458496094</v>
+      </c>
+      <c r="J221">
+        <v>121.19481658935547</v>
+      </c>
+      <c r="K221">
+        <v>22964.7109375</v>
+      </c>
+      <c r="L221">
+        <v>25779.8125</v>
+      </c>
+      <c r="M221">
+        <v>26733.904296875</v>
+      </c>
+      <c r="N221">
+        <v>0.9203861951828003</v>
+      </c>
+      <c r="O221">
+        <v>0.8854238390922546</v>
+      </c>
+      <c r="P221">
+        <v>0.9261387586593628</v>
+      </c>
+      <c r="Q221">
+        <v>75478.4296875</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B222" t="str">
+        <v>10:32:39 ч.</v>
+      </c>
+      <c r="C222" t="str">
+        <v>HOMO UHT</v>
+      </c>
+      <c r="D222">
+        <v>1828.0961837115738</v>
+      </c>
+      <c r="E222">
+        <v>234.9195556640625</v>
+      </c>
+      <c r="F222">
+        <v>235.6365966796875</v>
+      </c>
+      <c r="G222">
+        <v>236.96881103515625</v>
+      </c>
+      <c r="H222">
+        <v>0.23649069666862488</v>
+      </c>
+      <c r="I222">
+        <v>0.1221909448504448</v>
+      </c>
+      <c r="J222">
+        <v>0.21147409081459045</v>
+      </c>
+      <c r="K222">
+        <v>35.0538215637207</v>
+      </c>
+      <c r="L222">
+        <v>15.740822792053223</v>
+      </c>
+      <c r="M222">
+        <v>15.382892608642578</v>
+      </c>
+      <c r="N222">
+        <v>0.6310933828353882</v>
+      </c>
+      <c r="O222">
+        <v>0.5466957092285156</v>
+      </c>
+      <c r="P222">
+        <v>0.30696555972099304</v>
+      </c>
+      <c r="Q222">
+        <v>66.17753601074219</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B223" t="str">
+        <v>10:32:39 ч.</v>
+      </c>
+      <c r="C223" t="str">
+        <v>Priem KM</v>
+      </c>
+      <c r="D223">
+        <v>5579.37543885343</v>
+      </c>
+      <c r="E223">
+        <v>234.7892608642578</v>
+      </c>
+      <c r="F223">
+        <v>235.554443359375</v>
+      </c>
+      <c r="G223">
+        <v>237.11209106445312</v>
+      </c>
+      <c r="H223">
+        <v>37.753082275390625</v>
+      </c>
+      <c r="I223">
+        <v>37.30858612060547</v>
+      </c>
+      <c r="J223">
+        <v>40.97041702270508</v>
+      </c>
+      <c r="K223">
+        <v>3085.9765625</v>
+      </c>
+      <c r="L223">
+        <v>3747.2783203125</v>
+      </c>
+      <c r="M223">
+        <v>3556.634521484375</v>
+      </c>
+      <c r="N223">
+        <v>0.3469518721103668</v>
+      </c>
+      <c r="O223">
+        <v>0.42489486932754517</v>
+      </c>
+      <c r="P223">
+        <v>0.36584699153900146</v>
+      </c>
+      <c r="Q223">
+        <v>10373.34765625</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B224" t="str">
+        <v>10:32:39 ч.</v>
+      </c>
+      <c r="C224" t="str">
+        <v>Priem UHT</v>
+      </c>
+      <c r="D224">
+        <v>866.5527328672019</v>
+      </c>
+      <c r="E224">
+        <v>234.90582275390625</v>
+      </c>
+      <c r="F224">
+        <v>235.51368713378906</v>
+      </c>
+      <c r="G224">
+        <v>237.1381072998047</v>
+      </c>
+      <c r="H224">
+        <v>0.9221487045288086</v>
+      </c>
+      <c r="I224">
+        <v>0.5252125859260559</v>
+      </c>
+      <c r="J224">
+        <v>0.8285126686096191</v>
+      </c>
+      <c r="K224">
+        <v>115.14787292480469</v>
+      </c>
+      <c r="L224">
+        <v>85.23834991455078</v>
+      </c>
+      <c r="M224">
+        <v>59.813751220703125</v>
+      </c>
+      <c r="N224">
+        <v>0.5315708518028259</v>
+      </c>
+      <c r="O224">
+        <v>0.6891023516654968</v>
+      </c>
+      <c r="P224">
+        <v>0.30443915724754333</v>
+      </c>
+      <c r="Q224">
+        <v>260.1999816894531</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B225" t="str">
+        <v>10:34:39 ч.</v>
+      </c>
+      <c r="C225" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D225">
+        <v>139039.15769678925</v>
+      </c>
+      <c r="E225">
+        <v>232.5717315673828</v>
+      </c>
+      <c r="F225">
+        <v>233.80360412597656</v>
+      </c>
+      <c r="G225">
+        <v>235.7501678466797</v>
+      </c>
+      <c r="H225">
+        <v>1.6067326068878174</v>
+      </c>
+      <c r="I225">
+        <v>1.6316388845443726</v>
+      </c>
+      <c r="J225">
+        <v>1.480056881904602</v>
+      </c>
+      <c r="K225">
+        <v>264.6434326171875</v>
+      </c>
+      <c r="L225">
+        <v>201.40318298339844</v>
+      </c>
+      <c r="M225">
+        <v>215.10728454589844</v>
+      </c>
+      <c r="N225">
+        <v>0.7066896557807922</v>
+      </c>
+      <c r="O225">
+        <v>0.526275098323822</v>
+      </c>
+      <c r="P225">
+        <v>0.615264356136322</v>
+      </c>
+      <c r="Q225">
+        <v>682.79345703125</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B226" t="str">
+        <v>10:34:39 ч.</v>
+      </c>
+      <c r="C226" t="str">
+        <v>Ampak</v>
+      </c>
+      <c r="D226">
+        <v>41477.77505964046</v>
+      </c>
+      <c r="E226">
+        <v>233.18487548828125</v>
+      </c>
+      <c r="F226">
+        <v>234.05136108398438</v>
+      </c>
+      <c r="G226">
+        <v>236.44326782226562</v>
+      </c>
+      <c r="H226">
+        <v>25.97093963623047</v>
+      </c>
+      <c r="I226">
+        <v>23.469465255737305</v>
+      </c>
+      <c r="J226">
+        <v>18.74049949645996</v>
+      </c>
+      <c r="K226">
+        <v>5467.04833984375</v>
+      </c>
+      <c r="L226">
+        <v>4698.2353515625</v>
+      </c>
+      <c r="M226">
+        <v>3954.60693359375</v>
+      </c>
+      <c r="N226">
+        <v>0.9026757478713989</v>
+      </c>
+      <c r="O226">
+        <v>0.8554640412330627</v>
+      </c>
+      <c r="P226">
+        <v>0.8924732804298401</v>
+      </c>
+      <c r="Q226">
+        <v>14119.890625</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B227" t="str">
+        <v>10:34:39 ч.</v>
+      </c>
+      <c r="C227" t="str">
+        <v>Ledena Voda</v>
+      </c>
+      <c r="D227">
+        <v>246438.54091701013</v>
+      </c>
+      <c r="E227">
+        <v>236.31314086914062</v>
+      </c>
+      <c r="F227">
+        <v>236.30833435058594</v>
+      </c>
+      <c r="G227">
+        <v>238.18978881835938</v>
+      </c>
+      <c r="H227">
+        <v>0.1640390008687973</v>
+      </c>
+      <c r="I227">
+        <v>0.2728920578956604</v>
+      </c>
+      <c r="J227">
+        <v>0.43640607595443726</v>
+      </c>
+      <c r="K227">
+        <v>30.085166931152344</v>
+      </c>
+      <c r="L227">
+        <v>-13.003170013427734</v>
+      </c>
+      <c r="M227">
+        <v>54.13838195800781</v>
+      </c>
+      <c r="N227">
+        <v>0.7760995626449585</v>
+      </c>
+      <c r="O227">
+        <v>0.2016412317752838</v>
+      </c>
+      <c r="P227">
+        <v>0.5208244323730469</v>
+      </c>
+      <c r="Q227">
+        <v>71.22038269042969</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B228" t="str">
+        <v>10:34:39 ч.</v>
+      </c>
+      <c r="C228" t="str">
+        <v>Hladilnici</v>
+      </c>
+      <c r="D228">
+        <v>181740.82928331938</v>
+      </c>
+      <c r="E228">
+        <v>237.56675720214844</v>
+      </c>
+      <c r="F228">
+        <v>235.74375915527344</v>
+      </c>
+      <c r="G228">
+        <v>235.7783660888672</v>
+      </c>
+      <c r="H228">
+        <v>11.60966682434082</v>
+      </c>
+      <c r="I228">
+        <v>8.822927474975586</v>
+      </c>
+      <c r="J228">
+        <v>9.239479064941406</v>
+      </c>
+      <c r="K228">
+        <v>2381.129638671875</v>
+      </c>
+      <c r="L228">
+        <v>1736.773193359375</v>
+      </c>
+      <c r="M228">
+        <v>2029.2528076171875</v>
+      </c>
+      <c r="N228">
+        <v>0.8633315563201904</v>
+      </c>
+      <c r="O228">
+        <v>0.8350071907043457</v>
+      </c>
+      <c r="P228">
+        <v>0.9315040111541748</v>
+      </c>
+      <c r="Q228">
+        <v>6147.1552734375</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B229" t="str">
+        <v>10:34:39 ч.</v>
+      </c>
+      <c r="C229" t="str">
+        <v>Kompresorno</v>
+      </c>
+      <c r="D229">
+        <v>49920.35371108745</v>
+      </c>
+      <c r="E229">
+        <v>236.47999572753906</v>
+      </c>
+      <c r="F229">
+        <v>233.243408203125</v>
+      </c>
+      <c r="G229">
+        <v>233.6968536376953</v>
+      </c>
+      <c r="H229">
+        <v>43.76484298706055</v>
+      </c>
+      <c r="I229">
+        <v>37.02483367919922</v>
+      </c>
+      <c r="J229">
+        <v>41.407386779785156</v>
+      </c>
+      <c r="K229">
+        <v>8285.921875</v>
+      </c>
+      <c r="L229">
+        <v>6811.26904296875</v>
+      </c>
+      <c r="M229">
+        <v>7290.84765625</v>
+      </c>
+      <c r="N229">
+        <v>0.8006100058555603</v>
+      </c>
+      <c r="O229">
+        <v>0.7887248992919922</v>
+      </c>
+      <c r="P229">
+        <v>0.7480910420417786</v>
+      </c>
+      <c r="Q229">
+        <v>22119.31640625</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B230" t="str">
+        <v>10:34:39 ч.</v>
+      </c>
+      <c r="C230" t="str">
+        <v>Priemno</v>
+      </c>
+      <c r="D230">
+        <v>59439.85070276463</v>
+      </c>
+      <c r="E230">
+        <v>235.0366668701172</v>
+      </c>
+      <c r="F230">
+        <v>235.5770263671875</v>
+      </c>
+      <c r="G230">
+        <v>237.31906127929688</v>
+      </c>
+      <c r="H230">
+        <v>59.4576301574707</v>
+      </c>
+      <c r="I230">
+        <v>52.805206298828125</v>
+      </c>
+      <c r="J230">
+        <v>54.27684020996094</v>
+      </c>
+      <c r="K230">
+        <v>9908.8564453125</v>
+      </c>
+      <c r="L230">
+        <v>8234.298828125</v>
+      </c>
+      <c r="M230">
+        <v>8320.7587890625</v>
+      </c>
+      <c r="N230">
+        <v>0.7090556621551514</v>
+      </c>
+      <c r="O230">
+        <v>0.6617365479469299</v>
+      </c>
+      <c r="P230">
+        <v>0.643764853477478</v>
+      </c>
+      <c r="Q230">
+        <v>26438.123046875</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B231" t="str">
+        <v>10:34:39 ч.</v>
+      </c>
+      <c r="C231" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="D231">
+        <v>239042.49590486794</v>
+      </c>
+      <c r="E231">
+        <v>235.5507354736328</v>
+      </c>
+      <c r="F231">
+        <v>235.67279052734375</v>
+      </c>
+      <c r="G231">
+        <v>238.2930450439453</v>
+      </c>
+      <c r="H231">
+        <v>69.44644165039062</v>
+      </c>
+      <c r="I231">
+        <v>84.09033966064453</v>
+      </c>
+      <c r="J231">
+        <v>80.99153900146484</v>
+      </c>
+      <c r="K231">
+        <v>13720.9765625</v>
+      </c>
+      <c r="L231">
+        <v>16336.5908203125</v>
+      </c>
+      <c r="M231">
+        <v>17452.369140625</v>
+      </c>
+      <c r="N231">
+        <v>0.8386963605880737</v>
+      </c>
+      <c r="O231">
+        <v>0.824260413646698</v>
+      </c>
+      <c r="P231">
+        <v>0.9042809009552002</v>
+      </c>
+      <c r="Q231">
+        <v>47509.9375</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B232" t="str">
+        <v>10:34:39 ч.</v>
+      </c>
+      <c r="C232" t="str">
+        <v>HOMO UHT</v>
+      </c>
+      <c r="D232">
+        <v>1828.0983614845939</v>
+      </c>
+      <c r="E232">
+        <v>235.01296997070312</v>
+      </c>
+      <c r="F232">
+        <v>235.7880859375</v>
+      </c>
+      <c r="G232">
+        <v>237.2105712890625</v>
+      </c>
+      <c r="H232">
+        <v>0.22100380063056946</v>
+      </c>
+      <c r="I232">
+        <v>0.12831948697566986</v>
+      </c>
+      <c r="J232">
+        <v>0.19623446464538574</v>
+      </c>
+      <c r="K232">
+        <v>33.397125244140625</v>
+      </c>
+      <c r="L232">
+        <v>16.506959915161133</v>
+      </c>
+      <c r="M232">
+        <v>15.026349067687988</v>
+      </c>
+      <c r="N232">
+        <v>0.642995297908783</v>
+      </c>
+      <c r="O232">
+        <v>0.5455048680305481</v>
+      </c>
+      <c r="P232">
+        <v>0.3227136731147766</v>
+      </c>
+      <c r="Q232">
+        <v>64.93043518066406</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B233" t="str">
+        <v>10:34:39 ч.</v>
+      </c>
+      <c r="C233" t="str">
+        <v>Priem KM</v>
+      </c>
+      <c r="D233">
+        <v>5579.717986178206</v>
+      </c>
+      <c r="E233">
+        <v>235.05996704101562</v>
+      </c>
+      <c r="F233">
+        <v>235.75730895996094</v>
+      </c>
+      <c r="G233">
+        <v>237.4981231689453</v>
+      </c>
+      <c r="H233">
+        <v>37.668941497802734</v>
+      </c>
+      <c r="I233">
+        <v>37.21409225463867</v>
+      </c>
+      <c r="J233">
+        <v>41.200721740722656</v>
+      </c>
+      <c r="K233">
+        <v>2954.68115234375</v>
+      </c>
+      <c r="L233">
+        <v>3690.91162109375</v>
+      </c>
+      <c r="M233">
+        <v>3499.859619140625</v>
+      </c>
+      <c r="N233">
+        <v>0.33369410037994385</v>
+      </c>
+      <c r="O233">
+        <v>0.4235636591911316</v>
+      </c>
+      <c r="P233">
+        <v>0.3573322296142578</v>
+      </c>
+      <c r="Q233">
+        <v>10176.1279296875</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B234" t="str">
+        <v>10:34:39 ч.</v>
+      </c>
+      <c r="C234" t="str">
+        <v>Priem UHT</v>
+      </c>
+      <c r="D234">
+        <v>866.5613519980443</v>
+      </c>
+      <c r="E234">
+        <v>235.0978546142578</v>
+      </c>
+      <c r="F234">
+        <v>235.6148681640625</v>
+      </c>
+      <c r="G234">
+        <v>237.41651916503906</v>
+      </c>
+      <c r="H234">
+        <v>0.9103411436080933</v>
+      </c>
+      <c r="I234">
+        <v>0.530348539352417</v>
+      </c>
+      <c r="J234">
+        <v>0.8070218563079834</v>
+      </c>
+      <c r="K234">
+        <v>111.9571533203125</v>
+      </c>
+      <c r="L234">
+        <v>87.88150024414062</v>
+      </c>
+      <c r="M234">
+        <v>59.374839782714844</v>
+      </c>
+      <c r="N234">
+        <v>0.5231172442436218</v>
+      </c>
+      <c r="O234">
+        <v>0.7032883167266846</v>
+      </c>
+      <c r="P234">
+        <v>0.309889018535614</v>
+      </c>
+      <c r="Q234">
+        <v>259.2135009765625</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B235" t="str">
+        <v>10:36:39 ч.</v>
+      </c>
+      <c r="C235" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D235">
+        <v>139039.1804024279</v>
+      </c>
+      <c r="E235">
+        <v>233.89724731445312</v>
+      </c>
+      <c r="F235">
+        <v>234.15634155273438</v>
+      </c>
+      <c r="G235">
+        <v>236.2422637939453</v>
+      </c>
+      <c r="H235">
+        <v>1.6136256456375122</v>
+      </c>
+      <c r="I235">
+        <v>1.6371264457702637</v>
+      </c>
+      <c r="J235">
+        <v>1.4654370546340942</v>
+      </c>
+      <c r="K235">
+        <v>268.34844970703125</v>
+      </c>
+      <c r="L235">
+        <v>199.76702880859375</v>
+      </c>
+      <c r="M235">
+        <v>212.75010681152344</v>
+      </c>
+      <c r="N235">
+        <v>0.7096498012542725</v>
+      </c>
+      <c r="O235">
+        <v>0.5206393003463745</v>
+      </c>
+      <c r="P235">
+        <v>0.614662766456604</v>
+      </c>
+      <c r="Q235">
+        <v>680.8655395507812</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B236" t="str">
+        <v>10:36:39 ч.</v>
+      </c>
+      <c r="C236" t="str">
+        <v>Ampak</v>
+      </c>
+      <c r="D236">
+        <v>41478.40196850281</v>
+      </c>
+      <c r="E236">
+        <v>233.7876739501953</v>
+      </c>
+      <c r="F236">
+        <v>233.91256713867188</v>
+      </c>
+      <c r="G236">
+        <v>236.00991821289062</v>
+      </c>
+      <c r="H236">
+        <v>26.583209991455078</v>
+      </c>
+      <c r="I236">
+        <v>22.754497528076172</v>
+      </c>
+      <c r="J236">
+        <v>17.74081039428711</v>
+      </c>
+      <c r="K236">
+        <v>5654.93896484375</v>
+      </c>
+      <c r="L236">
+        <v>4576.2783203125</v>
+      </c>
+      <c r="M236">
+        <v>3672.895263671875</v>
+      </c>
+      <c r="N236">
+        <v>0.9101812839508057</v>
+      </c>
+      <c r="O236">
+        <v>0.8605206608772278</v>
+      </c>
+      <c r="P236">
+        <v>0.8769422173500061</v>
+      </c>
+      <c r="Q236">
+        <v>13904.1123046875</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B237" t="str">
+        <v>10:36:39 ч.</v>
+      </c>
+      <c r="C237" t="str">
+        <v>Ledena Voda</v>
+      </c>
+      <c r="D237">
+        <v>246438.56323324362</v>
+      </c>
+      <c r="E237">
+        <v>235.7342987060547</v>
+      </c>
+      <c r="F237">
+        <v>236.15362548828125</v>
+      </c>
+      <c r="G237">
+        <v>237.9691619873047</v>
+      </c>
+      <c r="H237">
+        <v>7.173914432525635</v>
+      </c>
+      <c r="I237">
+        <v>7.100147247314453</v>
+      </c>
+      <c r="J237">
+        <v>7.227443695068359</v>
+      </c>
+      <c r="K237">
+        <v>1202.351318359375</v>
+      </c>
+      <c r="L237">
+        <v>1191.7333984375</v>
+      </c>
+      <c r="M237">
+        <v>1256.5506591796875</v>
+      </c>
+      <c r="N237">
+        <v>0.7109718918800354</v>
+      </c>
+      <c r="O237">
+        <v>0.7107504606246948</v>
+      </c>
+      <c r="P237">
+        <v>0.7305915355682373</v>
+      </c>
+      <c r="Q237">
+        <v>3650.63525390625</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B238" t="str">
+        <v>10:36:39 ч.</v>
+      </c>
+      <c r="C238" t="str">
+        <v>Hladilnici</v>
+      </c>
+      <c r="D238">
+        <v>181741.04323989208</v>
+      </c>
+      <c r="E238">
+        <v>237.57762145996094</v>
+      </c>
+      <c r="F238">
+        <v>235.7257843017578</v>
+      </c>
+      <c r="G238">
+        <v>235.82302856445312</v>
+      </c>
+      <c r="H238">
+        <v>10.067845344543457</v>
+      </c>
+      <c r="I238">
+        <v>8.838626861572266</v>
+      </c>
+      <c r="J238">
+        <v>11.668725967407227</v>
+      </c>
+      <c r="K238">
+        <v>2058.7978515625</v>
+      </c>
+      <c r="L238">
+        <v>1740.518310546875</v>
+      </c>
+      <c r="M238">
+        <v>2548.764892578125</v>
+      </c>
+      <c r="N238">
+        <v>0.8607394099235535</v>
+      </c>
+      <c r="O238">
+        <v>0.8353849649429321</v>
+      </c>
+      <c r="P238">
+        <v>0.9262326955795288</v>
+      </c>
+      <c r="Q238">
+        <v>6348.0810546875</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B239" t="str">
+        <v>10:36:39 ч.</v>
+      </c>
+      <c r="C239" t="str">
+        <v>Kompresorno</v>
+      </c>
+      <c r="D239">
+        <v>49921.1188706467</v>
+      </c>
+      <c r="E239">
+        <v>236.30438232421875</v>
+      </c>
+      <c r="F239">
+        <v>234.05148315429688</v>
+      </c>
+      <c r="G239">
+        <v>233.73443603515625</v>
+      </c>
+      <c r="H239">
+        <v>45.8839111328125</v>
+      </c>
+      <c r="I239">
+        <v>37.149024963378906</v>
+      </c>
+      <c r="J239">
+        <v>40.34735870361328</v>
+      </c>
+      <c r="K239">
+        <v>8963.07421875</v>
+      </c>
+      <c r="L239">
+        <v>7031.2861328125</v>
+      </c>
+      <c r="M239">
+        <v>6953.81884765625</v>
+      </c>
+      <c r="N239">
+        <v>0.826655924320221</v>
+      </c>
+      <c r="O239">
+        <v>0.8086786270141602</v>
+      </c>
+      <c r="P239">
+        <v>0.7373701930046082</v>
+      </c>
+      <c r="Q239">
+        <v>22948.1796875</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B240" t="str">
+        <v>10:36:39 ч.</v>
+      </c>
+      <c r="C240" t="str">
+        <v>Priemno</v>
+      </c>
+      <c r="D240">
+        <v>59440.77237623726</v>
+      </c>
+      <c r="E240">
+        <v>234.89236450195312</v>
+      </c>
+      <c r="F240">
+        <v>235.6510772705078</v>
+      </c>
+      <c r="G240">
+        <v>237.36180114746094</v>
+      </c>
+      <c r="H240">
+        <v>62.59813690185547</v>
+      </c>
+      <c r="I240">
+        <v>53.55060958862305</v>
+      </c>
+      <c r="J240">
+        <v>55.38140106201172</v>
+      </c>
+      <c r="K240">
+        <v>10589.3310546875</v>
+      </c>
+      <c r="L240">
+        <v>8549.2783203125</v>
+      </c>
+      <c r="M240">
+        <v>8682.326171875</v>
+      </c>
+      <c r="N240">
+        <v>0.7201753258705139</v>
+      </c>
+      <c r="O240">
+        <v>0.6774786710739136</v>
+      </c>
+      <c r="P240">
+        <v>0.6604825258255005</v>
+      </c>
+      <c r="Q240">
+        <v>27981.556640625</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B241" t="str">
+        <v>10:36:39 ч.</v>
+      </c>
+      <c r="C241" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="D241">
+        <v>239044.21075635654</v>
+      </c>
+      <c r="E241">
+        <v>235.54049682617188</v>
+      </c>
+      <c r="F241">
+        <v>235.60464477539062</v>
+      </c>
+      <c r="G241">
+        <v>238.2957763671875</v>
+      </c>
+      <c r="H241">
+        <v>84.66468811035156</v>
+      </c>
+      <c r="I241">
+        <v>102.27224731445312</v>
+      </c>
+      <c r="J241">
+        <v>103.2851333618164</v>
+      </c>
+      <c r="K241">
+        <v>18256.34375</v>
+      </c>
+      <c r="L241">
+        <v>20857.16015625</v>
+      </c>
+      <c r="M241">
+        <v>22831.712890625</v>
+      </c>
+      <c r="N241">
+        <v>0.914203405380249</v>
+      </c>
+      <c r="O241">
+        <v>0.8655069470405579</v>
+      </c>
+      <c r="P241">
+        <v>0.9276080131530762</v>
+      </c>
+      <c r="Q241">
+        <v>61945.21484375</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B242" t="str">
+        <v>10:36:39 ч.</v>
+      </c>
+      <c r="C242" t="str">
+        <v>HOMO UHT</v>
+      </c>
+      <c r="D242">
+        <v>1828.1005323374543</v>
+      </c>
+      <c r="E242">
+        <v>234.90895080566406</v>
+      </c>
+      <c r="F242">
+        <v>235.7686767578125</v>
+      </c>
+      <c r="G242">
+        <v>237.26022338867188</v>
+      </c>
+      <c r="H242">
+        <v>0.2153719961643219</v>
+      </c>
+      <c r="I242">
+        <v>0.1194046288728714</v>
+      </c>
+      <c r="J242">
+        <v>0.19515810906887054</v>
+      </c>
+      <c r="K242">
+        <v>34.553226470947266</v>
+      </c>
+      <c r="L242">
+        <v>15.887799263000488</v>
+      </c>
+      <c r="M242">
+        <v>15.2201509475708</v>
+      </c>
+      <c r="N242">
+        <v>0.6558202505111694</v>
+      </c>
+      <c r="O242">
+        <v>0.5642855763435364</v>
+      </c>
+      <c r="P242">
+        <v>0.3286544382572174</v>
+      </c>
+      <c r="Q242">
+        <v>65.66117858886719</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B243" t="str">
+        <v>10:36:39 ч.</v>
+      </c>
+      <c r="C243" t="str">
+        <v>Priem KM</v>
+      </c>
+      <c r="D243">
+        <v>5580.07298292129</v>
+      </c>
+      <c r="E243">
+        <v>234.90077209472656</v>
+      </c>
+      <c r="F243">
+        <v>235.81698608398438</v>
+      </c>
+      <c r="G243">
+        <v>237.5458526611328</v>
+      </c>
+      <c r="H243">
+        <v>39.33921813964844</v>
+      </c>
+      <c r="I243">
+        <v>37.11605453491211</v>
+      </c>
+      <c r="J243">
+        <v>41.222312927246094</v>
+      </c>
+      <c r="K243">
+        <v>3327.426513671875</v>
+      </c>
+      <c r="L243">
+        <v>3734.04345703125</v>
+      </c>
+      <c r="M243">
+        <v>3515.120849609375</v>
+      </c>
+      <c r="N243">
+        <v>0.36007943749427795</v>
+      </c>
+      <c r="O243">
+        <v>0.4266212284564972</v>
+      </c>
+      <c r="P243">
+        <v>0.36152470111846924</v>
+      </c>
+      <c r="Q243">
+        <v>10617.125</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B244" t="str">
+        <v>10:36:39 ч.</v>
+      </c>
+      <c r="C244" t="str">
+        <v>Priem UHT</v>
+      </c>
+      <c r="D244">
+        <v>866.5699943788928</v>
+      </c>
+      <c r="E244">
+        <v>234.90170288085938</v>
+      </c>
+      <c r="F244">
+        <v>235.588134765625</v>
+      </c>
+      <c r="G244">
+        <v>237.39480590820312</v>
+      </c>
+      <c r="H244">
+        <v>0.9115591645240784</v>
+      </c>
+      <c r="I244">
+        <v>0.5165048241615295</v>
+      </c>
+      <c r="J244">
+        <v>0.8178279399871826</v>
+      </c>
+      <c r="K244">
+        <v>113.85226440429688</v>
+      </c>
+      <c r="L244">
+        <v>85.16337585449219</v>
+      </c>
+      <c r="M244">
+        <v>59.22567367553711</v>
+      </c>
+      <c r="N244">
+        <v>0.531696617603302</v>
+      </c>
+      <c r="O244">
+        <v>0.6999155282974243</v>
+      </c>
+      <c r="P244">
+        <v>0.30505409836769104</v>
+      </c>
+      <c r="Q244">
+        <v>258.2413024902344</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B245" t="str">
+        <v>10:37:16 ч.</v>
+      </c>
+      <c r="C245" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D245">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B246" t="str">
+        <v>10:40:06 ч.</v>
+      </c>
+      <c r="C246" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D246">
+        <v>139039.21953906835</v>
+      </c>
+      <c r="E246">
+        <v>233.3984375</v>
+      </c>
+      <c r="F246">
+        <v>232.98348999023438</v>
+      </c>
+      <c r="G246">
+        <v>236.0981903076172</v>
+      </c>
+      <c r="H246">
+        <v>1.5928025245666504</v>
+      </c>
+      <c r="I246">
+        <v>1.636141300201416</v>
+      </c>
+      <c r="J246">
+        <v>1.4666978120803833</v>
+      </c>
+      <c r="K246">
+        <v>266.66033935546875</v>
+      </c>
+      <c r="L246">
+        <v>200.92941284179688</v>
+      </c>
+      <c r="M246">
+        <v>212.55870056152344</v>
+      </c>
+      <c r="N246">
+        <v>0.7175413966178894</v>
+      </c>
+      <c r="O246">
+        <v>0.5250428915023804</v>
+      </c>
+      <c r="P246">
+        <v>0.6168241500854492</v>
+      </c>
+      <c r="Q246">
+        <v>680.1857299804688</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B247" t="str">
+        <v>10:40:06 ч.</v>
+      </c>
+      <c r="C247" t="str">
+        <v>Ampak</v>
+      </c>
+      <c r="D247">
+        <v>41479.559280142</v>
+      </c>
+      <c r="E247">
+        <v>233.59837341308594</v>
+      </c>
+      <c r="F247">
+        <v>233.46913146972656</v>
+      </c>
+      <c r="G247">
+        <v>235.89109802246094</v>
+      </c>
+      <c r="H247">
+        <v>42.30766296386719</v>
+      </c>
+      <c r="I247">
+        <v>46.07231140136719</v>
+      </c>
+      <c r="J247">
+        <v>39.83202362060547</v>
+      </c>
+      <c r="K247">
+        <v>8531.4169921875</v>
+      </c>
+      <c r="L247">
+        <v>9341.9169921875</v>
+      </c>
+      <c r="M247">
+        <v>8105.962890625</v>
+      </c>
+      <c r="N247">
+        <v>0.8632415533065796</v>
+      </c>
+      <c r="O247">
+        <v>0.868493378162384</v>
+      </c>
+      <c r="P247">
+        <v>0.8627017736434937</v>
+      </c>
+      <c r="Q247">
+        <v>25979.296875</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B248" t="str">
+        <v>10:40:06 ч.</v>
+      </c>
+      <c r="C248" t="str">
+        <v>Ledena Voda</v>
+      </c>
+      <c r="D248">
+        <v>246438.74927397812</v>
+      </c>
+      <c r="E248">
+        <v>236.27552795410156</v>
+      </c>
+      <c r="F248">
+        <v>236.4452667236328</v>
+      </c>
+      <c r="G248">
+        <v>238.18743896484375</v>
+      </c>
+      <c r="H248">
+        <v>6.601243495941162</v>
+      </c>
+      <c r="I248">
+        <v>6.490886688232422</v>
+      </c>
+      <c r="J248">
+        <v>6.572907447814941</v>
+      </c>
+      <c r="K248">
+        <v>1029.936767578125</v>
+      </c>
+      <c r="L248">
+        <v>1003.357177734375</v>
+      </c>
+      <c r="M248">
+        <v>1071.09326171875</v>
+      </c>
+      <c r="N248">
+        <v>0.6603376269340515</v>
+      </c>
+      <c r="O248">
+        <v>0.6532604694366455</v>
+      </c>
+      <c r="P248">
+        <v>0.6847626566886902</v>
+      </c>
+      <c r="Q248">
+        <v>3100.60302734375</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B249" t="str">
+        <v>10:40:06 ч.</v>
+      </c>
+      <c r="C249" t="str">
+        <v>Hladilnici</v>
+      </c>
+      <c r="D249">
+        <v>181741.4113652791</v>
+      </c>
+      <c r="E249">
+        <v>237.81272888183594</v>
+      </c>
+      <c r="F249">
+        <v>235.93658447265625</v>
+      </c>
+      <c r="G249">
+        <v>235.9821319580078</v>
+      </c>
+      <c r="H249">
+        <v>8.606767654418945</v>
+      </c>
+      <c r="I249">
+        <v>8.861143112182617</v>
+      </c>
+      <c r="J249">
+        <v>10.758027076721191</v>
+      </c>
+      <c r="K249">
+        <v>1735.0068359375</v>
+      </c>
+      <c r="L249">
+        <v>1746.144287109375</v>
+      </c>
+      <c r="M249">
+        <v>2372.95849609375</v>
+      </c>
+      <c r="N249">
+        <v>0.847884476184845</v>
+      </c>
+      <c r="O249">
+        <v>0.8344557881355286</v>
+      </c>
+      <c r="P249">
+        <v>0.934815526008606</v>
+      </c>
+      <c r="Q249">
+        <v>5846.275390625</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B250" t="str">
+        <v>10:40:06 ч.</v>
+      </c>
+      <c r="C250" t="str">
+        <v>Kompresorno</v>
+      </c>
+      <c r="D250">
+        <v>49922.51549228285</v>
+      </c>
+      <c r="E250">
+        <v>236.3805694580078</v>
+      </c>
+      <c r="F250">
+        <v>234.0081329345703</v>
+      </c>
+      <c r="G250">
+        <v>233.28976440429688</v>
+      </c>
+      <c r="H250">
+        <v>48.22032165527344</v>
+      </c>
+      <c r="I250">
+        <v>39.3026123046875</v>
+      </c>
+      <c r="J250">
+        <v>43.78318405151367</v>
+      </c>
+      <c r="K250">
+        <v>9540.3798828125</v>
+      </c>
+      <c r="L250">
+        <v>7482.3466796875</v>
+      </c>
+      <c r="M250">
+        <v>7730.890625</v>
+      </c>
+      <c r="N250">
+        <v>0.838183581829071</v>
+      </c>
+      <c r="O250">
+        <v>0.8139026165008545</v>
+      </c>
+      <c r="P250">
+        <v>0.7529270648956299</v>
+      </c>
+      <c r="Q250">
+        <v>24931.375</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B251" t="str">
+        <v>10:40:06 ч.</v>
+      </c>
+      <c r="C251" t="str">
+        <v>Priemno</v>
+      </c>
+      <c r="D251">
+        <v>59442.433150150646</v>
+      </c>
+      <c r="E251">
+        <v>235.05711364746094</v>
+      </c>
+      <c r="F251">
+        <v>235.76011657714844</v>
+      </c>
+      <c r="G251">
+        <v>237.53005981445312</v>
+      </c>
+      <c r="H251">
+        <v>69.62702941894531</v>
+      </c>
+      <c r="I251">
+        <v>60.997032165527344</v>
+      </c>
+      <c r="J251">
+        <v>64.01730346679688</v>
+      </c>
+      <c r="K251">
+        <v>11871.80859375</v>
+      </c>
+      <c r="L251">
+        <v>10214.494140625</v>
+      </c>
+      <c r="M251">
+        <v>10277.4755859375</v>
+      </c>
+      <c r="N251">
+        <v>0.7263919115066528</v>
+      </c>
+      <c r="O251">
+        <v>0.70912766456604</v>
+      </c>
+      <c r="P251">
+        <v>0.6770891547203064</v>
+      </c>
+      <c r="Q251">
+        <v>32379.08984375</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B252" t="str">
+        <v>10:40:06 ч.</v>
+      </c>
+      <c r="C252" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="D252">
+        <v>239047.38078830557</v>
+      </c>
+      <c r="E252">
+        <v>235.69537353515625</v>
+      </c>
+      <c r="F252">
+        <v>235.85118103027344</v>
+      </c>
+      <c r="G252">
+        <v>238.41787719726562</v>
+      </c>
+      <c r="H252">
+        <v>79.81590270996094</v>
+      </c>
+      <c r="I252">
+        <v>100.24121856689453</v>
+      </c>
+      <c r="J252">
+        <v>96.10077667236328</v>
+      </c>
+      <c r="K252">
+        <v>16435.94140625</v>
+      </c>
+      <c r="L252">
+        <v>19532.919921875</v>
+      </c>
+      <c r="M252">
+        <v>20339.583984375</v>
+      </c>
+      <c r="N252">
+        <v>0.8736834526062012</v>
+      </c>
+      <c r="O252">
+        <v>0.8261954188346863</v>
+      </c>
+      <c r="P252">
+        <v>0.8877207040786743</v>
+      </c>
+      <c r="Q252">
+        <v>56308.4453125</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B253" t="str">
+        <v>10:40:06 ч.</v>
+      </c>
+      <c r="C253" t="str">
+        <v>HOMO UHT</v>
+      </c>
+      <c r="D253">
+        <v>1828.1042844567999</v>
+      </c>
+      <c r="E253">
+        <v>235.05369567871094</v>
+      </c>
+      <c r="F253">
+        <v>235.89712524414062</v>
+      </c>
+      <c r="G253">
+        <v>237.2433319091797</v>
+      </c>
+      <c r="H253">
+        <v>0.23187346756458282</v>
+      </c>
+      <c r="I253">
+        <v>0.1136220246553421</v>
+      </c>
+      <c r="J253">
+        <v>0.20436441898345947</v>
+      </c>
+      <c r="K253">
+        <v>35.465572357177734</v>
+      </c>
+      <c r="L253">
+        <v>15.012643814086914</v>
+      </c>
+      <c r="M253">
+        <v>14.915885925292969</v>
+      </c>
+      <c r="N253">
+        <v>0.6507120132446289</v>
+      </c>
+      <c r="O253">
+        <v>0.5601083040237427</v>
+      </c>
+      <c r="P253">
+        <v>0.30764490365982056</v>
+      </c>
+      <c r="Q253">
+        <v>65.39410400390625</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B254" t="str">
+        <v>10:40:06 ч.</v>
+      </c>
+      <c r="C254" t="str">
+        <v>Priem KM</v>
+      </c>
+      <c r="D254">
+        <v>5580.689465321469</v>
+      </c>
+      <c r="E254">
+        <v>234.9888153076172</v>
+      </c>
+      <c r="F254">
+        <v>235.89231872558594</v>
+      </c>
+      <c r="G254">
+        <v>237.43502807617188</v>
+      </c>
+      <c r="H254">
+        <v>39.812618255615234</v>
+      </c>
+      <c r="I254">
+        <v>37.558006286621094</v>
+      </c>
+      <c r="J254">
+        <v>41.42351531982422</v>
+      </c>
+      <c r="K254">
+        <v>3553.279052734375</v>
+      </c>
+      <c r="L254">
+        <v>3911.94970703125</v>
+      </c>
+      <c r="M254">
+        <v>3717.763916015625</v>
+      </c>
+      <c r="N254">
+        <v>0.38154739141464233</v>
+      </c>
+      <c r="O254">
+        <v>0.4419892430305481</v>
+      </c>
+      <c r="P254">
+        <v>0.378376841545105</v>
+      </c>
+      <c r="Q254">
+        <v>11194.419921875</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B255" t="str">
+        <v>10:40:06 ч.</v>
+      </c>
+      <c r="C255" t="str">
+        <v>Priem UHT</v>
+      </c>
+      <c r="D255">
+        <v>866.5849196988066</v>
+      </c>
+      <c r="E255">
+        <v>234.8663330078125</v>
+      </c>
+      <c r="F255">
+        <v>235.5184326171875</v>
+      </c>
+      <c r="G255">
+        <v>237.2134246826172</v>
+      </c>
+      <c r="H255">
+        <v>0.92148357629776</v>
+      </c>
+      <c r="I255">
+        <v>0.4984115958213806</v>
+      </c>
+      <c r="J255">
+        <v>0.8426135778427124</v>
+      </c>
+      <c r="K255">
+        <v>117.85088348388672</v>
+      </c>
+      <c r="L255">
+        <v>82.02877044677734</v>
+      </c>
+      <c r="M255">
+        <v>60.03065490722656</v>
+      </c>
+      <c r="N255">
+        <v>0.544533371925354</v>
+      </c>
+      <c r="O255">
+        <v>0.6988005042076111</v>
+      </c>
+      <c r="P255">
+        <v>0.3003346025943756</v>
+      </c>
+      <c r="Q255">
+        <v>259.9103088378906</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B256" t="str">
+        <v>10:42:19 ч.</v>
+      </c>
+      <c r="C256" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D256">
+        <v>139039.2416039878</v>
+      </c>
+      <c r="E256">
+        <v>233.66790771484375</v>
+      </c>
+      <c r="F256">
+        <v>233.67189025878906</v>
+      </c>
+      <c r="G256">
+        <v>235.8277587890625</v>
+      </c>
+      <c r="H256">
+        <v>1.6152212619781494</v>
+      </c>
+      <c r="I256">
+        <v>1.6485873460769653</v>
+      </c>
+      <c r="J256">
+        <v>1.4700380563735962</v>
+      </c>
+      <c r="K256">
+        <v>268.3112487792969</v>
+      </c>
+      <c r="L256">
+        <v>200.69500732421875</v>
+      </c>
+      <c r="M256">
+        <v>213.32484436035156</v>
+      </c>
+      <c r="N256">
+        <v>0.7102516293525696</v>
+      </c>
+      <c r="O256">
+        <v>0.5196358561515808</v>
+      </c>
+      <c r="P256">
+        <v>0.6127038598060608</v>
+      </c>
+      <c r="Q256">
+        <v>679.697265625</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B257" t="str">
+        <v>10:42:19 ч.</v>
+      </c>
+      <c r="C257" t="str">
+        <v>Ampak</v>
+      </c>
+      <c r="D257">
+        <v>41480.31198649042</v>
+      </c>
+      <c r="E257">
+        <v>233.09861755371094</v>
+      </c>
+      <c r="F257">
+        <v>232.8889923095703</v>
+      </c>
+      <c r="G257">
+        <v>236.04319763183594</v>
+      </c>
+      <c r="H257">
+        <v>58.06642150878906</v>
+      </c>
+      <c r="I257">
+        <v>62.37663650512695</v>
+      </c>
+      <c r="J257">
+        <v>53.37752914428711</v>
+      </c>
+      <c r="K257">
+        <v>13769.0478515625</v>
+      </c>
+      <c r="L257">
+        <v>14078.1552734375</v>
+      </c>
+      <c r="M257">
+        <v>12282.9453125</v>
+      </c>
+      <c r="N257">
+        <v>0.9728079438209534</v>
+      </c>
+      <c r="O257">
+        <v>0.9693692326545715</v>
+      </c>
+      <c r="P257">
+        <v>0.9749309420585632</v>
+      </c>
+      <c r="Q257">
+        <v>40130.1484375</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B258" t="str">
+        <v>10:42:19 ч.</v>
+      </c>
+      <c r="C258" t="str">
+        <v>Ledena Voda</v>
+      </c>
+      <c r="D258">
+        <v>246438.85760605687</v>
+      </c>
+      <c r="E258">
+        <v>236.17449951171875</v>
+      </c>
+      <c r="F258">
+        <v>236.24488830566406</v>
+      </c>
+      <c r="G258">
+        <v>238.0792236328125</v>
+      </c>
+      <c r="H258">
+        <v>6.392311096191406</v>
+      </c>
+      <c r="I258">
+        <v>6.226422309875488</v>
+      </c>
+      <c r="J258">
+        <v>6.3013763427734375</v>
+      </c>
+      <c r="K258">
+        <v>959.7203369140625</v>
+      </c>
+      <c r="L258">
+        <v>919.449951171875</v>
+      </c>
+      <c r="M258">
+        <v>995.5667114257812</v>
+      </c>
+      <c r="N258">
+        <v>0.6361486911773682</v>
+      </c>
+      <c r="O258">
+        <v>0.6247012615203857</v>
+      </c>
+      <c r="P258">
+        <v>0.6638752818107605</v>
+      </c>
+      <c r="Q258">
+        <v>2874.73681640625</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B259" t="str">
+        <v>10:42:19 ч.</v>
+      </c>
+      <c r="C259" t="str">
+        <v>Hladilnici</v>
+      </c>
+      <c r="D259">
+        <v>181741.69395736887</v>
+      </c>
+      <c r="E259">
+        <v>237.36343383789062</v>
+      </c>
+      <c r="F259">
+        <v>235.7263946533203</v>
+      </c>
+      <c r="G259">
+        <v>235.5079345703125</v>
+      </c>
+      <c r="H259">
+        <v>37.78755569458008</v>
+      </c>
+      <c r="I259">
+        <v>35.43948745727539</v>
+      </c>
+      <c r="J259">
+        <v>36.37275695800781</v>
+      </c>
+      <c r="K259">
+        <v>5811.4619140625</v>
+      </c>
+      <c r="L259">
+        <v>5267.60546875</v>
+      </c>
+      <c r="M259">
+        <v>6310.4208984375</v>
+      </c>
+      <c r="N259">
+        <v>0.6479220986366272</v>
+      </c>
+      <c r="O259">
+        <v>0.6316612958908081</v>
+      </c>
+      <c r="P259">
+        <v>0.7371790409088135</v>
+      </c>
+      <c r="Q259">
+        <v>17397.77734375</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B260" t="str">
+        <v>10:42:19 ч.</v>
+      </c>
+      <c r="C260" t="str">
+        <v>Kompresorno</v>
+      </c>
+      <c r="D260">
+        <v>49923.41327435277</v>
+      </c>
+      <c r="E260">
+        <v>236.2966766357422</v>
+      </c>
+      <c r="F260">
+        <v>233.68524169921875</v>
+      </c>
+      <c r="G260">
+        <v>233.23825073242188</v>
+      </c>
+      <c r="H260">
+        <v>47.649959564208984</v>
+      </c>
+      <c r="I260">
+        <v>38.32468032836914</v>
+      </c>
+      <c r="J260">
+        <v>43.42443084716797</v>
+      </c>
+      <c r="K260">
+        <v>9399.9755859375</v>
+      </c>
+      <c r="L260">
+        <v>7257.95947265625</v>
+      </c>
+      <c r="M260">
+        <v>7584.7021484375</v>
+      </c>
+      <c r="N260">
+        <v>0.8348463773727417</v>
+      </c>
+      <c r="O260">
+        <v>0.8104098439216614</v>
+      </c>
+      <c r="P260">
+        <v>0.748866856098175</v>
+      </c>
+      <c r="Q260">
+        <v>24242.63671875</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B261" t="str">
+        <v>10:42:19 ч.</v>
+      </c>
+      <c r="C261" t="str">
+        <v>Priemno</v>
+      </c>
+      <c r="D261">
+        <v>59443.47519487082</v>
+      </c>
+      <c r="E261">
+        <v>234.9561309814453</v>
+      </c>
+      <c r="F261">
+        <v>235.4727325439453</v>
+      </c>
+      <c r="G261">
+        <v>237.30160522460938</v>
+      </c>
+      <c r="H261">
+        <v>62.35581588745117</v>
+      </c>
+      <c r="I261">
+        <v>51.24052047729492</v>
+      </c>
+      <c r="J261">
+        <v>53.6710205078125</v>
+      </c>
+      <c r="K261">
+        <v>10492.78515625</v>
+      </c>
+      <c r="L261">
+        <v>8006.91015625</v>
+      </c>
+      <c r="M261">
+        <v>8543.7158203125</v>
+      </c>
+      <c r="N261">
+        <v>0.7156137228012085</v>
+      </c>
+      <c r="O261">
+        <v>0.6635313034057617</v>
+      </c>
+      <c r="P261">
+        <v>0.6706818342208862</v>
+      </c>
+      <c r="Q261">
+        <v>27043.41015625</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B262" t="str">
+        <v>10:42:19 ч.</v>
+      </c>
+      <c r="C262" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="D262">
+        <v>239049.39777456457</v>
+      </c>
+      <c r="E262">
+        <v>235.39572143554688</v>
+      </c>
+      <c r="F262">
+        <v>235.73057556152344</v>
+      </c>
+      <c r="G262">
+        <v>238.2235107421875</v>
+      </c>
+      <c r="H262">
+        <v>83.26937866210938</v>
+      </c>
+      <c r="I262">
+        <v>105.8582992553711</v>
+      </c>
+      <c r="J262">
+        <v>102.15914154052734</v>
+      </c>
+      <c r="K262">
+        <v>16405.021484375</v>
+      </c>
+      <c r="L262">
+        <v>19721.283203125</v>
+      </c>
+      <c r="M262">
+        <v>21094.970703125</v>
+      </c>
+      <c r="N262">
+        <v>0.8369298577308655</v>
+      </c>
+      <c r="O262">
+        <v>0.7902686595916748</v>
+      </c>
+      <c r="P262">
+        <v>0.8667963743209839</v>
+      </c>
+      <c r="Q262">
+        <v>57221.27734375</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B263" t="str">
+        <v>10:42:19 ч.</v>
+      </c>
+      <c r="C263" t="str">
+        <v>HOMO UHT</v>
+      </c>
+      <c r="D263">
+        <v>1828.106687428456</v>
+      </c>
+      <c r="E263">
+        <v>234.99363708496094</v>
+      </c>
+      <c r="F263">
+        <v>235.6663360595703</v>
+      </c>
+      <c r="G263">
+        <v>237.1929168701172</v>
+      </c>
+      <c r="H263">
+        <v>0.24891191720962524</v>
+      </c>
+      <c r="I263">
+        <v>0.11104363948106766</v>
+      </c>
+      <c r="J263">
+        <v>0.22210776805877686</v>
+      </c>
+      <c r="K263">
+        <v>36.57011413574219</v>
+      </c>
+      <c r="L263">
+        <v>14.436485290527344</v>
+      </c>
+      <c r="M263">
+        <v>15.20820140838623</v>
+      </c>
+      <c r="N263">
+        <v>0.6248331665992737</v>
+      </c>
+      <c r="O263">
+        <v>0.5537427067756653</v>
+      </c>
+      <c r="P263">
+        <v>0.2938750386238098</v>
+      </c>
+      <c r="Q263">
+        <v>66.68893432617188</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B264" t="str">
+        <v>10:42:19 ч.</v>
+      </c>
+      <c r="C264" t="str">
+        <v>Priem KM</v>
+      </c>
+      <c r="D264">
+        <v>5581.1005204957</v>
+      </c>
+      <c r="E264">
+        <v>235.07916259765625</v>
+      </c>
+      <c r="F264">
+        <v>235.78253173828125</v>
+      </c>
+      <c r="G264">
+        <v>237.52073669433594</v>
+      </c>
+      <c r="H264">
+        <v>37.99555969238281</v>
+      </c>
+      <c r="I264">
+        <v>35.21348190307617</v>
+      </c>
+      <c r="J264">
+        <v>39.30424118041992</v>
+      </c>
+      <c r="K264">
+        <v>3117.142333984375</v>
+      </c>
+      <c r="L264">
+        <v>3366.38037109375</v>
+      </c>
+      <c r="M264">
+        <v>3302.292236328125</v>
+      </c>
+      <c r="N264">
+        <v>0.3463674783706665</v>
+      </c>
+      <c r="O264">
+        <v>0.40639469027519226</v>
+      </c>
+      <c r="P264">
+        <v>0.3542511761188507</v>
+      </c>
+      <c r="Q264">
+        <v>9763.5498046875</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B265" t="str">
+        <v>10:42:19 ч.</v>
+      </c>
+      <c r="C265" t="str">
+        <v>Priem UHT</v>
+      </c>
+      <c r="D265">
+        <v>866.5944535094632</v>
+      </c>
+      <c r="E265">
+        <v>235.08645629882812</v>
+      </c>
+      <c r="F265">
+        <v>235.56980895996094</v>
+      </c>
+      <c r="G265">
+        <v>237.42970275878906</v>
+      </c>
+      <c r="H265">
+        <v>0.923805296421051</v>
+      </c>
+      <c r="I265">
+        <v>0.49449265003204346</v>
+      </c>
+      <c r="J265">
+        <v>0.8477269411087036</v>
+      </c>
+      <c r="K265">
+        <v>117.94815826416016</v>
+      </c>
+      <c r="L265">
+        <v>81.07422637939453</v>
+      </c>
+      <c r="M265">
+        <v>59.32134246826172</v>
+      </c>
+      <c r="N265">
+        <v>0.5430070161819458</v>
+      </c>
+      <c r="O265">
+        <v>0.6964125633239746</v>
+      </c>
+      <c r="P265">
+        <v>0.2948538661003113</v>
+      </c>
+      <c r="Q265">
+        <v>258.34375</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q204"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q265"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
removed debuging console logs
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -992,7 +992,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q265"/>
+  <dimension ref="A1:Q276"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -15000,9 +15000,553 @@
         <v>258.34375</v>
       </c>
     </row>
+    <row r="266">
+      <c r="A266" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B266" t="str">
+        <v>11:16:57 ч.</v>
+      </c>
+      <c r="C266" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D266">
+        <v>139039.63744753267</v>
+      </c>
+      <c r="E266">
+        <v>234.0052947998047</v>
+      </c>
+      <c r="F266">
+        <v>233.3585205078125</v>
+      </c>
+      <c r="G266">
+        <v>236.10458374023438</v>
+      </c>
+      <c r="H266">
+        <v>1.6104230880737305</v>
+      </c>
+      <c r="I266">
+        <v>1.6447467803955078</v>
+      </c>
+      <c r="J266">
+        <v>1.4871313571929932</v>
+      </c>
+      <c r="K266">
+        <v>266.9630126953125</v>
+      </c>
+      <c r="L266">
+        <v>200.22129821777344</v>
+      </c>
+      <c r="M266">
+        <v>214.94773864746094</v>
+      </c>
+      <c r="N266">
+        <v>0.7092186212539673</v>
+      </c>
+      <c r="O266">
+        <v>0.5215973854064941</v>
+      </c>
+      <c r="P266">
+        <v>0.6117419004440308</v>
+      </c>
+      <c r="Q266">
+        <v>681.9057006835938</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B267" t="str">
+        <v>11:16:57 ч.</v>
+      </c>
+      <c r="C267" t="str">
+        <v>Ampak</v>
+      </c>
+      <c r="D267">
+        <v>41492.07184351986</v>
+      </c>
+      <c r="E267">
+        <v>233.51150512695312</v>
+      </c>
+      <c r="F267">
+        <v>232.83648681640625</v>
+      </c>
+      <c r="G267">
+        <v>236.0041046142578</v>
+      </c>
+      <c r="H267">
+        <v>50.05978012084961</v>
+      </c>
+      <c r="I267">
+        <v>52.341590881347656</v>
+      </c>
+      <c r="J267">
+        <v>44.68852615356445</v>
+      </c>
+      <c r="K267">
+        <v>10699.23828125</v>
+      </c>
+      <c r="L267">
+        <v>12327.1396484375</v>
+      </c>
+      <c r="M267">
+        <v>12122.505859375</v>
+      </c>
+      <c r="N267">
+        <v>0.9751510620117188</v>
+      </c>
+      <c r="O267">
+        <v>0.9646387100219727</v>
+      </c>
+      <c r="P267">
+        <v>0.9787526726722717</v>
+      </c>
+      <c r="Q267">
+        <v>37535.23828125</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B268" t="str">
+        <v>11:16:57 ч.</v>
+      </c>
+      <c r="C268" t="str">
+        <v>Ledena Voda</v>
+      </c>
+      <c r="D268">
+        <v>246439.25143916663</v>
+      </c>
+      <c r="E268">
+        <v>236.2144317626953</v>
+      </c>
+      <c r="F268">
+        <v>236.34744262695312</v>
+      </c>
+      <c r="G268">
+        <v>238.2026824951172</v>
+      </c>
+      <c r="H268">
+        <v>0.16359001398086548</v>
+      </c>
+      <c r="I268">
+        <v>0.28383511304855347</v>
+      </c>
+      <c r="J268">
+        <v>0.4385814070701599</v>
+      </c>
+      <c r="K268">
+        <v>29.50800132751465</v>
+      </c>
+      <c r="L268">
+        <v>-12.722734451293945</v>
+      </c>
+      <c r="M268">
+        <v>54.65665817260742</v>
+      </c>
+      <c r="N268">
+        <v>0.7636187076568604</v>
+      </c>
+      <c r="O268">
+        <v>0.1896546334028244</v>
+      </c>
+      <c r="P268">
+        <v>0.5194758176803589</v>
+      </c>
+      <c r="Q268">
+        <v>70.94840240478516</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B269" t="str">
+        <v>11:16:57 ч.</v>
+      </c>
+      <c r="C269" t="str">
+        <v>Hladilnici</v>
+      </c>
+      <c r="D269">
+        <v>181751.87124310728</v>
+      </c>
+      <c r="E269">
+        <v>237.23226928710938</v>
+      </c>
+      <c r="F269">
+        <v>235.4815216064453</v>
+      </c>
+      <c r="G269">
+        <v>235.48861694335938</v>
+      </c>
+      <c r="H269">
+        <v>47.897560119628906</v>
+      </c>
+      <c r="I269">
+        <v>44.31301498413086</v>
+      </c>
+      <c r="J269">
+        <v>50.400787353515625</v>
+      </c>
+      <c r="K269">
+        <v>8446.3515625</v>
+      </c>
+      <c r="L269">
+        <v>7618.98388671875</v>
+      </c>
+      <c r="M269">
+        <v>9553.1796875</v>
+      </c>
+      <c r="N269">
+        <v>0.742792546749115</v>
+      </c>
+      <c r="O269">
+        <v>0.7300994992256165</v>
+      </c>
+      <c r="P269">
+        <v>0.8047470450401306</v>
+      </c>
+      <c r="Q269">
+        <v>25618.515625</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B270" t="str">
+        <v>11:16:57 ч.</v>
+      </c>
+      <c r="C270" t="str">
+        <v>Kompresorno</v>
+      </c>
+      <c r="D270">
+        <v>49937.70486535381</v>
+      </c>
+      <c r="E270">
+        <v>236.3603973388672</v>
+      </c>
+      <c r="F270">
+        <v>234.01315307617188</v>
+      </c>
+      <c r="G270">
+        <v>233.09979248046875</v>
+      </c>
+      <c r="H270">
+        <v>49.409820556640625</v>
+      </c>
+      <c r="I270">
+        <v>39.47994613647461</v>
+      </c>
+      <c r="J270">
+        <v>45.09613800048828</v>
+      </c>
+      <c r="K270">
+        <v>9864.9736328125</v>
+      </c>
+      <c r="L270">
+        <v>7514.3408203125</v>
+      </c>
+      <c r="M270">
+        <v>7984.205078125</v>
+      </c>
+      <c r="N270">
+        <v>0.844710648059845</v>
+      </c>
+      <c r="O270">
+        <v>0.8133436441421509</v>
+      </c>
+      <c r="P270">
+        <v>0.7595396637916565</v>
+      </c>
+      <c r="Q270">
+        <v>25363.51953125</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B271" t="str">
+        <v>11:16:57 ч.</v>
+      </c>
+      <c r="C271" t="str">
+        <v>Priemno</v>
+      </c>
+      <c r="D271">
+        <v>59462.14705924951</v>
+      </c>
+      <c r="E271">
+        <v>234.79611206054688</v>
+      </c>
+      <c r="F271">
+        <v>235.6047821044922</v>
+      </c>
+      <c r="G271">
+        <v>237.4341278076172</v>
+      </c>
+      <c r="H271">
+        <v>68.70552062988281</v>
+      </c>
+      <c r="I271">
+        <v>55.061100006103516</v>
+      </c>
+      <c r="J271">
+        <v>58.588356018066406</v>
+      </c>
+      <c r="K271">
+        <v>14775.18359375</v>
+      </c>
+      <c r="L271">
+        <v>11879.611328125</v>
+      </c>
+      <c r="M271">
+        <v>12671.4580078125</v>
+      </c>
+      <c r="N271">
+        <v>0.9159048199653625</v>
+      </c>
+      <c r="O271">
+        <v>0.9154213070869446</v>
+      </c>
+      <c r="P271">
+        <v>0.910574197769165</v>
+      </c>
+      <c r="Q271">
+        <v>39292.79296875</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B272" t="str">
+        <v>11:16:57 ч.</v>
+      </c>
+      <c r="C272" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="D272">
+        <v>239083.8413587807</v>
+      </c>
+      <c r="E272">
+        <v>235.39181518554688</v>
+      </c>
+      <c r="F272">
+        <v>235.55604553222656</v>
+      </c>
+      <c r="G272">
+        <v>238.15274047851562</v>
+      </c>
+      <c r="H272">
+        <v>92.40723419189453</v>
+      </c>
+      <c r="I272">
+        <v>115.35205841064453</v>
+      </c>
+      <c r="J272">
+        <v>103.66046142578125</v>
+      </c>
+      <c r="K272">
+        <v>20089.630859375</v>
+      </c>
+      <c r="L272">
+        <v>23978.34375</v>
+      </c>
+      <c r="M272">
+        <v>23438.96875</v>
+      </c>
+      <c r="N272">
+        <v>0.9212222099304199</v>
+      </c>
+      <c r="O272">
+        <v>0.8883658051490784</v>
+      </c>
+      <c r="P272">
+        <v>0.9333217144012451</v>
+      </c>
+      <c r="Q272">
+        <v>67162.46875</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B273" t="str">
+        <v>11:16:57 ч.</v>
+      </c>
+      <c r="C273" t="str">
+        <v>HOMO UHT</v>
+      </c>
+      <c r="D273">
+        <v>1828.144352605426</v>
+      </c>
+      <c r="E273">
+        <v>234.77073669433594</v>
+      </c>
+      <c r="F273">
+        <v>235.64097595214844</v>
+      </c>
+      <c r="G273">
+        <v>237.18807983398438</v>
+      </c>
+      <c r="H273">
+        <v>0.24272455275058746</v>
+      </c>
+      <c r="I273">
+        <v>0.1157940998673439</v>
+      </c>
+      <c r="J273">
+        <v>0.21509790420532227</v>
+      </c>
+      <c r="K273">
+        <v>35.235694885253906</v>
+      </c>
+      <c r="L273">
+        <v>15.203989028930664</v>
+      </c>
+      <c r="M273">
+        <v>14.895801544189453</v>
+      </c>
+      <c r="N273">
+        <v>0.6183369159698486</v>
+      </c>
+      <c r="O273">
+        <v>0.5572118163108826</v>
+      </c>
+      <c r="P273">
+        <v>0.2919677197933197</v>
+      </c>
+      <c r="Q273">
+        <v>65.35221862792969</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B274" t="str">
+        <v>11:16:57 ч.</v>
+      </c>
+      <c r="C274" t="str">
+        <v>Priem KM</v>
+      </c>
+      <c r="D274">
+        <v>5583.742327712225</v>
+      </c>
+      <c r="E274">
+        <v>234.8002166748047</v>
+      </c>
+      <c r="F274">
+        <v>235.5829315185547</v>
+      </c>
+      <c r="G274">
+        <v>237.3838653564453</v>
+      </c>
+      <c r="H274">
+        <v>4.235062122344971</v>
+      </c>
+      <c r="I274">
+        <v>3.3814265727996826</v>
+      </c>
+      <c r="J274">
+        <v>3.6978399753570557</v>
+      </c>
+      <c r="K274">
+        <v>930.096923828125</v>
+      </c>
+      <c r="L274">
+        <v>753.10595703125</v>
+      </c>
+      <c r="M274">
+        <v>835.5184326171875</v>
+      </c>
+      <c r="N274">
+        <v>0.9351935386657715</v>
+      </c>
+      <c r="O274">
+        <v>0.9433372020721436</v>
+      </c>
+      <c r="P274">
+        <v>0.9489923715591431</v>
+      </c>
+      <c r="Q274">
+        <v>2521.452880859375</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B275" t="str">
+        <v>11:16:57 ч.</v>
+      </c>
+      <c r="C275" t="str">
+        <v>Priem UHT</v>
+      </c>
+      <c r="D275">
+        <v>866.7629464016726</v>
+      </c>
+      <c r="E275">
+        <v>234.94393920898438</v>
+      </c>
+      <c r="F275">
+        <v>235.50057983398438</v>
+      </c>
+      <c r="G275">
+        <v>237.44993591308594</v>
+      </c>
+      <c r="H275">
+        <v>0.9267055988311768</v>
+      </c>
+      <c r="I275">
+        <v>0.5124959945678711</v>
+      </c>
+      <c r="J275">
+        <v>0.8479539155960083</v>
+      </c>
+      <c r="K275">
+        <v>117.0469970703125</v>
+      </c>
+      <c r="L275">
+        <v>82.79336547851562</v>
+      </c>
+      <c r="M275">
+        <v>59.741458892822266</v>
+      </c>
+      <c r="N275">
+        <v>0.5375937819480896</v>
+      </c>
+      <c r="O275">
+        <v>0.6859825253486633</v>
+      </c>
+      <c r="P275">
+        <v>0.2967095375061035</v>
+      </c>
+      <c r="Q275">
+        <v>259.5818176269531</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B276" t="str">
+        <v>11:18:45 ч.</v>
+      </c>
+      <c r="C276" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D276">
+        <v>-1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q265"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q276"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added globas leading spinners
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -992,7 +992,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q276"/>
+  <dimension ref="A1:Q326"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -15544,9 +15544,2659 @@
         <v>-1</v>
       </c>
     </row>
+    <row r="277">
+      <c r="A277" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B277" t="str">
+        <v>11:31:05 ч.</v>
+      </c>
+      <c r="C277" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D277">
+        <v>139039.7978514951</v>
+      </c>
+      <c r="E277">
+        <v>233.73463439941406</v>
+      </c>
+      <c r="F277">
+        <v>233.00213623046875</v>
+      </c>
+      <c r="G277">
+        <v>234.86280822753906</v>
+      </c>
+      <c r="H277">
+        <v>1.627046823501587</v>
+      </c>
+      <c r="I277">
+        <v>1.6590168476104736</v>
+      </c>
+      <c r="J277">
+        <v>1.4618874788284302</v>
+      </c>
+      <c r="K277">
+        <v>271.545166015625</v>
+      </c>
+      <c r="L277">
+        <v>199.2617950439453</v>
+      </c>
+      <c r="M277">
+        <v>208.83255004882812</v>
+      </c>
+      <c r="N277">
+        <v>0.7133756875991821</v>
+      </c>
+      <c r="O277">
+        <v>0.5148011445999146</v>
+      </c>
+      <c r="P277">
+        <v>0.6112751960754395</v>
+      </c>
+      <c r="Q277">
+        <v>681.5712890625</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B278" t="str">
+        <v>11:31:05 ч.</v>
+      </c>
+      <c r="C278" t="str">
+        <v>Ampak</v>
+      </c>
+      <c r="D278">
+        <v>41496.86415191441</v>
+      </c>
+      <c r="E278">
+        <v>233.72946166992188</v>
+      </c>
+      <c r="F278">
+        <v>232.63185119628906</v>
+      </c>
+      <c r="G278">
+        <v>234.86795043945312</v>
+      </c>
+      <c r="H278">
+        <v>32.440650939941406</v>
+      </c>
+      <c r="I278">
+        <v>30.103357315063477</v>
+      </c>
+      <c r="J278">
+        <v>23.819684982299805</v>
+      </c>
+      <c r="K278">
+        <v>6256.59423828125</v>
+      </c>
+      <c r="L278">
+        <v>5885.615234375</v>
+      </c>
+      <c r="M278">
+        <v>4458.1826171875</v>
+      </c>
+      <c r="N278">
+        <v>0.8539040088653564</v>
+      </c>
+      <c r="O278">
+        <v>0.840115487575531</v>
+      </c>
+      <c r="P278">
+        <v>0.7970345616340637</v>
+      </c>
+      <c r="Q278">
+        <v>16600.392578125</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B279" t="str">
+        <v>11:31:05 ч.</v>
+      </c>
+      <c r="C279" t="str">
+        <v>Ledena Voda</v>
+      </c>
+      <c r="D279">
+        <v>246442.2111848997</v>
+      </c>
+      <c r="E279">
+        <v>228.19558715820312</v>
+      </c>
+      <c r="F279">
+        <v>232.5736541748047</v>
+      </c>
+      <c r="G279">
+        <v>232.75286865234375</v>
+      </c>
+      <c r="H279">
+        <v>211.0689697265625</v>
+      </c>
+      <c r="I279">
+        <v>213.8896484375</v>
+      </c>
+      <c r="J279">
+        <v>221.85879516601562</v>
+      </c>
+      <c r="K279">
+        <v>36517.6796875</v>
+      </c>
+      <c r="L279">
+        <v>40642.58203125</v>
+      </c>
+      <c r="M279">
+        <v>39650.30859375</v>
+      </c>
+      <c r="N279">
+        <v>0.7854851484298706</v>
+      </c>
+      <c r="O279">
+        <v>0.8172846436500549</v>
+      </c>
+      <c r="P279">
+        <v>0.7680467367172241</v>
+      </c>
+      <c r="Q279">
+        <v>116810.5625</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B280" t="str">
+        <v>11:31:05 ч.</v>
+      </c>
+      <c r="C280" t="str">
+        <v>Hladilnici</v>
+      </c>
+      <c r="D280">
+        <v>181755.4499857191</v>
+      </c>
+      <c r="E280">
+        <v>236.143310546875</v>
+      </c>
+      <c r="F280">
+        <v>234.62168884277344</v>
+      </c>
+      <c r="G280">
+        <v>234.44187927246094</v>
+      </c>
+      <c r="H280">
+        <v>8.032161712646484</v>
+      </c>
+      <c r="I280">
+        <v>8.874295234680176</v>
+      </c>
+      <c r="J280">
+        <v>10.381035804748535</v>
+      </c>
+      <c r="K280">
+        <v>1545.6712646484375</v>
+      </c>
+      <c r="L280">
+        <v>1741.9249267578125</v>
+      </c>
+      <c r="M280">
+        <v>2232.20263671875</v>
+      </c>
+      <c r="N280">
+        <v>0.8149469494819641</v>
+      </c>
+      <c r="O280">
+        <v>0.8366184234619141</v>
+      </c>
+      <c r="P280">
+        <v>0.9171866774559021</v>
+      </c>
+      <c r="Q280">
+        <v>5519.798828125</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B281" t="str">
+        <v>11:31:05 ч.</v>
+      </c>
+      <c r="C281" t="str">
+        <v>Kompresorno</v>
+      </c>
+      <c r="D281">
+        <v>49943.64729386495</v>
+      </c>
+      <c r="E281">
+        <v>234.4947967529297</v>
+      </c>
+      <c r="F281">
+        <v>234.22457885742188</v>
+      </c>
+      <c r="G281">
+        <v>232.3428955078125</v>
+      </c>
+      <c r="H281">
+        <v>44.509525299072266</v>
+      </c>
+      <c r="I281">
+        <v>45.03188705444336</v>
+      </c>
+      <c r="J281">
+        <v>42.241512298583984</v>
+      </c>
+      <c r="K281">
+        <v>8283.171875</v>
+      </c>
+      <c r="L281">
+        <v>8706.7978515625</v>
+      </c>
+      <c r="M281">
+        <v>7879.78466796875</v>
+      </c>
+      <c r="N281">
+        <v>0.7936161756515503</v>
+      </c>
+      <c r="O281">
+        <v>0.8254786729812622</v>
+      </c>
+      <c r="P281">
+        <v>0.802870512008667</v>
+      </c>
+      <c r="Q281">
+        <v>24919.267578125</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B282" t="str">
+        <v>11:31:05 ч.</v>
+      </c>
+      <c r="C282" t="str">
+        <v>Priemno</v>
+      </c>
+      <c r="D282">
+        <v>59470.85422640192</v>
+      </c>
+      <c r="E282">
+        <v>233.7315673828125</v>
+      </c>
+      <c r="F282">
+        <v>234.4432830810547</v>
+      </c>
+      <c r="G282">
+        <v>236.00970458984375</v>
+      </c>
+      <c r="H282">
+        <v>65.40093994140625</v>
+      </c>
+      <c r="I282">
+        <v>52.585426330566406</v>
+      </c>
+      <c r="J282">
+        <v>55.24220657348633</v>
+      </c>
+      <c r="K282">
+        <v>14128.537109375</v>
+      </c>
+      <c r="L282">
+        <v>11179.4775390625</v>
+      </c>
+      <c r="M282">
+        <v>11849.71484375</v>
+      </c>
+      <c r="N282">
+        <v>0.9282891750335693</v>
+      </c>
+      <c r="O282">
+        <v>0.9070557951927185</v>
+      </c>
+      <c r="P282">
+        <v>0.908933699131012</v>
+      </c>
+      <c r="Q282">
+        <v>37157.7265625</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B283" t="str">
+        <v>11:31:05 ч.</v>
+      </c>
+      <c r="C283" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="D283">
+        <v>239099.7376751426</v>
+      </c>
+      <c r="E283">
+        <v>234.06004333496094</v>
+      </c>
+      <c r="F283">
+        <v>234.62350463867188</v>
+      </c>
+      <c r="G283">
+        <v>236.76812744140625</v>
+      </c>
+      <c r="H283">
+        <v>189.80886840820312</v>
+      </c>
+      <c r="I283">
+        <v>193.47756958007812</v>
+      </c>
+      <c r="J283">
+        <v>192.2771759033203</v>
+      </c>
+      <c r="K283">
+        <v>38551.3125</v>
+      </c>
+      <c r="L283">
+        <v>38834.02734375</v>
+      </c>
+      <c r="M283">
+        <v>39483.17578125</v>
+      </c>
+      <c r="N283">
+        <v>0.8677289485931396</v>
+      </c>
+      <c r="O283">
+        <v>0.8552947044372559</v>
+      </c>
+      <c r="P283">
+        <v>0.8672835826873779</v>
+      </c>
+      <c r="Q283">
+        <v>116868.515625</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B284" t="str">
+        <v>11:31:05 ч.</v>
+      </c>
+      <c r="C284" t="str">
+        <v>HOMO UHT</v>
+      </c>
+      <c r="D284">
+        <v>1828.1597032248771</v>
+      </c>
+      <c r="E284">
+        <v>233.7738800048828</v>
+      </c>
+      <c r="F284">
+        <v>234.73841857910156</v>
+      </c>
+      <c r="G284">
+        <v>235.9399871826172</v>
+      </c>
+      <c r="H284">
+        <v>0.2622023820877075</v>
+      </c>
+      <c r="I284">
+        <v>0.10924334824085236</v>
+      </c>
+      <c r="J284">
+        <v>0.2356082946062088</v>
+      </c>
+      <c r="K284">
+        <v>36.38713073730469</v>
+      </c>
+      <c r="L284">
+        <v>13.918783187866211</v>
+      </c>
+      <c r="M284">
+        <v>14.813091278076172</v>
+      </c>
+      <c r="N284">
+        <v>0.5910863280296326</v>
+      </c>
+      <c r="O284">
+        <v>0.544315755367279</v>
+      </c>
+      <c r="P284">
+        <v>0.26726508140563965</v>
+      </c>
+      <c r="Q284">
+        <v>64.8245620727539</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B285" t="str">
+        <v>11:31:05 ч.</v>
+      </c>
+      <c r="C285" t="str">
+        <v>Priem KM</v>
+      </c>
+      <c r="D285">
+        <v>5584.372263926307</v>
+      </c>
+      <c r="E285">
+        <v>233.81314086914062</v>
+      </c>
+      <c r="F285">
+        <v>234.73146057128906</v>
+      </c>
+      <c r="G285">
+        <v>236.09176635742188</v>
+      </c>
+      <c r="H285">
+        <v>4.115927696228027</v>
+      </c>
+      <c r="I285">
+        <v>3.1616854667663574</v>
+      </c>
+      <c r="J285">
+        <v>3.4296419620513916</v>
+      </c>
+      <c r="K285">
+        <v>902.0286865234375</v>
+      </c>
+      <c r="L285">
+        <v>692.7800903320312</v>
+      </c>
+      <c r="M285">
+        <v>771.2911376953125</v>
+      </c>
+      <c r="N285">
+        <v>0.9374160170555115</v>
+      </c>
+      <c r="O285">
+        <v>0.9336604475975037</v>
+      </c>
+      <c r="P285">
+        <v>0.952552080154419</v>
+      </c>
+      <c r="Q285">
+        <v>2366.099853515625</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B286" t="str">
+        <v>11:31:05 ч.</v>
+      </c>
+      <c r="C286" t="str">
+        <v>Priem UHT</v>
+      </c>
+      <c r="D286">
+        <v>866.841458558811</v>
+      </c>
+      <c r="E286">
+        <v>233.8354034423828</v>
+      </c>
+      <c r="F286">
+        <v>234.43409729003906</v>
+      </c>
+      <c r="G286">
+        <v>235.98875427246094</v>
+      </c>
+      <c r="H286">
+        <v>0.9257919192314148</v>
+      </c>
+      <c r="I286">
+        <v>0.4919263422489166</v>
+      </c>
+      <c r="J286">
+        <v>1.9446885585784912</v>
+      </c>
+      <c r="K286">
+        <v>119.0114517211914</v>
+      </c>
+      <c r="L286">
+        <v>82.5771255493164</v>
+      </c>
+      <c r="M286">
+        <v>424.0621643066406</v>
+      </c>
+      <c r="N286">
+        <v>0.5497498512268066</v>
+      </c>
+      <c r="O286">
+        <v>0.7160426378250122</v>
+      </c>
+      <c r="P286">
+        <v>0.9240344762802124</v>
+      </c>
+      <c r="Q286">
+        <v>625.6506958007812</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B287" t="str">
+        <v>11:34:59 ч.</v>
+      </c>
+      <c r="C287" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D287">
+        <v>139039.84287220243</v>
+      </c>
+      <c r="E287">
+        <v>234.04708862304688</v>
+      </c>
+      <c r="F287">
+        <v>232.30006408691406</v>
+      </c>
+      <c r="G287">
+        <v>234.02671813964844</v>
+      </c>
+      <c r="H287">
+        <v>1.6108572483062744</v>
+      </c>
+      <c r="I287">
+        <v>1.6497472524642944</v>
+      </c>
+      <c r="J287">
+        <v>1.4497126340866089</v>
+      </c>
+      <c r="K287">
+        <v>273.1100769042969</v>
+      </c>
+      <c r="L287">
+        <v>199.96592712402344</v>
+      </c>
+      <c r="M287">
+        <v>208.5653076171875</v>
+      </c>
+      <c r="N287">
+        <v>0.7247591018676758</v>
+      </c>
+      <c r="O287">
+        <v>0.5180574655532837</v>
+      </c>
+      <c r="P287">
+        <v>0.6132330298423767</v>
+      </c>
+      <c r="Q287">
+        <v>681.29638671875</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B288" t="str">
+        <v>11:34:59 ч.</v>
+      </c>
+      <c r="C288" t="str">
+        <v>Ampak</v>
+      </c>
+      <c r="D288">
+        <v>41498.19333059519</v>
+      </c>
+      <c r="E288">
+        <v>233.59188842773438</v>
+      </c>
+      <c r="F288">
+        <v>231.6588897705078</v>
+      </c>
+      <c r="G288">
+        <v>234.00479125976562</v>
+      </c>
+      <c r="H288">
+        <v>61.16294860839844</v>
+      </c>
+      <c r="I288">
+        <v>59.90518569946289</v>
+      </c>
+      <c r="J288">
+        <v>53.413726806640625</v>
+      </c>
+      <c r="K288">
+        <v>13908.85546875</v>
+      </c>
+      <c r="L288">
+        <v>13485.943359375</v>
+      </c>
+      <c r="M288">
+        <v>11271.138671875</v>
+      </c>
+      <c r="N288">
+        <v>0.9704294800758362</v>
+      </c>
+      <c r="O288">
+        <v>0.9652419686317444</v>
+      </c>
+      <c r="P288">
+        <v>0.9695830345153809</v>
+      </c>
+      <c r="Q288">
+        <v>36413.8203125</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B289" t="str">
+        <v>11:34:59 ч.</v>
+      </c>
+      <c r="C289" t="str">
+        <v>Ledena Voda</v>
+      </c>
+      <c r="D289">
+        <v>246450.58792943895</v>
+      </c>
+      <c r="E289">
+        <v>227.3567657470703</v>
+      </c>
+      <c r="F289">
+        <v>232.06906127929688</v>
+      </c>
+      <c r="G289">
+        <v>232.31817626953125</v>
+      </c>
+      <c r="H289">
+        <v>218.82286071777344</v>
+      </c>
+      <c r="I289">
+        <v>228.66888427734375</v>
+      </c>
+      <c r="J289">
+        <v>238.2329559326172</v>
+      </c>
+      <c r="K289">
+        <v>39714.1796875</v>
+      </c>
+      <c r="L289">
+        <v>44117.06640625</v>
+      </c>
+      <c r="M289">
+        <v>43379.78125</v>
+      </c>
+      <c r="N289">
+        <v>0.7971324324607849</v>
+      </c>
+      <c r="O289">
+        <v>0.8315795063972473</v>
+      </c>
+      <c r="P289">
+        <v>0.7846367955207825</v>
+      </c>
+      <c r="Q289">
+        <v>127211.03125</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B290" t="str">
+        <v>11:34:59 ч.</v>
+      </c>
+      <c r="C290" t="str">
+        <v>Hladilnici</v>
+      </c>
+      <c r="D290">
+        <v>181756.3530135374</v>
+      </c>
+      <c r="E290">
+        <v>235.97203063964844</v>
+      </c>
+      <c r="F290">
+        <v>234.3617706298828</v>
+      </c>
+      <c r="G290">
+        <v>233.99009704589844</v>
+      </c>
+      <c r="H290">
+        <v>24.339866638183594</v>
+      </c>
+      <c r="I290">
+        <v>22.833919525146484</v>
+      </c>
+      <c r="J290">
+        <v>25.498685836791992</v>
+      </c>
+      <c r="K290">
+        <v>3681.775390625</v>
+      </c>
+      <c r="L290">
+        <v>3454.43408203125</v>
+      </c>
+      <c r="M290">
+        <v>4533.7490234375</v>
+      </c>
+      <c r="N290">
+        <v>0.6410303115844727</v>
+      </c>
+      <c r="O290">
+        <v>0.6554543972015381</v>
+      </c>
+      <c r="P290">
+        <v>0.7524726986885071</v>
+      </c>
+      <c r="Q290">
+        <v>11629.658203125</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B291" t="str">
+        <v>11:34:59 ч.</v>
+      </c>
+      <c r="C291" t="str">
+        <v>Kompresorno</v>
+      </c>
+      <c r="D291">
+        <v>49945.332177275406</v>
+      </c>
+      <c r="E291">
+        <v>234.25942993164062</v>
+      </c>
+      <c r="F291">
+        <v>234.1260223388672</v>
+      </c>
+      <c r="G291">
+        <v>232.0445098876953</v>
+      </c>
+      <c r="H291">
+        <v>48.105220794677734</v>
+      </c>
+      <c r="I291">
+        <v>44.277427673339844</v>
+      </c>
+      <c r="J291">
+        <v>45.05955505371094</v>
+      </c>
+      <c r="K291">
+        <v>9359.166015625</v>
+      </c>
+      <c r="L291">
+        <v>8538.8203125</v>
+      </c>
+      <c r="M291">
+        <v>8388.5205078125</v>
+      </c>
+      <c r="N291">
+        <v>0.8303981423377991</v>
+      </c>
+      <c r="O291">
+        <v>0.8236907124519348</v>
+      </c>
+      <c r="P291">
+        <v>0.8022822141647339</v>
+      </c>
+      <c r="Q291">
+        <v>26286.505859375</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B292" t="str">
+        <v>11:34:59 ч.</v>
+      </c>
+      <c r="C292" t="str">
+        <v>Priemno</v>
+      </c>
+      <c r="D292">
+        <v>59473.28491970646</v>
+      </c>
+      <c r="E292">
+        <v>233.6055450439453</v>
+      </c>
+      <c r="F292">
+        <v>234.0975341796875</v>
+      </c>
+      <c r="G292">
+        <v>236.05703735351562</v>
+      </c>
+      <c r="H292">
+        <v>67.63082122802734</v>
+      </c>
+      <c r="I292">
+        <v>52.299827575683594</v>
+      </c>
+      <c r="J292">
+        <v>56.111480712890625</v>
+      </c>
+      <c r="K292">
+        <v>14530.265625</v>
+      </c>
+      <c r="L292">
+        <v>10998.3720703125</v>
+      </c>
+      <c r="M292">
+        <v>12069.259765625</v>
+      </c>
+      <c r="N292">
+        <v>0.91844642162323</v>
+      </c>
+      <c r="O292">
+        <v>0.9020472764968872</v>
+      </c>
+      <c r="P292">
+        <v>0.9108167886734009</v>
+      </c>
+      <c r="Q292">
+        <v>37597.89453125</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B293" t="str">
+        <v>11:34:59 ч.</v>
+      </c>
+      <c r="C293" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="D293">
+        <v>239108.11288025504</v>
+      </c>
+      <c r="E293">
+        <v>233.76661682128906</v>
+      </c>
+      <c r="F293">
+        <v>234.62265014648438</v>
+      </c>
+      <c r="G293">
+        <v>236.83143615722656</v>
+      </c>
+      <c r="H293">
+        <v>203.2560577392578</v>
+      </c>
+      <c r="I293">
+        <v>210.5198211669922</v>
+      </c>
+      <c r="J293">
+        <v>208.9992218017578</v>
+      </c>
+      <c r="K293">
+        <v>41235.37109375</v>
+      </c>
+      <c r="L293">
+        <v>41704.91015625</v>
+      </c>
+      <c r="M293">
+        <v>42962.4921875</v>
+      </c>
+      <c r="N293">
+        <v>0.8678485155105591</v>
+      </c>
+      <c r="O293">
+        <v>0.8443534970283508</v>
+      </c>
+      <c r="P293">
+        <v>0.8679714798927307</v>
+      </c>
+      <c r="Q293">
+        <v>127124.65625</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B294" t="str">
+        <v>11:34:59 ч.</v>
+      </c>
+      <c r="C294" t="str">
+        <v>HOMO UHT</v>
+      </c>
+      <c r="D294">
+        <v>1828.1639539651658</v>
+      </c>
+      <c r="E294">
+        <v>233.6693878173828</v>
+      </c>
+      <c r="F294">
+        <v>234.373046875</v>
+      </c>
+      <c r="G294">
+        <v>236.0165557861328</v>
+      </c>
+      <c r="H294">
+        <v>0.25350138545036316</v>
+      </c>
+      <c r="I294">
+        <v>0.108648382127285</v>
+      </c>
+      <c r="J294">
+        <v>0.22688724100589752</v>
+      </c>
+      <c r="K294">
+        <v>35.604496002197266</v>
+      </c>
+      <c r="L294">
+        <v>13.950051307678223</v>
+      </c>
+      <c r="M294">
+        <v>14.54134750366211</v>
+      </c>
+      <c r="N294">
+        <v>0.6010667085647583</v>
+      </c>
+      <c r="O294">
+        <v>0.5478288531303406</v>
+      </c>
+      <c r="P294">
+        <v>0.2715514302253723</v>
+      </c>
+      <c r="Q294">
+        <v>64.09590148925781</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B295" t="str">
+        <v>11:34:59 ч.</v>
+      </c>
+      <c r="C295" t="str">
+        <v>Priem KM</v>
+      </c>
+      <c r="D295">
+        <v>5584.533528252194</v>
+      </c>
+      <c r="E295">
+        <v>233.54371643066406</v>
+      </c>
+      <c r="F295">
+        <v>234.22499084472656</v>
+      </c>
+      <c r="G295">
+        <v>236.0897979736328</v>
+      </c>
+      <c r="H295">
+        <v>4.352241516113281</v>
+      </c>
+      <c r="I295">
+        <v>3.225029945373535</v>
+      </c>
+      <c r="J295">
+        <v>3.69028902053833</v>
+      </c>
+      <c r="K295">
+        <v>946.023681640625</v>
+      </c>
+      <c r="L295">
+        <v>709.0487670898438</v>
+      </c>
+      <c r="M295">
+        <v>826.8490600585938</v>
+      </c>
+      <c r="N295">
+        <v>0.9302613139152527</v>
+      </c>
+      <c r="O295">
+        <v>0.937965989112854</v>
+      </c>
+      <c r="P295">
+        <v>0.949285626411438</v>
+      </c>
+      <c r="Q295">
+        <v>2481.921630859375</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B296" t="str">
+        <v>11:34:59 ч.</v>
+      </c>
+      <c r="C296" t="str">
+        <v>Priem UHT</v>
+      </c>
+      <c r="D296">
+        <v>866.8611334619393</v>
+      </c>
+      <c r="E296">
+        <v>233.50526428222656</v>
+      </c>
+      <c r="F296">
+        <v>233.92816162109375</v>
+      </c>
+      <c r="G296">
+        <v>235.94696044921875</v>
+      </c>
+      <c r="H296">
+        <v>0.9348407983779907</v>
+      </c>
+      <c r="I296">
+        <v>0.4906616806983948</v>
+      </c>
+      <c r="J296">
+        <v>0.8669565916061401</v>
+      </c>
+      <c r="K296">
+        <v>120.87081909179688</v>
+      </c>
+      <c r="L296">
+        <v>78.07147216796875</v>
+      </c>
+      <c r="M296">
+        <v>59.65293884277344</v>
+      </c>
+      <c r="N296">
+        <v>0.5537160634994507</v>
+      </c>
+      <c r="O296">
+        <v>0.6803232431411743</v>
+      </c>
+      <c r="P296">
+        <v>0.2928257882595062</v>
+      </c>
+      <c r="Q296">
+        <v>259.3312072753906</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B297" t="str">
+        <v>11:35:16 ч.</v>
+      </c>
+      <c r="C297" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D297">
+        <v>139039.84596084838</v>
+      </c>
+      <c r="E297">
+        <v>233.48904418945312</v>
+      </c>
+      <c r="F297">
+        <v>232.649658203125</v>
+      </c>
+      <c r="G297">
+        <v>235.26255798339844</v>
+      </c>
+      <c r="H297">
+        <v>1.6052494049072266</v>
+      </c>
+      <c r="I297">
+        <v>1.6629436016082764</v>
+      </c>
+      <c r="J297">
+        <v>1.473067045211792</v>
+      </c>
+      <c r="K297">
+        <v>269.45465087890625</v>
+      </c>
+      <c r="L297">
+        <v>202.2846221923828</v>
+      </c>
+      <c r="M297">
+        <v>213.44476318359375</v>
+      </c>
+      <c r="N297">
+        <v>0.7145059108734131</v>
+      </c>
+      <c r="O297">
+        <v>0.5214928388595581</v>
+      </c>
+      <c r="P297">
+        <v>0.6103470325469971</v>
+      </c>
+      <c r="Q297">
+        <v>682.157470703125</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B298" t="str">
+        <v>11:35:16 ч.</v>
+      </c>
+      <c r="C298" t="str">
+        <v>Ampak</v>
+      </c>
+      <c r="D298">
+        <v>41498.281765527776</v>
+      </c>
+      <c r="E298">
+        <v>232.9197235107422</v>
+      </c>
+      <c r="F298">
+        <v>233.00082397460938</v>
+      </c>
+      <c r="G298">
+        <v>235.95347595214844</v>
+      </c>
+      <c r="H298">
+        <v>29.345827102661133</v>
+      </c>
+      <c r="I298">
+        <v>27.894498825073242</v>
+      </c>
+      <c r="J298">
+        <v>22.0338134765625</v>
+      </c>
+      <c r="K298">
+        <v>5940.46484375</v>
+      </c>
+      <c r="L298">
+        <v>5401.4599609375</v>
+      </c>
+      <c r="M298">
+        <v>4356.6494140625</v>
+      </c>
+      <c r="N298">
+        <v>0.888822078704834</v>
+      </c>
+      <c r="O298">
+        <v>0.8584547638893127</v>
+      </c>
+      <c r="P298">
+        <v>0.9037415385246277</v>
+      </c>
+      <c r="Q298">
+        <v>18357.869140625</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B299" t="str">
+        <v>11:35:16 ч.</v>
+      </c>
+      <c r="C299" t="str">
+        <v>Ledena Voda</v>
+      </c>
+      <c r="D299">
+        <v>246451.03486804437</v>
+      </c>
+      <c r="E299">
+        <v>233.65443420410156</v>
+      </c>
+      <c r="F299">
+        <v>234.73373413085938</v>
+      </c>
+      <c r="G299">
+        <v>236.160400390625</v>
+      </c>
+      <c r="H299">
+        <v>75.52364349365234</v>
+      </c>
+      <c r="I299">
+        <v>79.38651275634766</v>
+      </c>
+      <c r="J299">
+        <v>82.65031433105469</v>
+      </c>
+      <c r="K299">
+        <v>15210.7607421875</v>
+      </c>
+      <c r="L299">
+        <v>16639.978515625</v>
+      </c>
+      <c r="M299">
+        <v>16711.609375</v>
+      </c>
+      <c r="N299">
+        <v>0.8548843860626221</v>
+      </c>
+      <c r="O299">
+        <v>0.8872960209846497</v>
+      </c>
+      <c r="P299">
+        <v>0.8560949563980103</v>
+      </c>
+      <c r="Q299">
+        <v>48562.34765625</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B300" t="str">
+        <v>11:35:16 ч.</v>
+      </c>
+      <c r="C300" t="str">
+        <v>Hladilnici</v>
+      </c>
+      <c r="D300">
+        <v>181756.40351985826</v>
+      </c>
+      <c r="E300">
+        <v>237.12899780273438</v>
+      </c>
+      <c r="F300">
+        <v>235.44996643066406</v>
+      </c>
+      <c r="G300">
+        <v>235.03982543945312</v>
+      </c>
+      <c r="H300">
+        <v>8.10897159576416</v>
+      </c>
+      <c r="I300">
+        <v>8.881720542907715</v>
+      </c>
+      <c r="J300">
+        <v>11.534865379333496</v>
+      </c>
+      <c r="K300">
+        <v>1564.95556640625</v>
+      </c>
+      <c r="L300">
+        <v>1749.2691650390625</v>
+      </c>
+      <c r="M300">
+        <v>2636.84814453125</v>
+      </c>
+      <c r="N300">
+        <v>0.8138635158538818</v>
+      </c>
+      <c r="O300">
+        <v>0.8364903330802917</v>
+      </c>
+      <c r="P300">
+        <v>0.9726058840751648</v>
+      </c>
+      <c r="Q300">
+        <v>5939.6572265625</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B301" t="str">
+        <v>11:35:16 ч.</v>
+      </c>
+      <c r="C301" t="str">
+        <v>Kompresorno</v>
+      </c>
+      <c r="D301">
+        <v>49945.455629817945</v>
+      </c>
+      <c r="E301">
+        <v>235.53659057617188</v>
+      </c>
+      <c r="F301">
+        <v>233.004150390625</v>
+      </c>
+      <c r="G301">
+        <v>232.6078643798828</v>
+      </c>
+      <c r="H301">
+        <v>50.97119140625</v>
+      </c>
+      <c r="I301">
+        <v>42.33242416381836</v>
+      </c>
+      <c r="J301">
+        <v>47.95822525024414</v>
+      </c>
+      <c r="K301">
+        <v>10216.9384765625</v>
+      </c>
+      <c r="L301">
+        <v>8051.875</v>
+      </c>
+      <c r="M301">
+        <v>8759.533203125</v>
+      </c>
+      <c r="N301">
+        <v>0.8514642715454102</v>
+      </c>
+      <c r="O301">
+        <v>0.8177018761634827</v>
+      </c>
+      <c r="P301">
+        <v>0.7861248850822449</v>
+      </c>
+      <c r="Q301">
+        <v>27028.34765625</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B302" t="str">
+        <v>11:35:16 ч.</v>
+      </c>
+      <c r="C302" t="str">
+        <v>Priemno</v>
+      </c>
+      <c r="D302">
+        <v>59473.46005099165</v>
+      </c>
+      <c r="E302">
+        <v>234.58277893066406</v>
+      </c>
+      <c r="F302">
+        <v>234.83827209472656</v>
+      </c>
+      <c r="G302">
+        <v>236.9456787109375</v>
+      </c>
+      <c r="H302">
+        <v>66.48416900634766</v>
+      </c>
+      <c r="I302">
+        <v>53.01124572753906</v>
+      </c>
+      <c r="J302">
+        <v>54.96250915527344</v>
+      </c>
+      <c r="K302">
+        <v>14363.8916015625</v>
+      </c>
+      <c r="L302">
+        <v>11236.7138671875</v>
+      </c>
+      <c r="M302">
+        <v>11750.9306640625</v>
+      </c>
+      <c r="N302">
+        <v>0.9214116930961609</v>
+      </c>
+      <c r="O302">
+        <v>0.901561975479126</v>
+      </c>
+      <c r="P302">
+        <v>0.9037612676620483</v>
+      </c>
+      <c r="Q302">
+        <v>37357.4140625</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B303" t="str">
+        <v>11:35:16 ч.</v>
+      </c>
+      <c r="C303" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="D303">
+        <v>239108.59391478854</v>
+      </c>
+      <c r="E303">
+        <v>234.6153564453125</v>
+      </c>
+      <c r="F303">
+        <v>235.27105712890625</v>
+      </c>
+      <c r="G303">
+        <v>237.60450744628906</v>
+      </c>
+      <c r="H303">
+        <v>123.7481689453125</v>
+      </c>
+      <c r="I303">
+        <v>138.0262908935547</v>
+      </c>
+      <c r="J303">
+        <v>131.62881469726562</v>
+      </c>
+      <c r="K303">
+        <v>26836.208984375</v>
+      </c>
+      <c r="L303">
+        <v>29129.416015625</v>
+      </c>
+      <c r="M303">
+        <v>29167.7421875</v>
+      </c>
+      <c r="N303">
+        <v>0.9243276715278625</v>
+      </c>
+      <c r="O303">
+        <v>0.8970186710357666</v>
+      </c>
+      <c r="P303">
+        <v>0.9326038360595703</v>
+      </c>
+      <c r="Q303">
+        <v>85133.3671875</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B304" t="str">
+        <v>11:35:16 ч.</v>
+      </c>
+      <c r="C304" t="str">
+        <v>HOMO UHT</v>
+      </c>
+      <c r="D304">
+        <v>1828.1642501946308</v>
+      </c>
+      <c r="E304">
+        <v>234.4953155517578</v>
+      </c>
+      <c r="F304">
+        <v>235.0742645263672</v>
+      </c>
+      <c r="G304">
+        <v>236.78314208984375</v>
+      </c>
+      <c r="H304">
+        <v>0.24488231539726257</v>
+      </c>
+      <c r="I304">
+        <v>0.10911817848682404</v>
+      </c>
+      <c r="J304">
+        <v>0.21594427525997162</v>
+      </c>
+      <c r="K304">
+        <v>36.14398193359375</v>
+      </c>
+      <c r="L304">
+        <v>14.070292472839355</v>
+      </c>
+      <c r="M304">
+        <v>14.920917510986328</v>
+      </c>
+      <c r="N304">
+        <v>0.6294256448745728</v>
+      </c>
+      <c r="O304">
+        <v>0.5485306978225708</v>
+      </c>
+      <c r="P304">
+        <v>0.2918119430541992</v>
+      </c>
+      <c r="Q304">
+        <v>65.13519287109375</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B305" t="str">
+        <v>11:35:16 ч.</v>
+      </c>
+      <c r="C305" t="str">
+        <v>Priem KM</v>
+      </c>
+      <c r="D305">
+        <v>5584.544894995728</v>
+      </c>
+      <c r="E305">
+        <v>234.50540161132812</v>
+      </c>
+      <c r="F305">
+        <v>235.05462646484375</v>
+      </c>
+      <c r="G305">
+        <v>237.01084899902344</v>
+      </c>
+      <c r="H305">
+        <v>4.306962013244629</v>
+      </c>
+      <c r="I305">
+        <v>3.260758876800537</v>
+      </c>
+      <c r="J305">
+        <v>3.668287754058838</v>
+      </c>
+      <c r="K305">
+        <v>941.7518310546875</v>
+      </c>
+      <c r="L305">
+        <v>721.24853515625</v>
+      </c>
+      <c r="M305">
+        <v>825.9464111328125</v>
+      </c>
+      <c r="N305">
+        <v>0.9322017431259155</v>
+      </c>
+      <c r="O305">
+        <v>0.9408215284347534</v>
+      </c>
+      <c r="P305">
+        <v>0.9498557448387146</v>
+      </c>
+      <c r="Q305">
+        <v>2488.94677734375</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B306" t="str">
+        <v>11:35:16 ч.</v>
+      </c>
+      <c r="C306" t="str">
+        <v>Priem UHT</v>
+      </c>
+      <c r="D306">
+        <v>866.8623434111719</v>
+      </c>
+      <c r="E306">
+        <v>234.66085815429688</v>
+      </c>
+      <c r="F306">
+        <v>234.96824645996094</v>
+      </c>
+      <c r="G306">
+        <v>236.9959259033203</v>
+      </c>
+      <c r="H306">
+        <v>0.9322619438171387</v>
+      </c>
+      <c r="I306">
+        <v>0.4838990569114685</v>
+      </c>
+      <c r="J306">
+        <v>0.861859917640686</v>
+      </c>
+      <c r="K306">
+        <v>121.11306762695312</v>
+      </c>
+      <c r="L306">
+        <v>78.44915771484375</v>
+      </c>
+      <c r="M306">
+        <v>59.587432861328125</v>
+      </c>
+      <c r="N306">
+        <v>0.5534821152687073</v>
+      </c>
+      <c r="O306">
+        <v>0.6887516975402832</v>
+      </c>
+      <c r="P306">
+        <v>0.2927297353744507</v>
+      </c>
+      <c r="Q306">
+        <v>259.4530944824219</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B307" t="str">
+        <v>11:35:37 ч.</v>
+      </c>
+      <c r="C307" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D307">
+        <v>139039.8481421165</v>
+      </c>
+      <c r="E307">
+        <v>233.43109130859375</v>
+      </c>
+      <c r="F307">
+        <v>233.36380004882812</v>
+      </c>
+      <c r="G307">
+        <v>235.82131958007812</v>
+      </c>
+      <c r="H307">
+        <v>1.6107711791992188</v>
+      </c>
+      <c r="I307">
+        <v>1.6577550172805786</v>
+      </c>
+      <c r="J307">
+        <v>1.4731987714767456</v>
+      </c>
+      <c r="K307">
+        <v>268.1653747558594</v>
+      </c>
+      <c r="L307">
+        <v>199.87063598632812</v>
+      </c>
+      <c r="M307">
+        <v>213.7029571533203</v>
+      </c>
+      <c r="N307">
+        <v>0.7126326560974121</v>
+      </c>
+      <c r="O307">
+        <v>0.5168653130531311</v>
+      </c>
+      <c r="P307">
+        <v>0.6145339608192444</v>
+      </c>
+      <c r="Q307">
+        <v>681.2852172851562</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B308" t="str">
+        <v>11:35:37 ч.</v>
+      </c>
+      <c r="C308" t="str">
+        <v>Ampak</v>
+      </c>
+      <c r="D308">
+        <v>41498.38234095054</v>
+      </c>
+      <c r="E308">
+        <v>233.37045288085938</v>
+      </c>
+      <c r="F308">
+        <v>232.99302673339844</v>
+      </c>
+      <c r="G308">
+        <v>235.72781372070312</v>
+      </c>
+      <c r="H308">
+        <v>31.499082565307617</v>
+      </c>
+      <c r="I308">
+        <v>28.86552619934082</v>
+      </c>
+      <c r="J308">
+        <v>23.925735473632812</v>
+      </c>
+      <c r="K308">
+        <v>6404.1455078125</v>
+      </c>
+      <c r="L308">
+        <v>5531.98828125</v>
+      </c>
+      <c r="M308">
+        <v>4655.5595703125</v>
+      </c>
+      <c r="N308">
+        <v>0.8711991310119629</v>
+      </c>
+      <c r="O308">
+        <v>0.8225434422492981</v>
+      </c>
+      <c r="P308">
+        <v>0.840507447719574</v>
+      </c>
+      <c r="Q308">
+        <v>16149.875</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B309" t="str">
+        <v>11:35:37 ч.</v>
+      </c>
+      <c r="C309" t="str">
+        <v>Ledena Voda</v>
+      </c>
+      <c r="D309">
+        <v>246451.28533854388</v>
+      </c>
+      <c r="E309">
+        <v>229.91197204589844</v>
+      </c>
+      <c r="F309">
+        <v>233.41314697265625</v>
+      </c>
+      <c r="G309">
+        <v>234.389892578125</v>
+      </c>
+      <c r="H309">
+        <v>209.6635284423828</v>
+      </c>
+      <c r="I309">
+        <v>209.90069580078125</v>
+      </c>
+      <c r="J309">
+        <v>226.75096130371094</v>
+      </c>
+      <c r="K309">
+        <v>24826.064453125</v>
+      </c>
+      <c r="L309">
+        <v>28073.72265625</v>
+      </c>
+      <c r="M309">
+        <v>28256.9140625</v>
+      </c>
+      <c r="N309">
+        <v>0.5150191783905029</v>
+      </c>
+      <c r="O309">
+        <v>0.573008120059967</v>
+      </c>
+      <c r="P309">
+        <v>0.751428484916687</v>
+      </c>
+      <c r="Q309">
+        <v>110054.734375</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B310" t="str">
+        <v>11:35:37 ч.</v>
+      </c>
+      <c r="C310" t="str">
+        <v>Hladilnici</v>
+      </c>
+      <c r="D310">
+        <v>181756.43338112513</v>
+      </c>
+      <c r="E310">
+        <v>236.72586059570312</v>
+      </c>
+      <c r="F310">
+        <v>234.92893981933594</v>
+      </c>
+      <c r="G310">
+        <v>234.93479919433594</v>
+      </c>
+      <c r="H310">
+        <v>8.140167236328125</v>
+      </c>
+      <c r="I310">
+        <v>8.853060722351074</v>
+      </c>
+      <c r="J310">
+        <v>11.038558959960938</v>
+      </c>
+      <c r="K310">
+        <v>1571.2003173828125</v>
+      </c>
+      <c r="L310">
+        <v>1741.9781494140625</v>
+      </c>
+      <c r="M310">
+        <v>2485.08349609375</v>
+      </c>
+      <c r="N310">
+        <v>0.8152654767036438</v>
+      </c>
+      <c r="O310">
+        <v>0.837906002998352</v>
+      </c>
+      <c r="P310">
+        <v>0.963256299495697</v>
+      </c>
+      <c r="Q310">
+        <v>5798.26220703125</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B311" t="str">
+        <v>11:35:37 ч.</v>
+      </c>
+      <c r="C311" t="str">
+        <v>Kompresorno</v>
+      </c>
+      <c r="D311">
+        <v>49945.596086638914</v>
+      </c>
+      <c r="E311">
+        <v>235.37252807617188</v>
+      </c>
+      <c r="F311">
+        <v>233.87686157226562</v>
+      </c>
+      <c r="G311">
+        <v>232.40858459472656</v>
+      </c>
+      <c r="H311">
+        <v>50.41556930541992</v>
+      </c>
+      <c r="I311">
+        <v>44.6947021484375</v>
+      </c>
+      <c r="J311">
+        <v>46.0716667175293</v>
+      </c>
+      <c r="K311">
+        <v>9938.4560546875</v>
+      </c>
+      <c r="L311">
+        <v>8627.3056640625</v>
+      </c>
+      <c r="M311">
+        <v>8444.37109375</v>
+      </c>
+      <c r="N311">
+        <v>0.8386992812156677</v>
+      </c>
+      <c r="O311">
+        <v>0.8245523571968079</v>
+      </c>
+      <c r="P311">
+        <v>0.7883039116859436</v>
+      </c>
+      <c r="Q311">
+        <v>27010.1328125</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B312" t="str">
+        <v>11:35:37 ч.</v>
+      </c>
+      <c r="C312" t="str">
+        <v>Priemno</v>
+      </c>
+      <c r="D312">
+        <v>59473.65998018133</v>
+      </c>
+      <c r="E312">
+        <v>233.99838256835938</v>
+      </c>
+      <c r="F312">
+        <v>234.68359375</v>
+      </c>
+      <c r="G312">
+        <v>236.5565185546875</v>
+      </c>
+      <c r="H312">
+        <v>67.80782318115234</v>
+      </c>
+      <c r="I312">
+        <v>53.78722381591797</v>
+      </c>
+      <c r="J312">
+        <v>56.42068862915039</v>
+      </c>
+      <c r="K312">
+        <v>14606.9501953125</v>
+      </c>
+      <c r="L312">
+        <v>11396.453125</v>
+      </c>
+      <c r="M312">
+        <v>12082.8935546875</v>
+      </c>
+      <c r="N312">
+        <v>0.9205912947654724</v>
+      </c>
+      <c r="O312">
+        <v>0.9028339385986328</v>
+      </c>
+      <c r="P312">
+        <v>0.9049559831619263</v>
+      </c>
+      <c r="Q312">
+        <v>38036.796875</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B313" t="str">
+        <v>11:35:37 ч.</v>
+      </c>
+      <c r="C313" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="D313">
+        <v>239109.06428105576</v>
+      </c>
+      <c r="E313">
+        <v>234.3719024658203</v>
+      </c>
+      <c r="F313">
+        <v>234.84817504882812</v>
+      </c>
+      <c r="G313">
+        <v>237.24990844726562</v>
+      </c>
+      <c r="H313">
+        <v>182.03570556640625</v>
+      </c>
+      <c r="I313">
+        <v>190.66297912597656</v>
+      </c>
+      <c r="J313">
+        <v>190.01429748535156</v>
+      </c>
+      <c r="K313">
+        <v>39080.42578125</v>
+      </c>
+      <c r="L313">
+        <v>37729.23828125</v>
+      </c>
+      <c r="M313">
+        <v>39087.93359375</v>
+      </c>
+      <c r="N313">
+        <v>0.9085410833358765</v>
+      </c>
+      <c r="O313">
+        <v>0.8768681287765503</v>
+      </c>
+      <c r="P313">
+        <v>0.9066787362098694</v>
+      </c>
+      <c r="Q313">
+        <v>114376.4375</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B314" t="str">
+        <v>11:35:37 ч.</v>
+      </c>
+      <c r="C314" t="str">
+        <v>HOMO UHT</v>
+      </c>
+      <c r="D314">
+        <v>1828.1646144887634</v>
+      </c>
+      <c r="E314">
+        <v>233.9027557373047</v>
+      </c>
+      <c r="F314">
+        <v>234.84759521484375</v>
+      </c>
+      <c r="G314">
+        <v>236.36849975585938</v>
+      </c>
+      <c r="H314">
+        <v>0.2408410608768463</v>
+      </c>
+      <c r="I314">
+        <v>0.11055883765220642</v>
+      </c>
+      <c r="J314">
+        <v>0.21268784999847412</v>
+      </c>
+      <c r="K314">
+        <v>34.88323974609375</v>
+      </c>
+      <c r="L314">
+        <v>14.304891586303711</v>
+      </c>
+      <c r="M314">
+        <v>14.313095092773438</v>
+      </c>
+      <c r="N314">
+        <v>0.6192284822463989</v>
+      </c>
+      <c r="O314">
+        <v>0.5509408712387085</v>
+      </c>
+      <c r="P314">
+        <v>0.28470903635025024</v>
+      </c>
+      <c r="Q314">
+        <v>64.47151947021484</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B315" t="str">
+        <v>11:35:37 ч.</v>
+      </c>
+      <c r="C315" t="str">
+        <v>Priem KM</v>
+      </c>
+      <c r="D315">
+        <v>5584.5587924794945</v>
+      </c>
+      <c r="E315">
+        <v>233.8892822265625</v>
+      </c>
+      <c r="F315">
+        <v>234.8009033203125</v>
+      </c>
+      <c r="G315">
+        <v>236.4967498779297</v>
+      </c>
+      <c r="H315">
+        <v>4.268750190734863</v>
+      </c>
+      <c r="I315">
+        <v>3.3020808696746826</v>
+      </c>
+      <c r="J315">
+        <v>3.648548126220703</v>
+      </c>
+      <c r="K315">
+        <v>933.584228515625</v>
+      </c>
+      <c r="L315">
+        <v>729.8442993164062</v>
+      </c>
+      <c r="M315">
+        <v>817.8096923828125</v>
+      </c>
+      <c r="N315">
+        <v>0.9347811341285706</v>
+      </c>
+      <c r="O315">
+        <v>0.9411607384681702</v>
+      </c>
+      <c r="P315">
+        <v>0.950427234172821</v>
+      </c>
+      <c r="Q315">
+        <v>2474.43408203125</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B316" t="str">
+        <v>11:35:37 ч.</v>
+      </c>
+      <c r="C316" t="str">
+        <v>Priem UHT</v>
+      </c>
+      <c r="D316">
+        <v>866.8637933700217</v>
+      </c>
+      <c r="E316">
+        <v>233.94052124023438</v>
+      </c>
+      <c r="F316">
+        <v>234.6814727783203</v>
+      </c>
+      <c r="G316">
+        <v>236.46115112304688</v>
+      </c>
+      <c r="H316">
+        <v>0.9294095039367676</v>
+      </c>
+      <c r="I316">
+        <v>0.4953721761703491</v>
+      </c>
+      <c r="J316">
+        <v>0.8503389358520508</v>
+      </c>
+      <c r="K316">
+        <v>118.70856475830078</v>
+      </c>
+      <c r="L316">
+        <v>80.72882843017578</v>
+      </c>
+      <c r="M316">
+        <v>59.85017776489258</v>
+      </c>
+      <c r="N316">
+        <v>0.545805037021637</v>
+      </c>
+      <c r="O316">
+        <v>0.694383442401886</v>
+      </c>
+      <c r="P316">
+        <v>0.297630250453949</v>
+      </c>
+      <c r="Q316">
+        <v>259.2875671386719</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B317" t="str">
+        <v>11:37:19 ч.</v>
+      </c>
+      <c r="C317" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D317">
+        <v>139039.86923576595</v>
+      </c>
+      <c r="E317">
+        <v>232.81832885742188</v>
+      </c>
+      <c r="F317">
+        <v>233.16192626953125</v>
+      </c>
+      <c r="G317">
+        <v>236.4571533203125</v>
+      </c>
+      <c r="H317">
+        <v>1.606011152267456</v>
+      </c>
+      <c r="I317">
+        <v>1.647168755531311</v>
+      </c>
+      <c r="J317">
+        <v>1.489527702331543</v>
+      </c>
+      <c r="K317">
+        <v>264.9479675292969</v>
+      </c>
+      <c r="L317">
+        <v>201.7086944580078</v>
+      </c>
+      <c r="M317">
+        <v>215.3571319580078</v>
+      </c>
+      <c r="N317">
+        <v>0.7076433897018433</v>
+      </c>
+      <c r="O317">
+        <v>0.5217576622962952</v>
+      </c>
+      <c r="P317">
+        <v>0.6138358116149902</v>
+      </c>
+      <c r="Q317">
+        <v>682.0137939453125</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B318" t="str">
+        <v>11:37:19 ч.</v>
+      </c>
+      <c r="C318" t="str">
+        <v>Ampak</v>
+      </c>
+      <c r="D318">
+        <v>41498.96723986035</v>
+      </c>
+      <c r="E318">
+        <v>232.66925048828125</v>
+      </c>
+      <c r="F318">
+        <v>233.12191772460938</v>
+      </c>
+      <c r="G318">
+        <v>236.58998107910156</v>
+      </c>
+      <c r="H318">
+        <v>57.94940948486328</v>
+      </c>
+      <c r="I318">
+        <v>58.71915817260742</v>
+      </c>
+      <c r="J318">
+        <v>52.13019943237305</v>
+      </c>
+      <c r="K318">
+        <v>13016.8828125</v>
+      </c>
+      <c r="L318">
+        <v>13117.4072265625</v>
+      </c>
+      <c r="M318">
+        <v>4651.029296875</v>
+      </c>
+      <c r="N318">
+        <v>0.8558935523033142</v>
+      </c>
+      <c r="O318">
+        <v>0.8381749987602234</v>
+      </c>
+      <c r="P318">
+        <v>0.8574268221855164</v>
+      </c>
+      <c r="Q318">
+        <v>15889.470703125</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B319" t="str">
+        <v>11:37:19 ч.</v>
+      </c>
+      <c r="C319" t="str">
+        <v>Ledena Voda</v>
+      </c>
+      <c r="D319">
+        <v>246451.99019911184</v>
+      </c>
+      <c r="E319">
+        <v>236.3610076904297</v>
+      </c>
+      <c r="F319">
+        <v>236.25392150878906</v>
+      </c>
+      <c r="G319">
+        <v>238.35177612304688</v>
+      </c>
+      <c r="H319">
+        <v>7.052023410797119</v>
+      </c>
+      <c r="I319">
+        <v>8.0681734085083</v>
+      </c>
+      <c r="J319">
+        <v>7.056722164154053</v>
+      </c>
+      <c r="K319">
+        <v>1159.5728759765625</v>
+      </c>
+      <c r="L319">
+        <v>1459.978759765625</v>
+      </c>
+      <c r="M319">
+        <v>1222.1314697265625</v>
+      </c>
+      <c r="N319">
+        <v>0.6958251595497131</v>
+      </c>
+      <c r="O319">
+        <v>0.7661461234092712</v>
+      </c>
+      <c r="P319">
+        <v>0.7270365357398987</v>
+      </c>
+      <c r="Q319">
+        <v>3841.68310546875</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B320" t="str">
+        <v>11:37:19 ч.</v>
+      </c>
+      <c r="C320" t="str">
+        <v>Hladilnici</v>
+      </c>
+      <c r="D320">
+        <v>181756.60998403063</v>
+      </c>
+      <c r="E320">
+        <v>237.76820373535156</v>
+      </c>
+      <c r="F320">
+        <v>236.08717346191406</v>
+      </c>
+      <c r="G320">
+        <v>235.72084045410156</v>
+      </c>
+      <c r="H320">
+        <v>11.042110443115234</v>
+      </c>
+      <c r="I320">
+        <v>8.874364852905273</v>
+      </c>
+      <c r="J320">
+        <v>14.171689987182617</v>
+      </c>
+      <c r="K320">
+        <v>2189.535888671875</v>
+      </c>
+      <c r="L320">
+        <v>1748.3226318359375</v>
+      </c>
+      <c r="M320">
+        <v>3017.9384765625</v>
+      </c>
+      <c r="N320">
+        <v>0.8341121673583984</v>
+      </c>
+      <c r="O320">
+        <v>0.8348723649978638</v>
+      </c>
+      <c r="P320">
+        <v>0.9052847623825073</v>
+      </c>
+      <c r="Q320">
+        <v>6960.1865234375</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B321" t="str">
+        <v>11:37:19 ч.</v>
+      </c>
+      <c r="C321" t="str">
+        <v>Kompresorno</v>
+      </c>
+      <c r="D321">
+        <v>49946.33893364857</v>
+      </c>
+      <c r="E321">
+        <v>236.73252868652344</v>
+      </c>
+      <c r="F321">
+        <v>233.38832092285156</v>
+      </c>
+      <c r="G321">
+        <v>233.49424743652344</v>
+      </c>
+      <c r="H321">
+        <v>49.25482940673828</v>
+      </c>
+      <c r="I321">
+        <v>39.03001403808594</v>
+      </c>
+      <c r="J321">
+        <v>46.15657043457031</v>
+      </c>
+      <c r="K321">
+        <v>9862.7060546875</v>
+      </c>
+      <c r="L321">
+        <v>7389.064453125</v>
+      </c>
+      <c r="M321">
+        <v>8248.8388671875</v>
+      </c>
+      <c r="N321">
+        <v>0.8460661172866821</v>
+      </c>
+      <c r="O321">
+        <v>0.8110784292221069</v>
+      </c>
+      <c r="P321">
+        <v>0.7653905153274536</v>
+      </c>
+      <c r="Q321">
+        <v>25500.607421875</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B322" t="str">
+        <v>11:37:19 ч.</v>
+      </c>
+      <c r="C322" t="str">
+        <v>Priemno</v>
+      </c>
+      <c r="D322">
+        <v>59474.78988396704</v>
+      </c>
+      <c r="E322">
+        <v>235.24911499023438</v>
+      </c>
+      <c r="F322">
+        <v>235.51597595214844</v>
+      </c>
+      <c r="G322">
+        <v>237.62327575683594</v>
+      </c>
+      <c r="H322">
+        <v>68.07608795166016</v>
+      </c>
+      <c r="I322">
+        <v>54.004417419433594</v>
+      </c>
+      <c r="J322">
+        <v>57.02568435668945</v>
+      </c>
+      <c r="K322">
+        <v>14766.6826171875</v>
+      </c>
+      <c r="L322">
+        <v>11481.9990234375</v>
+      </c>
+      <c r="M322">
+        <v>12280.193359375</v>
+      </c>
+      <c r="N322">
+        <v>0.9192704558372498</v>
+      </c>
+      <c r="O322">
+        <v>0.9013424515724182</v>
+      </c>
+      <c r="P322">
+        <v>0.906389057636261</v>
+      </c>
+      <c r="Q322">
+        <v>38528.875</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B323" t="str">
+        <v>11:37:19 ч.</v>
+      </c>
+      <c r="C323" t="str">
+        <v>Trafo#1-7</v>
+      </c>
+      <c r="D323">
+        <v>239110.99210047512</v>
+      </c>
+      <c r="E323">
+        <v>235.35711669921875</v>
+      </c>
+      <c r="F323">
+        <v>235.88331604003906</v>
+      </c>
+      <c r="G323">
+        <v>238.30984497070312</v>
+      </c>
+      <c r="H323">
+        <v>79.33167266845703</v>
+      </c>
+      <c r="I323">
+        <v>97.25820922851562</v>
+      </c>
+      <c r="J323">
+        <v>88.05786895751953</v>
+      </c>
+      <c r="K323">
+        <v>17025.267578125</v>
+      </c>
+      <c r="L323">
+        <v>20328.39453125</v>
+      </c>
+      <c r="M323">
+        <v>19591.427734375</v>
+      </c>
+      <c r="N323">
+        <v>0.9118428826332092</v>
+      </c>
+      <c r="O323">
+        <v>0.8860935568809509</v>
+      </c>
+      <c r="P323">
+        <v>0.9309186339378357</v>
+      </c>
+      <c r="Q323">
+        <v>56592.16796875</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B324" t="str">
+        <v>11:37:19 ч.</v>
+      </c>
+      <c r="C324" t="str">
+        <v>HOMO UHT</v>
+      </c>
+      <c r="D324">
+        <v>1828.166480100625</v>
+      </c>
+      <c r="E324">
+        <v>235.2416534423828</v>
+      </c>
+      <c r="F324">
+        <v>235.748046875</v>
+      </c>
+      <c r="G324">
+        <v>237.52276611328125</v>
+      </c>
+      <c r="H324">
+        <v>0.24274863302707672</v>
+      </c>
+      <c r="I324">
+        <v>0.11179256439208984</v>
+      </c>
+      <c r="J324">
+        <v>0.2135954201221466</v>
+      </c>
+      <c r="K324">
+        <v>35.7476692199707</v>
+      </c>
+      <c r="L324">
+        <v>14.579123497009277</v>
+      </c>
+      <c r="M324">
+        <v>15.044944763183594</v>
+      </c>
+      <c r="N324">
+        <v>0.6260034441947937</v>
+      </c>
+      <c r="O324">
+        <v>0.5531850457191467</v>
+      </c>
+      <c r="P324">
+        <v>0.29654690623283386</v>
+      </c>
+      <c r="Q324">
+        <v>65.49597930908203</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B325" t="str">
+        <v>11:37:19 ч.</v>
+      </c>
+      <c r="C325" t="str">
+        <v>Priem KM</v>
+      </c>
+      <c r="D325">
+        <v>5584.628850987176</v>
+      </c>
+      <c r="E325">
+        <v>235.22039794921875</v>
+      </c>
+      <c r="F325">
+        <v>235.7249298095703</v>
+      </c>
+      <c r="G325">
+        <v>237.72528076171875</v>
+      </c>
+      <c r="H325">
+        <v>4.199803352355957</v>
+      </c>
+      <c r="I325">
+        <v>3.308820962905884</v>
+      </c>
+      <c r="J325">
+        <v>3.638700485229492</v>
+      </c>
+      <c r="K325">
+        <v>923.0313110351562</v>
+      </c>
+      <c r="L325">
+        <v>733.2921142578125</v>
+      </c>
+      <c r="M325">
+        <v>822.472412109375</v>
+      </c>
+      <c r="N325">
+        <v>0.9346168041229248</v>
+      </c>
+      <c r="O325">
+        <v>0.9403176307678223</v>
+      </c>
+      <c r="P325">
+        <v>0.9509884715080261</v>
+      </c>
+      <c r="Q325">
+        <v>2478.7958984375</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="str">
+        <v>24.12.2024 г.</v>
+      </c>
+      <c r="B326" t="str">
+        <v>11:37:19 ч.</v>
+      </c>
+      <c r="C326" t="str">
+        <v>Priem UHT</v>
+      </c>
+      <c r="D326">
+        <v>866.8711574631204</v>
+      </c>
+      <c r="E326">
+        <v>235.26199340820312</v>
+      </c>
+      <c r="F326">
+        <v>235.5532989501953</v>
+      </c>
+      <c r="G326">
+        <v>237.64085388183594</v>
+      </c>
+      <c r="H326">
+        <v>0.9222043752670288</v>
+      </c>
+      <c r="I326">
+        <v>0.5075970888137817</v>
+      </c>
+      <c r="J326">
+        <v>0.8379509449005127</v>
+      </c>
+      <c r="K326">
+        <v>116.86293029785156</v>
+      </c>
+      <c r="L326">
+        <v>82.85575103759766</v>
+      </c>
+      <c r="M326">
+        <v>59.3443489074707</v>
+      </c>
+      <c r="N326">
+        <v>0.539839506149292</v>
+      </c>
+      <c r="O326">
+        <v>0.6924997568130493</v>
+      </c>
+      <c r="P326">
+        <v>0.29856327176094055</v>
+      </c>
+      <c r="Q326">
+        <v>259.4527893066406</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q276"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q326"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>